<commit_message>
Regenerate tracker.xlsx after merging the 09-05 update
Never got regenerated in that run (openpyxl was missing from the
python resolved at the time) or in the earlier manual 08-29 merge.
Now current for all 36 tracked programs.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/EconGradAlert/data/tracker.xlsx
+++ b/apps/EconGradAlert/data/tracker.xlsx
@@ -438,7 +438,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last full research pass: 2026-08-29</t>
+          <t>Last full research pass: 2026-09-05</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Program count: 35</t>
+          <t>Program count: 36</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y36"/>
+  <dimension ref="A1:Y37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2737,7 +2737,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>~#192 (University of Vienna, Institute for Economics) — search-derived, not independently verified against the live RePEc table</t>
+          <t>#192 (University of Vienna, Fakultät für Wirtschaftswissenschaften) — confirmed via direct fetch of the live RePEc table</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2827,12 +2827,12 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Confirmed RePEc rank (#192) via direct fetch of the live table, removing the prior unverified caveat</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>~#24 (Tilburg School of Economics and Management) — search-derived, not independently verified</t>
+          <t>#24 (Tilburg School of Economics and Management) — confirmed via direct fetch of the live RePEc table</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2954,12 +2954,12 @@
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Confirmed RePEc rank (#24) via direct fetch of the live table, removing the prior unverified caveat</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>~#40 (KU Leuven, Faculteit Economie en Bedrijfswetenschappen) — search-derived, not independently verified</t>
+          <t>#40 (KU Leuven, Faculteit Economie en Bedrijfswetenschappen) — confirmed via direct fetch of the live RePEc table</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -3081,12 +3081,12 @@
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Confirmed RePEc rank (#40) via direct fetch of the live table, removing the prior unverified caveat</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>~#164 (Humboldt-Universität zu Berlin, Wirtschaftswissenschaftliche Fakultät, as coordinating institution) — search-derived; BSE is a multi-institution consortium so this reflects only the host department, not the consortium as a whole</t>
+          <t>#164 (Humboldt-Universität zu Berlin, Wirtschaftswissenschaftliche Fakultät, as coordinating institution) — confirmed via direct fetch of the live RePEc table; BSE is a multi-institution consortium so this reflects only the host department, not the consortium as a whole</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -3208,12 +3208,12 @@
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Confirmed RePEc rank (#164) via direct fetch of the live table, removing the prior unverified caveat</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
@@ -3225,7 +3225,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-21</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3240,139 +3240,139 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>National University of Singapore (NUS)</t>
+          <t>Sciences Po</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>#120</t>
+          <t>#42</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>France</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
+          <t>https://www.sciencespo.fr/ecole-recherche/en/admissions/phd/</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>No standardized test required; an optional English-language test may be requested for Economics applicants</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>See IELTS field</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Not mentioned on this page</t>
+          <t>Not required</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Non-English-medium graduates may need to take a Graduate English Course; good undergraduate honours degree (first class or high 2:1 equivalent) or Master's, in economics or another quantitative subject</t>
+          <t>Two academic recommendations, CV, cover letter, doctoral thesis topic proposal (max 5,000 words), thesis abstract (2 pages), Master's degree + transcripts; applicants who already have secured external funding must submit official proof of it</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Not specified on official pages checked</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Early: 30 September 2026; Main: 1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
+          <t>Two admissions sessions per year: 10 February and 17 May (dates shown were for the 2026 cohort, already closed) — recurring annual pattern, next expected ~Feb/May 2027</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
+          <t>2 (academic)</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>Not detailed (fully funded — see funding)</t>
+          <t>Tuition-exempt for enrolled doctoral students (D1-D6); CVEC student contribution still payable</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Yes — all admitted students</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
+          <t>Primary funding is a 3-year Doctoral Contract: gross salary ~EUR 2,100/month (2024 rate) for research/teaching duties. Additional Doctoral Research Funding Scheme provides quasi-lump-sum funding through year 4, plus yearly competitive calls for proposals. Note: some applicants are expected to already hold external funding at the time of application (proof required if so) — funding route should be confirmed directly with the department.</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>Confirmed deadlines unchanged; added admission requirement detail</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics</t>
+          <t>New find Sep 2026; funding model mixes an in-house Doctoral Contract with an expectation that some applicants already have external funding secured — verify which route applies before relying on the Doctoral Contract as guaranteed.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MPhil/PhD</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Hong Kong University of Science and Technology (HKUST)</t>
+          <t>National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>#287</t>
+          <t>#120</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -3382,47 +3382,47 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
+          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>6.5 overall, no subscore below 5.5 (university-wide standard; waived if English-medium/first-language English)</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>iBT 80 / pBT 550 / Revised PBT 60 (university-wide standard)</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Required ("satisfactory score")</t>
+          <t>Not mentioned on this page</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Conditional offers require official documents by end of July</t>
+          <t>Non-English-medium graduates may need to take a Graduate English Course; good undergraduate honours degree (first class or high 2:1 equivalent) or Master's, in economics or another quantitative subject</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Fall semester</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
+          <t>Early: 30 September 2026; Main: 1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -3437,22 +3437,22 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>HK$180, non-refundable</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>HK$47,000/year (2026/27 rate, full-time or part-time)</t>
+          <t>Not detailed (fully funded — see funding)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — all admitted students</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>Postgraduate Studentship (PGS): HK$229,620/year (2025/26 rate); recipients serve as Graduate Teaching Assistants. HKUST RedBird PhD Award stacks with HKPFS: Recruitment Award HK$40,000 (year 1) + Academic Excellence Award HK$20,000/year (later years). Conference &amp; Travel Allowance ~HK$14,200/year for HKPFS holders. Also cross-reference Hong Kong PhD Fellowship Scheme (ASA-03).</t>
+          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
@@ -3467,39 +3467,39 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr), fees, and IELTS/TOEFL standards; upgraded funding_status from Likely to Yes</t>
+          <t>Confirmed deadlines unchanged; added admission requirement detail</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026</t>
+          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PhD (Fellowship, cross-university)</t>
+          <t>MPhil/PhD</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
+          <t>MPhil/PhD in Economics</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Varies by host university (scheme spans multiple HK institutions)</t>
+          <t>#287</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3519,37 +3519,37 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
+          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>6.5 overall, no subscore below 5.5 (university-wide standard; waived if English-medium/first-language English)</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>iBT 80 / pBT 550 / Revised PBT 60 (university-wide standard)</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>Required ("satisfactory score")</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
+          <t>Conditional offers require official documents by end of July</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Typically September (Fall)</t>
+          <t>Fall semester</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
+          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -3559,27 +3559,27 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$180, non-refundable</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Waived (see funding)</t>
+          <t>HK$47,000/year (2026/27 rate, full-time or part-time)</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Yes — major fellowship</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
+          <t>Postgraduate Studentship (PGS): HK$229,620/year (2025/26 rate); recipients serve as Graduate Teaching Assistants. HKUST RedBird PhD Award stacks with HKPFS: Recruitment Award HK$40,000 (year 1) + Academic Excellence Award HK$20,000/year (later years). Conference &amp; Travel Allowance ~HK$14,200/year for HKPFS holders. Also cross-reference Hong Kong PhD Fellowship Scheme (ASA-03).</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
@@ -3589,44 +3589,44 @@
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr), fees, and IELTS/TOEFL standards; upgraded funding_status from Likely to Yes</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
+          <t>Seed entry Aug 2026</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>ASA-03</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>PhD (Fellowship, cross-university)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Nanyang Technological University (NTU Singapore)</t>
+          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>#253</t>
+          <t>Varies by host university (scheme spans multiple HK institutions)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3636,47 +3636,47 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
+          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>7.0 minimum (preferred)</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>105 minimum</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Not mandatory, but scores considered if submitted; recommended for applicants without a degree from an autonomous university</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders; 2 referee reports required</t>
+          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Two intakes/year: August (main) and January</t>
+          <t>Typically September (Fall)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>August intake: applications open 1 Oct-15 Nov (results Mar-May); January intake: applications open 1 Jun-31 Jul (results Nov-Dec) — recurring annual pattern, confirmed via direct official fetch</t>
+          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -3686,27 +3686,27 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>2 (referee reports)</t>
+          <t>Not specified in scheme rules</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>S$50</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Not specified (MOE-subsidised place)</t>
+          <t>Waived (see funding)</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — major fellowship</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>MOE-subsidised programme; funded via Nanyang President's Graduate Scholarship or Nanyang Research Scholarship, which carries Graduate Assistantship Programme (GAP) teaching/research duties.</t>
+          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
@@ -3716,24 +3716,24 @@
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>Confirmed application windows, referee/fee requirements via direct official fetch; urgency upgraded from tba to soon</t>
+          <t>Added (seed)</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; tuition fee figure still not found</t>
+          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3743,17 +3743,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD)</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>University of Tokyo</t>
+          <t>Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>#110</t>
+          <t>#253</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3763,77 +3763,77 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Tokyo</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
+          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>7.0 minimum (preferred)</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>105 minimum</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not mandatory, but scores considered if submitted; recommended for applicants without a degree from an autonomous university</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>English-taught international program; site (gaia.e.u-tokyo.ac.jp) unreachable for a third consecutive pass — DNS resolution failure confirmed again via independent fetch attempts. As of April 2023, UTIPE PhD applicants are generally required to first complete UTIPE's own Master's program and be admitted to candidacy; direct external PhD entry is closed except for applicants with 2+ years of research experience at a university/research institute abroad (following 16 years of foreign schooling), who may be recognized as equivalent to a Master's holder and apply directly. Corroborated via search snippets quoting the official admission/FAQ pages, not a direct primary-source fetch.</t>
+          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders; 2 referee reports required</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Two intakes/year: August (main) and January</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Not yet confirmed — needs manual check</t>
+          <t>August intake: applications open 1 Oct-15 Nov (results Mar-May); January intake: applications open 1 Jun-31 Jul (results Nov-Dec) — recurring annual pattern, confirmed via direct official fetch</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>2 (referee reports)</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>S$50</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not specified (MOE-subsidised place)</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
+          <t>MOE-subsidised programme; funded via Nanyang President's Graduate Scholarship or Nanyang Research Scholarship, which carries Graduate Assistantship Programme (GAP) teaching/research duties.</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
@@ -3848,19 +3848,19 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>Corroborated (via search snippets of official FAQ/admission pages) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad; site itself remains unreachable (DNS failure, third consecutive pass)</t>
+          <t>Confirmed application windows, referee/fee requirements via direct official fetch; urgency upgraded from tba to soon</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>INCOMPLETE — prioritise for next refresh, though the site has now failed to resolve on three consecutive passes; consider a manual browser check. The 2023 admission-policy restriction is now corroborated by multiple search snippets quoting the official pages, but still not confirmed via a direct primary-source fetch.</t>
+          <t>Seed entry Aug 2026; tuition fee figure still not found</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3870,17 +3870,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD)</t>
+          <t>International Program in Economics (PhD)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Hitotsubashi University</t>
+          <t>University of Tokyo</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>#390 (confirmed still outside global top 300)</t>
+          <t>#110</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3895,72 +3895,72 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Tokyo (Kunitachi)</t>
+          <t>Tokyo</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://www.econ.hit-u.ac.jp/eng/page/graduate/admission.html</t>
+          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Not stated (page mentions TOEFL/TOEIC only)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>TOEFL or TOEIC score required as part of application materials; specific minimum score not stated</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Two intakes/year (Spring and Autumn); international applicants without a Hitotsubashi Master's apply via an AO exam route — either general AO (2+ years work experience post-master's) or AO for international applicants with a Master's from outside Japan; admission mainly via submitted documents, interview may follow (online option for overseas applicants)</t>
+          <t>English-taught international program; site (gaia.e.u-tokyo.ac.jp) unreachable for a fourth consecutive pass — DNS resolution failure confirmed again via independent fetch attempts. As of April 2023, UTIPE PhD applicants are generally required to first complete UTIPE's own Master's program and be admitted to candidacy; direct external PhD entry is closed except for applicants with 2+ years of research experience at a university/research institute abroad (following 16 years of foreign schooling), who may be recognized as equivalent to a Master's holder and apply directly. Corroborated via search snippets quoting the official admission/FAQ pages, not a direct primary-source fetch.</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Spring or Autumn intake (two cycles/year)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Spring intake: document submission window ~14-17 Oct annually (confirmed for the Spring 2026 cohort: 14-17 Oct 2025, results ~11 Nov 2025), so the next window is expected ~mid-Oct 2026 for Spring 2027 entry. Autumn intake: opens ~April, exact window not confirmed this pass.</t>
+          <t>Not yet confirmed — needs manual check</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>tba</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>At least 1 recommendation letter required (AO exam route requires an English-language Letter of Recommendation); exact number for other routes not specified</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>~JPY 30,000 reported (university-wide general graduate-school figure, not confirmed Economics-specific)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>~JPY 535,800/year reported (university-wide figure, not confirmed Economics-PhD-specific)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible)</t>
+          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>MEXT scholarship route confirmed to exist, administered via a separate central international-office page (requires embassy/consulate preliminary candidacy). No department-specific stipend/assistantship figures found.</t>
+          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
@@ -3970,24 +3970,24 @@
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration (official PDF/page blocked direct fetch by an SSL certificate error); urgency upgraded from tba to soon</t>
+          <t>Site remains unreachable (DNS failure, fourth consecutive pass) — no new information found this pass</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Partially complete — fee figures are university-wide, not Economics-PhD-confirmed; exact Autumn-intake window still needed</t>
+          <t>INCOMPLETE — the official site has now failed to resolve on four consecutive passes; a manual browser check is recommended rather than further automated retries. The 2023 admission-policy restriction is corroborated by multiple search snippets quoting the official pages, but still not confirmed via a direct primary-source fetch.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3997,17 +3997,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD)</t>
+          <t>Graduate School of Economics (PhD)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Seoul National University (SNU)</t>
+          <t>Hitotsubashi University</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>#189</t>
+          <t>#390 (confirmed still outside global top 300)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -4017,77 +4017,77 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Seoul</t>
+          <t>Tokyo (Kunitachi)</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://en.snu.ac.kr/admission</t>
+          <t>https://www.econ.hit-u.ac.jp/eng/page/graduate/admission.html</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>6.0 minimum (university-wide standard)</t>
+          <t>Not stated (page mentions TOEFL/TOEIC only)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>iBT 80, or TEPS 551 (university-wide standard, alternative to IELTS)</t>
+          <t>TOEFL or TOEIC score required as part of application materials; specific minimum score not stated</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Not required (no GRE requirement found in central admissions materials)</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
+          <t>Two intakes/year (Spring and Autumn); international applicants without a Hitotsubashi Master's apply via an AO exam route — either general AO (2+ years work experience post-master's) or AO for international applicants with a Master's from outside Japan; admission mainly via submitted documents, interview may follow (online option for overseas applicants)</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Spring or Autumn intake (two cycles/year)</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>University-wide pattern: Fall-intake applications open ~early March (2026 Fall: 3-5 Mar); Spring-intake applications open ~early July (2027 Spring: 6-9 Jul) — both 2026 cycles already closed; 2027 Fall cycle not yet announced. Department-specific PhD deadline still not separately confirmed.</t>
+          <t>Spring intake: document submission window ~14-17 Oct annually (confirmed for the Spring 2026 cohort: 14-17 Oct 2025, results ~11 Nov 2025), so the next window is expected ~mid-Oct 2026 for Spring 2027 entry. Autumn intake: opens ~April, exact window not confirmed this pass.</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>later</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>At least 1 recommendation letter required (AO exam route requires an English-language Letter of Recommendation); exact number for other routes not specified</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>KRW 90,000 (no fee waivers offered)</t>
+          <t>~JPY 30,000 reported (university-wide general graduate-school figure, not confirmed Economics-specific)</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>~JPY 535,800/year reported (university-wide figure, not confirmed Economics-PhD-specific)</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Likely (university-wide scholarships only)</t>
+          <t>Likely (MEXT scholarship-eligible)</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Confirmed via direct fetch of the Department of Economics' own PhD page: no department-specific funding scheme exists — funding runs entirely through the university-wide scholarships above.</t>
+          <t>MEXT scholarship route confirmed to exist, administered via a separate central international-office page (requires embassy/consulate preliminary candidacy). No department-specific stipend/assistantship figures found.</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
@@ -4102,19 +4102,19 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; admissions and funding run entirely through the university-wide portal and scholarships</t>
+          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration (official PDF/page blocked direct fetch by an SSL certificate error); urgency upgraded from tba to soon</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>Confirmed (Aug 2026) that Economics PhD funding at SNU is university-wide only, with no departmental top-up scheme; department page exists but defers entirely to the central international-admissions portal for deadlines/fees</t>
+          <t>Partially complete — fee figures are university-wide, not Economics-PhD-confirmed; exact Autumn-intake window still needed</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ASA-08</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4124,17 +4124,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PhD in Business (Economics track)</t>
+          <t>Department of Economics (PhD)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>University of Hong Kong (Faculty of Business and Economics)</t>
+          <t>Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>#106</t>
+          <t>#189</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -4144,104 +4144,104 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Seoul</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://phd.hkubs.hku.hk/admissions/admission-application-and-tuition-fee</t>
+          <t>https://en.snu.ac.kr/admission</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Academic overall 6.5, all subtests &gt;= 6.0 (waived if prior degree was taught in English)</t>
+          <t>6.0 minimum (university-wide standard)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>iBT &gt;= 85</t>
+          <t>iBT 80, or TEPS 551 (university-wide standard, alternative to IELTS)</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>GRE or GMAT required, score &lt;5 years old (institution codes: GRE 2482, GMAT FS2-WL-48)</t>
+          <t>Not required (no GRE requirement found in central admissions materials)</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Bachelor's with first-class honours (or equivalent), or Bachelor's + Master's from a recognized university; 3-year track with a research Master's, 4-year track without one; Economics is one of six FBE PhD fields</t>
+          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Fall semester, normally September (matriculates once a year)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Applications open 1 September; Main Round closes 1 December (recurring annual cycle; late applications considered only if places remain)</t>
+          <t>University-wide pattern: Fall-intake applications open ~early March (2026 Fall: 3-5 Mar); Spring-intake applications open ~early July (2027 Spring: 6-9 Jul) — both 2026 cycles already closed; 2027 Fall cycle not yet announced. Department-specific PhD deadline still not separately confirmed.</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2 (academic referee reports, submitted directly by referees)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>HK$600 (paid online via HKU Graduate School application system)</t>
+          <t>KRW 90,000 (no fee waivers offered)</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>HK$49,500/year (2027-28 rate) for full-time PhD — typically waived/covered for scholarship holders</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Likely (university-wide scholarships only)</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>Standard Postgraduate Scholarship (PGS) pays HK$19,135/month (rising to HK$19,655/month once candidature is confirmed), available to essentially all admitted PhD students regardless of HKPFS status. HKPFS awardees instead receive HK$28,700/month plus HK$14,400/year travel allowance for up to 3 years.</t>
+          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Confirmed via direct fetch of the Department of Economics' own PhD page: no department-specific funding scheme exists — funding runs entirely through the university-wide scholarships above.</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; admissions and funding run entirely through the university-wide portal and scholarships</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>Distinct from the cross-institution HKPFS scheme already tracked (ASA-03) — nearly all admitted PhD students get baseline PGS funding here even without winning HKPFS, a broader guarantee than HKPFS alone.</t>
+          <t>Confirmed (Aug 2026) that Economics PhD funding at SNU is university-wide only, with no departmental top-up scheme; department page exists but defers entirely to the central international-admissions portal for deadlines/fees</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4251,17 +4251,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD in Business (Economics track)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>~#369 — search-derived, not independently verified against the live RePEc table</t>
+          <t>#106</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -4281,37 +4281,37 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://admission.econ.cuhk.edu.hk/pg/phd-economics/</t>
+          <t>https://phd.hkubs.hku.hk/admissions/admission-application-and-tuition-fee</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Academic overall 6.5</t>
+          <t>Academic overall 6.5, all subtests &gt;= 6.0 (waived if prior degree was taught in English)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>79 iBT (or 4.5-6.0 Home Edition) — see IELTS field for alternatives (GMAT Verbal &gt;=21, or a degree from an English-medium institution, also accepted)</t>
+          <t>iBT &gt;= 85</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Required (institution code 3153, department code 1801); no published hard cutoff, but absence of a score disadvantages applicants</t>
+          <t>GRE or GMAT required, score &lt;5 years old (institution codes: GRE 2482, GMAT FS2-WL-48)</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Master's in economics or a related field with a strong math/stats background expected; strong bachelor's-only applicants can also apply with sufficient research potential. Official transcripts, degree certificates, a 5-page research proposal and/or working papers, resume, and typically an interview all required</t>
+          <t>Bachelor's with first-class honours (or equivalent), or Bachelor's + Master's from a recognized university; 3-year track with a research Master's, 4-year track without one; Economics is one of six FBE PhD fields</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Fall intake (standard)</t>
+          <t>Fall semester, normally September (matriculates once a year)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Applications open 1 Sept 2026; HKPFS-track deadline 1 Dec 2026 (11:59am); non-HKPFS deadline 1 Dec 2026 (11:59pm); referee letters due by 4 Dec 2026</t>
+          <t>Applications open 1 September; Main Round closes 1 December (recurring annual cycle; late applications considered only if places remain)</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -4321,37 +4321,37 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>3 confidential recommendation letters</t>
+          <t>2 (academic referee reports, submitted directly by referees)</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>HK$500 per programme</t>
+          <t>HK$600 (paid online via HKU Graduate School application system)</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>HK$47,000 (2026/27) / HK$49,500 (2027/28)</t>
+          <t>HK$49,500/year (2027-28 rate) for full-time PhD — typically waived/covered for scholarship holders</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Yes — guaranteed assistantship for all admits</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>All successful full-time PhD admits receive a teaching/research assistantship with a monthly stipend of ~HK$19,100. HKPFS awardees additionally receive a full tuition waiver plus HK$40,000 (year 1) / HK$20,000/year (subsequent years) and housing benefits. Local students separately receive a government tuition waiver. Cross-reference the cross-institution HKPFS scheme already tracked (ASA-03).</t>
+          <t>Standard Postgraduate Scholarship (PGS) pays HK$19,135/month (rising to HK$19,655/month once candidature is confirmed), available to essentially all admitted PhD students regardless of HKPFS status. HKPFS awardees instead receive HK$28,700/month plus HK$14,400/year travel allowance for up to 3 years.</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
@@ -4361,14 +4361,14 @@
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>New find Aug 2026; distinct from HKU (ASA-08) and the cross-institution HKPFS scheme (ASA-03) — CUHK guarantees baseline assistantship funding to all admits independent of HKPFS.</t>
+          <t>Distinct from the cross-institution HKPFS scheme already tracked (ASA-03) — nearly all admitted PhD students get baseline PGS funding here even without winning HKPFS, a broader guarantee than HKPFS alone.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4383,119 +4383,119 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Australian National University (ANU)</t>
+          <t>Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>#124</t>
+          <t>#369 — confirmed via direct fetch of the live RePEc table</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Canberra</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
+          <t>https://admission.econ.cuhk.edu.hk/pg/phd-economics/</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>6.5 overall (no band below 6.0)</t>
+          <t>Academic overall 6.5</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>570 (paper-based; essay ≥4.5)</t>
+          <t>79 iBT (or 4.5-6.0 Home Edition) — see IELTS field for alternatives (GMAT Verbal &gt;=21, or a degree from an English-medium institution, also accepted)</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
+          <t>Required (institution code 3153, department code 1801); no published hard cutoff, but absence of a score disadvantages applicants</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
+          <t>Master's in economics or a related field with a strong math/stats background expected; strong bachelor's-only applicants can also apply with sufficient research potential. Official transcripts, degree certificates, a 5-page research proposal and/or working papers, resume, and typically an interview all required</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>February (Semester 1); Semester 2 entry possible (July)</t>
+          <t>Fall intake (standard)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>For Feb 2027 start: international scholarship applicants before 31 Aug 2026 (imminent — 2 days away as of 29 Aug 2026, reconfirmed still live via search corroboration of the official ANU text), standard before 31 Oct 2026; Sem 2 entry before 31 Mar</t>
+          <t>Applications open 1 Sept 2026; HKPFS-track deadline 1 Dec 2026 (11:59am); non-HKPFS deadline 1 Dec 2026 (11:59pm); referee letters due by 4 Dec 2026</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3 confidential recommendation letters</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$500 per programme</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$47,000 (2026/27) / HK$49,500 (2027/28)</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — guaranteed assistantship for all admits</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>Australian Government RTP Stipend: AUD $39,069/year (2026 full-time base rate, ANU-wide), paid fortnightly, up to 3.5 years. Some HDR supplementary scholarships add AUD $7,000/year on top, for up to 3 years. Domestic candidates pay no tuition (RTP-covered); international candidates can compete for HDR Fee Remission Merit Scholarships covering up to 4 years.</t>
+          <t>All successful full-time PhD admits receive a teaching/research assistantship with a monthly stipend of ~HK$19,100. HKPFS awardees additionally receive a full tuition waiver plus HK$40,000 (year 1) / HK$20,000/year (subsequent years) and housing benefits. Local students separately receive a government tuition waiver. Cross-reference the cross-institution HKPFS scheme already tracked (ASA-03).</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>Reconfirmed the imminent 31 Aug 2026 deadline is still live (ANU site returned HTTP 504 to direct fetch this pass, confirmed instead via search corroboration of the official text); set 7-day reminder flag</t>
+          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026 — international scholarship deadline is imminent (2 days away as of this update)</t>
+          <t>New find Aug 2026; distinct from HKU (ASA-08) and the cross-institution HKPFS scheme (ASA-03) — CUHK guarantees baseline assistantship funding to all admits independent of HKPFS.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4505,17 +4505,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>University of Melbourne</t>
+          <t>Australian National University (ANU)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>#151</t>
+          <t>#124</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -4530,42 +4530,42 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Melbourne</t>
+          <t>Canberra</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
+          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
+          <t>6.5 overall (no band below 6.0)</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>94 iBT (W27/S18/R13/L13)</t>
+          <t>570 (paper-based; essay ≥4.5)</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Not mentioned in entry requirements</t>
+          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
+          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>March intake</t>
+          <t>February (Semester 1); Semester 2 entry possible (July)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>March 2027 intake deadline reported as 30 November 2026 — found via search summary only; the official how-to-apply/key-dates pages returned HTTP 403 on every direct fetch attempt this pass, so this date is unconfirmed by primary source and should be manually verified</t>
+          <t>For Feb 2027 start: international scholarship deadline (31 Aug 2026) has now closed; the standard/domestic deadline of 31 Oct 2026 is the next live deadline (confirmed via search corroboration, ANU site still returning HTTP 504 to direct fetch); Sem 2 entry deadline (31 Mar) also already closed for this cycle</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -4575,17 +4575,17 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Not detailed — full tuition fee waiver reported (see funding)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
@@ -4595,7 +4595,7 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>Australian Government Research Training Program (RTP) funded places available: RTP stipend reported at AUD $39,500/year (2026 rate) plus full tuition fee waiver and AUD $15,000 research/conference travel funding for confirmed PhD candidates (unconfirmed by primary source — see deadline note). Program structure: 2-year Master of Commerce coursework + 3-year PhD.</t>
+          <t>Australian Government RTP Stipend: AUD $39,069/year (2026 full-time base rate, ANU-wide), paid fortnightly, up to 3.5 years. Some HDR supplementary scholarships add AUD $7,000/year on top, for up to 3 years. Domestic candidates pay no tuition (RTP-covered); international candidates can compete for HDR Fee Remission Merit Scholarships covering up to 4 years.</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
@@ -4605,24 +4605,24 @@
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>Found a reported deadline and funding figures via search, but could not confirm via direct page fetch (403 blocked) — flagged as lower confidence</t>
+          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline — reset reminder flags for the new date</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches this pass — recommend a manual browser check before relying on the reported 30 Nov 2026 deadline</t>
+          <t>Seed entry Aug 2026 — international-applicant deadline has closed; domestic deadline (31 Oct 2026) is next</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4632,17 +4632,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PhD (Economics)</t>
+          <t>Doctoral Program in Economics</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Monash Business School</t>
+          <t>University of Melbourne</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>#46</t>
+          <t>#151</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4657,47 +4657,47 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Melbourne (Clayton)</t>
+          <t>Melbourne</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
+          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>7.0 minimum reported (third-party source, not confirmed on official Monash page — page returned HTTP 403 to direct fetch)</t>
+          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>94 minimum reported (same caveat as IELTS — unconfirmed by primary source)</t>
+          <t>94 iBT (W27/S18/R13/L13)</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Not mentioned in entry requirements</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
+          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>March intake</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Two pathways found (via search — official pages returned HTTP 403 to direct fetch, unconfirmed by primary source): Integrated PhD program (Master of Commerce + PhD), Feb/Semester-1 entry — applications open 1 Jul-31 Aug (closing imminently); Jul/Semester-2 entry — applications open 1 Dec-1 Feb. Separately, general Graduate Research Scholarship rounds: international Round 1 closes 31 Mar, Round 3 closes ~31 Jul/31 Aug; domestic Round 2 closes 31 May, Round 4 closes 31 Oct.</t>
+          <t>March 2027 intake deadline reported as 30 November 2026 — found via search summary only; the official how-to-apply/key-dates pages returned HTTP 403 on every direct fetch attempt this pass, so this date is unconfirmed by primary source and should be manually verified</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -4707,12 +4707,12 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>International ~AUD $38,900/yr, domestic ~AUD $37,100/yr reported (third-party aggregator source, not confirmed by official Monash page)</t>
+          <t>Not detailed — full tuition fee waiver reported (see funding)</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -4722,7 +4722,7 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places — general RTP stipend reported at AUD $37,145/yr (2026 rate) plus a $1,500 relocation allowance (not confirmed Economics-specific).</t>
+          <t>Australian Government Research Training Program (RTP) funded places available: RTP stipend reported at AUD $39,500/year (2026 rate) plus full tuition fee waiver and AUD $15,000 research/conference travel funding for confirmed PhD candidates (unconfirmed by primary source — see deadline note). Program structure: 2-year Master of Commerce coursework + 3-year PhD.</t>
         </is>
       </c>
       <c r="V33" t="inlineStr">
@@ -4732,24 +4732,24 @@
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>Reconfirmed the imminent ~31 Aug 2026 integrated-pathway deadline is still accurate (search-only — monash.edu continues to block all direct fetches with HTTP 403); found a general RTP stipend figure (AUD $37,145/yr); set 7-day reminder flag</t>
+          <t>Found a reported deadline and funding figures via search, but could not confirm via direct page fetch (403 blocked) — flagged as lower confidence</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; monash.edu has blocked all automated fetches on every pass so far (scholarships-and-fees, apply, and program pages all 403'd) — every figure in this entry is lower-confidence (search snippets/third-party aggregator only) and needs a manual browser check, especially the imminent 31 Aug 2026 integrated-pathway deadline</t>
+          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches this pass — recommend a manual browser check before relying on the reported 30 Nov 2026 deadline</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4759,17 +4759,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD (Economics)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>University of Sydney</t>
+          <t>Monash Business School</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>#87</t>
+          <t>#46</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4784,32 +4784,32 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Sydney</t>
+          <t>Melbourne (Clayton)</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://www.sydney.edu.au/scholarships/</t>
+          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>7.0 minimum reported (third-party source, not confirmed on official Monash page — page returned HTTP 403 to direct fetch)</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>94 minimum reported (same caveat as IELTS — unconfirmed by primary source)</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP. Material finding: Sydney has no dedicated 'PhD in Economics' program page — the Economics coursework handbook explicitly states it "does not include a research component and thus does not provide a pathway to higher degree by research (e.g. PhD) studies." PhD study is pursued via the general Doctor of Philosophy degree with a nominated Economics supervisor/discipline, not a single named landing page.</t>
+          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -4819,17 +4819,17 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>General Research Training Program (RTP) scholarship rounds for 2027 entry (found via search, not a directly-fetched dedicated Economics PhD page): Research Period 1 &amp; 2 — deadline 11 September 2026; Research Period 3 &amp; 4 — deadline 18 December 2026.</t>
+          <t>Integrated-pathway Feb/Semester-1 entry window (1 Jul-31 Aug) has closed; next integrated-pathway window (Jul/Semester-2 entry) opens ~1 Dec-1 Feb. Separately, general Graduate Research Scholarship rounds: international Round 3 (~31 Jul/31 Aug) has closed; domestic Round 4 closes 31 Oct 2026 (confirmed via search, monash.edu still blocking direct fetch with HTTP 403) — this is the next live deadline.</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>1 (for named scholarship example; general program may differ)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -4839,7 +4839,7 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>International ~AUD $38,900/yr, domestic ~AUD $37,100/yr reported (third-party aggregator source, not confirmed by official Monash page)</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -4849,7 +4849,7 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly.</t>
+          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places — general RTP stipend reported at AUD $37,145/yr (2026 rate) plus a $1,500 relocation allowance (not confirmed Economics-specific).</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
@@ -4859,24 +4859,24 @@
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>Found general RTP scholarship round deadlines (11 Sep / 18 Dec 2026); confirmed there is no dedicated Sydney 'PhD in Economics' page — entry is via the general PhD degree with an Economics supervisor; set 30-day reminder flag</t>
+          <t>Confirmed the ~31 Aug 2026 integrated-pathway and international-round deadlines have closed; domestic Graduate Research Scholarship Round 4 (31 Oct 2026) is the next live deadline — reset reminder flags for the new date</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check; no dedicated Economics-specific PhD admissions page exists at Sydney</t>
+          <t>Seed entry Aug 2026; monash.edu has blocked all automated fetches on every pass so far (scholarships-and-fees, apply, and program pages all 403'd) — every figure in this entry is lower-confidence (search snippets/third-party aggregator only) and needs a manual browser check</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AUS-05</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4891,12 +4891,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>UNSW Sydney</t>
+          <t>University of Sydney</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>#80</t>
+          <t>#87</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4916,67 +4916,67 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://www.unsw.edu.au/business/study-with-us/postgraduate-research/phd-degrees/doctor-philosophy-phd-economics</t>
+          <t>https://www.sydney.edu.au/scholarships/</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Not listed on this page (exemptions for AU/CA/UK/US/NZ citizens); non-English-speaking-country applicants need IELTS/TOEFL/PTE/Cambridge or the UNSW Global English Course</t>
+          <t>Not specified at general program level</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Not listed on this page — see IELTS field for alternatives</t>
+          <t>Not specified at general program level</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Optional but recommended overall; one source indicates GRE may be specifically required for the Economics stream — this conflicts with the general 'optional' language elsewhere and needs manual confirmation</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course. Program begins with a 1-year Master of Pre-Doctoral Business Studies, followed by 3-3.5 years of doctoral research; direct entry to the 3-year PhD is possible for candidates with first-class Honours/Master's plus independent funding (Stream 2).</t>
+          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP. Material finding: Sydney has no dedicated 'PhD in Economics' program page — the Economics coursework handbook explicitly states it "does not include a research component and thus does not provide a pathway to higher degree by research (e.g. PhD) studies." PhD study is pursued via the general Doctor of Philosophy degree with a nominated Economics supervisor/discipline, not a single named landing page.</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Term 1 – February</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Confirmed still closed as of 23 Aug 2026 (verified directly on program page): EOI window opened 20 March 2026, closed 15 August 2026, no newer/next EOI window posted. Note: a separate 26 August 2026 formal-application deadline exists, but it applies only to candidates already invited to apply from the closed EOI round, not to new applicants.</t>
+          <t>General Research Training Program (RTP) scholarship rounds for 2027 entry (reconfirmed via search, not a directly-fetched dedicated Economics PhD page): Research Period 1 &amp; 2 — deadline 11 September 2026 (imminent — 6 days away as of 5 Sep 2026); Research Period 3 &amp; 4 — deadline 18 December 2026.</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>urgent</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
+          <t>1 (for named scholarship example; general program may differ)</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R35" t="inlineStr">
+      <c r="S35" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t>Not detailed (fully funded — see funding)</t>
-        </is>
-      </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>Yes — all admitted students</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>Full tuition waiver + stipend AUD 35,000-45,000/yr, up to 4.5 years (+1 optional fellowship year), plus substantial research/conference travel funding.</t>
+          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly.</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
@@ -4986,144 +4986,271 @@
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>Confirmed EOI window remains closed with no new window announced; added program structure and English-test details</t>
+          <t>Reconfirmed the 11 Sep 2026 Research Period 1 &amp; 2 deadline is still live and now imminent; set 7-day reminder flag</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026 — EOI window closed 15 Aug 2026, still no next window announced as of this update</t>
+          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check; no dedicated Economics-specific PhD admissions page exists at Sydney</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>AUS-05</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>PhD in Economics</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>UNSW Sydney</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>#80</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://www.unsw.edu.au/business/study-with-us/postgraduate-research/phd-degrees/doctor-philosophy-phd-economics</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Not listed on this page (exemptions for AU/CA/UK/US/NZ citizens); non-English-speaking-country applicants need IELTS/TOEFL/PTE/Cambridge or the UNSW Global English Course</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Not listed on this page — see IELTS field for alternatives</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Optional but recommended overall; one source indicates GRE may be specifically required for the Economics stream — this conflicts with the general 'optional' language elsewhere and needs manual confirmation</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course. Program begins with a 1-year Master of Pre-Doctoral Business Studies, followed by 3-3.5 years of doctoral research; direct entry to the 3-year PhD is possible for candidates with first-class Honours/Master's plus independent funding (Stream 2).</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Term 1 – February</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Confirmed still closed as of 23 Aug 2026 (verified directly on program page): EOI window opened 20 March 2026, closed 15 August 2026, no newer/next EOI window posted. Note: a separate 26 August 2026 formal-application deadline exists, but it applies only to candidates already invited to apply from the closed EOI round, not to new applicants.</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Not detailed (fully funded — see funding)</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Yes — all admitted students</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Full tuition waiver + stipend AUD 35,000-45,000/yr, up to 4.5 years (+1 optional fellowship year), plus substantial research/conference travel funding.</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>Confirmed EOI window remains closed with no new window announced; added program structure and English-test details</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026 — EOI window closed 15 Aug 2026, still no next window announced as of this update</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>AUS-06</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>Doctor of Philosophy (Economics)</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>University of Queensland (School of Economics)</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>#71</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>Brisbane</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>https://economics.uq.edu.au/study/phd</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>Academic overall 6.5, with 6.0 minimum in each of reading/writing/speaking/listening</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>Not specified on the economics-specific page (UQ university-wide PhD pages generally accept TOEFL iBT as an alternative to IELTS)</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>Not confirmed as required; application package can include GRE/GMAT score sheets, suggesting optional/supplementary rather than mandatory</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="M37" t="inlineStr">
         <is>
           <t>Academic CV, transcripts; MPhil/research master's options also available; can join a funded project with scholarship support as an alternative entry route</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t>Quarterly intakes (research quarters begin 1 Jan, 1 Apr, 1 Jul, 1 Oct); applications for RHD programs can be submitted any time</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>Confirmed via direct fetch of the UQ Graduate Research School Scholarships page (exact quoted text): 'Monday 31 August 2026 – Application closing date' (Domestic Round 1) and 'Monday 19 October 2026 – Application closing date' (International round), for upcoming 2027 research quarters</t>
-        </is>
-      </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>urgent</t>
-        </is>
-      </c>
-      <c r="Q36" t="inlineStr">
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Domestic Round 1 (31 Aug 2026) has now closed; the International round deadline of 19 Oct 2026 is confirmed still live via search corroboration and is the next relevant deadline for upcoming 2027 research quarters.</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>soon</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
         <is>
           <t>Minimum 2 referee reports</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr">
+      <c r="R37" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="S36" t="inlineStr">
+      <c r="S37" t="inlineStr">
         <is>
           <t>Not specified (international RTP scholarship recipients typically get a full tuition fee offset)</t>
         </is>
       </c>
-      <c r="T36" t="inlineStr">
+      <c r="T37" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr">
+      <c r="U37" t="inlineStr">
         <is>
           <t>RTP/UQGRSS provides a tax-free living stipend of AUD $39,220/year (2026 rate, indexed annually — updated from a previously-recorded AUD $37,500 figure) plus, for eligible international candidates, a tuition fee offset; no separate application needed beyond the program EOI.</t>
         </is>
       </c>
-      <c r="V36" t="inlineStr">
+      <c r="V37" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="W36" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
-      </c>
-      <c r="X36" t="inlineStr">
-        <is>
-          <t>Confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to the current AUD $39,220/yr (2026) rate; set 7-day reminder flag</t>
-        </is>
-      </c>
-      <c r="Y36" t="inlineStr">
-        <is>
-          <t>Scholarship is university-wide (RTP/UQGRSS), not economics-specific, but School of Economics PhD candidates are eligible. The 31 Aug 2026 round is imminent — 2 days away as of this update.</t>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026) — reset reminder flags for the new date</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>Scholarship is university-wide (RTP/UQGRSS), not economics-specific, but School of Economics PhD candidates are eligible.</t>
         </is>
       </c>
     </row>
@@ -5138,7 +5265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5178,152 +5305,152 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>EUR-17</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>New find: FWF-grant-funded PhD positions at the University of Vienna; admission-round dates inconsistent across sources, recommend a manual spot-check.</t>
+          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline, urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EUR-18</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>New find: PhD structured as a salaried employment contract (~EUR 2,750-3,500/month); official site blocked automated fetches, several fields search-only.</t>
+          <t>Confirmed the integrated-pathway and international scholarship round deadlines have closed; now tracking the domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026), urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EUR-19</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>New find: RePEc ~#40, funded PhD positions up to 4 years plus IRO Doctoral Scholarships for developing-country students; deadlines are vacancy-by-vacancy.</t>
+          <t>7-day reminder: the 11 Sep 2026 Research Period 1 &amp; 2 deadline is confirmed still live and now imminent.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>EUR-20</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>New find: joint Berlin-area doctoral school, funded via a EUR 1,650/month qualification-phase stipend then dissertation-phase employment.</t>
+          <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026), urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>New find: guaranteed teaching/research assistantship (~HK$19,100/month) for all admits, independent of the HKPFS scheme already tracked (ASA-03).</t>
+          <t>Confirmed RePEc rank (#192) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -5333,24 +5460,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Confirmed application windows (Aug intake: 1 Oct-15 Nov; Jan intake: 1 Jun-31 Jul), referee/fee requirements, and Graduate Assistantship Programme detail via direct official fetch; urgency upgraded from tba to soon.</t>
+          <t>Confirmed RePEc rank (#24) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -5360,24 +5487,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Corroborated via search snippets (site unreachable for a third consecutive pass) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad.</t>
+          <t>Confirmed RePEc rank (#40) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -5387,24 +5514,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration; urgency upgraded from tba to soon.</t>
+          <t>Confirmed RePEc rank (#164) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -5414,61 +5541,61 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; funding runs entirely through university-wide scholarships.</t>
+          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>7-day reminder: the 31 Aug 2026 international scholarship deadline is confirmed still live via search corroboration (ANU site returned HTTP 504 to direct fetch).</t>
+          <t>Official site remains unreachable (DNS failure, fourth consecutive pass); recommend a manual browser check rather than further automated retries.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>EUR-21</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>PhD in Economics — Sciences Po</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>7-day reminder: the imminent ~31 Aug 2026 integrated-pathway deadline is reconfirmed via search (monash.edu still blocking direct fetch); added a general RTP stipend figure (AUD $37,145/yr).</t>
+          <t>New find: RePEc #42, funded via a 3-year Doctoral Contract (~EUR 2,100/month) plus tuition exemption; some applicants expected to already hold external funding.</t>
         </is>
       </c>
     </row>
@@ -5480,147 +5607,147 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>7-day reminder: confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to AUD $39,220/yr (2026 rate).</t>
+          <t>New find: FWF-grant-funded PhD positions at the University of Vienna; admission-round dates inconsistent across sources, recommend a manual spot-check.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
+          <t>New find: PhD structured as a salaried employment contract (~EUR 2,750-3,500/month); official site blocked automated fetches, several fields search-only.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
+          <t>New find: RePEc ~#40, funded PhD positions up to 4 years plus IRO Doctoral Scholarships for developing-country students; deadlines are vacancy-by-vacancy.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
+          <t>New find: joint Berlin-area doctoral school, funded via a EUR 1,650/month qualification-phase stipend then dissertation-phase employment.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
+          <t>New find: guaranteed teaching/research assistantship (~HK$19,100/month) for all admits, independent of the HKPFS scheme already tracked (ASA-03).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -5630,24 +5757,24 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
+          <t>Confirmed application windows (Aug intake: 1 Oct-15 Nov; Jan intake: 1 Jun-31 Jul), referee/fee requirements, and Graduate Assistantship Programme detail via direct official fetch; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -5657,24 +5784,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
+          <t>Corroborated via search snippets (site unreachable for a third consecutive pass) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -5684,24 +5811,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
+          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -5711,88 +5838,88 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
+          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; funding runs entirely through university-wide scholarships.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
+          <t>7-day reminder: the 31 Aug 2026 international scholarship deadline is confirmed still live via search corroboration (ANU site returned HTTP 504 to direct fetch).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
+          <t>7-day reminder: the imminent ~31 Aug 2026 integrated-pathway deadline is reconfirmed via search (monash.edu still blocking direct fetch); added a general RTP stipend figure (AUD $37,145/yr).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
+          <t>7-day reminder: confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to AUD $39,220/yr (2026 rate).</t>
         </is>
       </c>
     </row>
@@ -5804,12 +5931,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -5819,7 +5946,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
+          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
         </is>
       </c>
     </row>
@@ -5831,12 +5958,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -5846,7 +5973,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
+          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
         </is>
       </c>
     </row>
@@ -5858,12 +5985,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>AUS-05</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PhD in Economics — UNSW Sydney</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -5873,7 +6000,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
+          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
         </is>
       </c>
     </row>
@@ -5885,22 +6012,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EUR-13</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
+          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
         </is>
       </c>
     </row>
@@ -5912,22 +6039,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EUR-14</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
+          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
         </is>
       </c>
     </row>
@@ -5939,22 +6066,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EUR-15</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
         </is>
       </c>
     </row>
@@ -5966,22 +6093,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>EUR-16</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
+          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
         </is>
       </c>
     </row>
@@ -5993,22 +6120,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ASA-08</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
+          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
         </is>
       </c>
     </row>
@@ -6020,319 +6147,319 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
+          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>EUR-03</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>EUR-04</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EUR-05</t>
+          <t>AUS-05</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PhD in Economics — CEMFI</t>
+          <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>EUR-06</t>
+          <t>EUR-13</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
+          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EUR-07</t>
+          <t>EUR-14</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PhD Program — Paris School of Economics (PSE)</t>
+          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>EUR-08</t>
+          <t>EUR-15</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — Stockholm University / IIES</t>
+          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EUR-09</t>
+          <t>EUR-16</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MPhil + DPhil in Economics — University of Oxford</t>
+          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
         </is>
       </c>
     </row>
@@ -6344,12 +6471,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>EUR-12</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -6371,12 +6498,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -6398,12 +6525,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>EUR-03</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -6425,12 +6552,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>EUR-04</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -6452,12 +6579,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-05</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>PhD in Economics — CEMFI</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -6479,12 +6606,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-06</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -6506,12 +6633,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-07</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>PhD Program — Paris School of Economics (PSE)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -6533,12 +6660,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>EUR-08</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD Programme in Economics — Stockholm University / IIES</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6560,12 +6687,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>EUR-09</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>MPhil + DPhil in Economics — University of Oxford</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6587,12 +6714,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6614,12 +6741,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6641,12 +6768,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>EUR-12</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -6668,20 +6795,317 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
+          <t>ASA-01</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>ASA-02</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ASA-03</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>ASA-04</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>ASA-05</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>ASA-06</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>ASA-07</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>AUS-01</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>PhD in Economics — Australian National University (ANU)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>AUS-02</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>AUS-03</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>PhD (Economics) — Monash Business School</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>AUS-04</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>PhD in Economics — University of Sydney</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
           <t>AUS-05</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D68" t="inlineStr">
         <is>
           <t>Added (seed)</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E68" t="inlineStr">
         <is>
           <t>Initial research pass — program added to tracker.</t>
         </is>

</xml_diff>

<commit_message>
Econ ledger update 2026-09-14: 1 added, 3 updated, 1 reminder flag
</commit_message>
<xml_diff>
--- a/apps/EconGradAlert/data/tracker.xlsx
+++ b/apps/EconGradAlert/data/tracker.xlsx
@@ -438,7 +438,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last full research pass: 2026-09-05</t>
+          <t>Last full research pass: 2026-09-14</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Program count: 36</t>
+          <t>Program count: 37</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y37"/>
+  <dimension ref="A1:Y38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3352,7 +3352,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-22</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3367,62 +3367,62 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>National University of Singapore (NUS)</t>
+          <t>University of Cambridge</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>#120</t>
+          <t>#50</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Cambridge</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
+          <t>https://www.econ.cam.ac.uk/apply/postgraduate/courses/phd-economics</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>7.5 overall, 7.0 minimum per component</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>110 overall, 25 minimum per section</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Not mentioned on this page</t>
+          <t>Not mentioned as required in the entry-requirements/how-to-apply pages checked this pass</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Non-English-medium graduates may need to take a Graduate English Course; good undergraduate honours degree (first class or high 2:1 equivalent) or Master's, in economics or another quantitative subject</t>
+          <t>Distinction-level Master's degree in Economics required, with advanced technical training in microeconomics, macroeconomics and econometrics; C1 Advanced (Grade A/B, 193+ overall) or C2 Proficiency (Grade A/B/C, 200+ overall) also accepted in place of IELTS/TOEFL; no ATAS certificate required for this course</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>1 October 2027 (Michaelmas term)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Early: 30 September 2026; Main: 1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
+          <t>Applications for Michaelmas 2027 entry open 9 September 2026; funding-competition deadline 8 December 2026 (apply by this date to be considered for most scholarships); final application deadline 2 February 2027</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -3432,74 +3432,74 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not confirmed this pass</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not confirmed this pass</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Not detailed (fully funded — see funding)</t>
+          <t>Not confirmed this pass</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Yes — all admitted students</t>
+          <t>Yes — majority funded</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
+          <t>University-wide reporting cited on the funding pages: roughly 66% of Cambridge doctoral students are fully funded (2024/25 figures). Funding sources include the Cambridge Trust, Gates Cambridge, individual Colleges, ESRC studentships (Doctoral Training Partnership), and central University funds; awarded via the single funding-deadline application rather than a separate scholarship form for most schemes. Exact stipend/tuition figures for Economics specifically not confirmed this pass — see the Postgraduate Funding Search for current amounts.</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>Confirmed deadlines unchanged; added admission requirement detail</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics</t>
+          <t>New find Sep 2026; a top-ranked UK econ PhD not previously tracked. Department pages (econ.cam.ac.uk) blocked automated fetches (HTTP 403) — deadline/requirement detail sourced from the central postgraduate.study.cam.ac.uk pages instead; references, application fee, and exact funding amounts still need direct confirmation.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MPhil/PhD</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Hong Kong University of Science and Technology (HKUST)</t>
+          <t>National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>#287</t>
+          <t>#120</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3509,52 +3509,52 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
+          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>6.5 overall, no subscore below 5.5 (university-wide standard; waived if English-medium/first-language English)</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>iBT 80 / pBT 550 / Revised PBT 60 (university-wide standard)</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Required ("satisfactory score")</t>
+          <t>Not mentioned on this page</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Conditional offers require official documents by end of July</t>
+          <t>Non-English-medium graduates may need to take a Graduate English Course; good undergraduate honours degree (first class or high 2:1 equivalent) or Master's, in economics or another quantitative subject</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Fall semester</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
+          <t>Early: 30 September 2026 (now within 30 days — imminent); Main: 1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>urgent</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -3564,22 +3564,22 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>HK$180, non-refundable</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>HK$47,000/year (2026/27 rate, full-time or part-time)</t>
+          <t>Not detailed (fully funded — see funding)</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — all admitted students</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>Postgraduate Studentship (PGS): HK$229,620/year (2025/26 rate); recipients serve as Graduate Teaching Assistants. HKUST RedBird PhD Award stacks with HKPFS: Recruitment Award HK$40,000 (year 1) + Academic Excellence Award HK$20,000/year (later years). Conference &amp; Travel Allowance ~HK$14,200/year for HKPFS holders. Also cross-reference Hong Kong PhD Fellowship Scheme (ASA-03).</t>
+          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
@@ -3589,44 +3589,44 @@
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr), fees, and IELTS/TOEFL standards; upgraded funding_status from Likely to Yes</t>
+          <t>Early-round deadline (30 Sep 2026) is now within 30 days — urgency upgraded from soon to urgent, 30-day reminder flag set</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026</t>
+          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PhD (Fellowship, cross-university)</t>
+          <t>MPhil/PhD</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
+          <t>MPhil/PhD in Economics</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Varies by host university (scheme spans multiple HK institutions)</t>
+          <t>#287</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3646,37 +3646,37 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
+          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>6.5 overall, no subscore below 5.5 (university-wide standard; waived if English-medium/first-language English)</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>iBT 80 / pBT 550 / Revised PBT 60 (university-wide standard)</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>Required ("satisfactory score")</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
+          <t>Conditional offers require official documents by end of July</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Typically September (Fall)</t>
+          <t>Fall semester</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
+          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -3686,27 +3686,27 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$180, non-refundable</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Waived (see funding)</t>
+          <t>HK$47,000/year (2026/27 rate, full-time or part-time)</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Yes — major fellowship</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
+          <t>Postgraduate Studentship (PGS): HK$229,620/year (2025/26 rate); recipients serve as Graduate Teaching Assistants. HKUST RedBird PhD Award stacks with HKPFS: Recruitment Award HK$40,000 (year 1) + Academic Excellence Award HK$20,000/year (later years). Conference &amp; Travel Allowance ~HK$14,200/year for HKPFS holders. Also cross-reference Hong Kong PhD Fellowship Scheme (ASA-03).</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
@@ -3716,44 +3716,44 @@
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr), fees, and IELTS/TOEFL standards; upgraded funding_status from Likely to Yes</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
+          <t>Seed entry Aug 2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>ASA-03</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>PhD (Fellowship, cross-university)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Nanyang Technological University (NTU Singapore)</t>
+          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>#253</t>
+          <t>Varies by host university (scheme spans multiple HK institutions)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3763,47 +3763,47 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
+          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>7.0 minimum (preferred)</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>105 minimum</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Not mandatory, but scores considered if submitted; recommended for applicants without a degree from an autonomous university</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders; 2 referee reports required</t>
+          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Two intakes/year: August (main) and January</t>
+          <t>Typically September (Fall)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>August intake: applications open 1 Oct-15 Nov (results Mar-May); January intake: applications open 1 Jun-31 Jul (results Nov-Dec) — recurring annual pattern, confirmed via direct official fetch</t>
+          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -3813,27 +3813,27 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>2 (referee reports)</t>
+          <t>Not specified in scheme rules</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>S$50</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Not specified (MOE-subsidised place)</t>
+          <t>Waived (see funding)</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — major fellowship</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>MOE-subsidised programme; funded via Nanyang President's Graduate Scholarship or Nanyang Research Scholarship, which carries Graduate Assistantship Programme (GAP) teaching/research duties.</t>
+          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
@@ -3843,24 +3843,24 @@
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>Confirmed application windows, referee/fee requirements via direct official fetch; urgency upgraded from tba to soon</t>
+          <t>Added (seed)</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; tuition fee figure still not found</t>
+          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3870,17 +3870,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD)</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>University of Tokyo</t>
+          <t>Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>#110</t>
+          <t>#253</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3890,77 +3890,77 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Tokyo</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
+          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>7.0 minimum (preferred)</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>105 minimum</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not mandatory, but scores considered if submitted; recommended for applicants without a degree from an autonomous university</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>English-taught international program; site (gaia.e.u-tokyo.ac.jp) unreachable for a fourth consecutive pass — DNS resolution failure confirmed again via independent fetch attempts. As of April 2023, UTIPE PhD applicants are generally required to first complete UTIPE's own Master's program and be admitted to candidacy; direct external PhD entry is closed except for applicants with 2+ years of research experience at a university/research institute abroad (following 16 years of foreign schooling), who may be recognized as equivalent to a Master's holder and apply directly. Corroborated via search snippets quoting the official admission/FAQ pages, not a direct primary-source fetch.</t>
+          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders; 2 referee reports required</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Two intakes/year: August (main) and January</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Not yet confirmed — needs manual check</t>
+          <t>August intake: applications open 1 Oct-15 Nov (results Mar-May); January intake: applications open 1 Jun-31 Jul (results Nov-Dec) — recurring annual pattern, confirmed via direct official fetch</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>2 (referee reports)</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>S$50</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not specified (MOE-subsidised place)</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
+          <t>MOE-subsidised programme; funded via Nanyang President's Graduate Scholarship or Nanyang Research Scholarship, which carries Graduate Assistantship Programme (GAP) teaching/research duties.</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
@@ -3970,24 +3970,24 @@
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>Site remains unreachable (DNS failure, fourth consecutive pass) — no new information found this pass</t>
+          <t>Confirmed application windows, referee/fee requirements via direct official fetch; urgency upgraded from tba to soon</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>INCOMPLETE — the official site has now failed to resolve on four consecutive passes; a manual browser check is recommended rather than further automated retries. The 2023 admission-policy restriction is corroborated by multiple search snippets quoting the official pages, but still not confirmed via a direct primary-source fetch.</t>
+          <t>Seed entry Aug 2026; tuition fee figure still not found</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3997,17 +3997,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD)</t>
+          <t>International Program in Economics (PhD)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Hitotsubashi University</t>
+          <t>University of Tokyo</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>#390 (confirmed still outside global top 300)</t>
+          <t>#110</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -4022,72 +4022,72 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Tokyo (Kunitachi)</t>
+          <t>Tokyo</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://www.econ.hit-u.ac.jp/eng/page/graduate/admission.html</t>
+          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Not stated (page mentions TOEFL/TOEIC only)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>TOEFL or TOEIC score required as part of application materials; specific minimum score not stated</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Two intakes/year (Spring and Autumn); international applicants without a Hitotsubashi Master's apply via an AO exam route — either general AO (2+ years work experience post-master's) or AO for international applicants with a Master's from outside Japan; admission mainly via submitted documents, interview may follow (online option for overseas applicants)</t>
+          <t>English-taught international program; site (gaia.e.u-tokyo.ac.jp) unreachable for a fifth consecutive pass — DNS resolution failure confirmed again via independent fetch attempts. As of April 2023, UTIPE PhD applicants are generally required to first complete UTIPE's own Master's program and be admitted to candidacy; direct external PhD entry is closed except for applicants with 2+ years of research experience at a university/research institute abroad (following 16 years of foreign schooling), who may be recognized as equivalent to a Master's holder and apply directly. Corroborated via search snippets quoting the official admission/FAQ pages, not a direct primary-source fetch. New this pass (via search only): since the 2025 enrollment cycle the Department of Economics reportedly merged the general Master's program and the previous UTIPE program, now admitting into a single Master's program twice a year — suggests the standalone "UTIPE Master's" entry point may itself have changed; unconfirmed by primary source.</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Spring or Autumn intake (two cycles/year)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Spring intake: document submission window ~14-17 Oct annually (confirmed for the Spring 2026 cohort: 14-17 Oct 2025, results ~11 Nov 2025), so the next window is expected ~mid-Oct 2026 for Spring 2027 entry. Autumn intake: opens ~April, exact window not confirmed this pass.</t>
+          <t>Not yet confirmed — needs manual check</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>tba</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>At least 1 recommendation letter required (AO exam route requires an English-language Letter of Recommendation); exact number for other routes not specified</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>~JPY 30,000 reported (university-wide general graduate-school figure, not confirmed Economics-specific)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>~JPY 535,800/year reported (university-wide figure, not confirmed Economics-PhD-specific)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible)</t>
+          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>MEXT scholarship route confirmed to exist, administered via a separate central international-office page (requires embassy/consulate preliminary candidacy). No department-specific stipend/assistantship figures found.</t>
+          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
@@ -4097,24 +4097,24 @@
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration (official PDF/page blocked direct fetch by an SSL certificate error); urgency upgraded from tba to soon</t>
+          <t>Site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>Partially complete — fee figures are university-wide, not Economics-PhD-confirmed; exact Autumn-intake window still needed</t>
+          <t>INCOMPLETE — the official site has now failed to resolve on five consecutive passes; a manual browser check is recommended rather than further automated retries. The 2023 admission-policy restriction is corroborated by multiple search snippets quoting the official pages, but still not confirmed via a direct primary-source fetch.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4124,17 +4124,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD)</t>
+          <t>Graduate School of Economics (PhD)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Seoul National University (SNU)</t>
+          <t>Hitotsubashi University</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>#189</t>
+          <t>#390 (confirmed still outside global top 300)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -4144,77 +4144,77 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Seoul</t>
+          <t>Tokyo (Kunitachi)</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://en.snu.ac.kr/admission</t>
+          <t>https://www.econ.hit-u.ac.jp/eng/page/graduate/admission.html</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>6.0 minimum (university-wide standard)</t>
+          <t>Not stated (page mentions TOEFL/TOEIC only)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>iBT 80, or TEPS 551 (university-wide standard, alternative to IELTS)</t>
+          <t>TOEFL or TOEIC score required as part of application materials; specific minimum score not stated</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Not required (no GRE requirement found in central admissions materials)</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
+          <t>Two intakes/year (Spring and Autumn); international applicants without a Hitotsubashi Master's apply via an AO exam route — either general AO (2+ years work experience post-master's) or AO for international applicants with a Master's from outside Japan; admission mainly via submitted documents, interview may follow (online option for overseas applicants)</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Spring or Autumn intake (two cycles/year)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>University-wide pattern: Fall-intake applications open ~early March (2026 Fall: 3-5 Mar); Spring-intake applications open ~early July (2027 Spring: 6-9 Jul) — both 2026 cycles already closed; 2027 Fall cycle not yet announced. Department-specific PhD deadline still not separately confirmed.</t>
+          <t>Spring intake: document submission window ~14-17 Oct annually (confirmed for the Spring 2026 cohort: 14-17 Oct 2025, results ~11 Nov 2025), so the next window is expected ~mid-Oct 2026 for Spring 2027 entry. Autumn intake: opens ~April, exact window not confirmed this pass.</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>later</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>At least 1 recommendation letter required (AO exam route requires an English-language Letter of Recommendation); exact number for other routes not specified</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>KRW 90,000 (no fee waivers offered)</t>
+          <t>~JPY 30,000 reported (university-wide general graduate-school figure, not confirmed Economics-specific)</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>~JPY 535,800/year reported (university-wide figure, not confirmed Economics-PhD-specific)</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>Likely (university-wide scholarships only)</t>
+          <t>Likely (MEXT scholarship-eligible)</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Confirmed via direct fetch of the Department of Economics' own PhD page: no department-specific funding scheme exists — funding runs entirely through the university-wide scholarships above.</t>
+          <t>MEXT scholarship route confirmed to exist, administered via a separate central international-office page (requires embassy/consulate preliminary candidacy). No department-specific stipend/assistantship figures found.</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
@@ -4229,19 +4229,19 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; admissions and funding run entirely through the university-wide portal and scholarships</t>
+          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration (official PDF/page blocked direct fetch by an SSL certificate error); urgency upgraded from tba to soon</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>Confirmed (Aug 2026) that Economics PhD funding at SNU is university-wide only, with no departmental top-up scheme; department page exists but defers entirely to the central international-admissions portal for deadlines/fees</t>
+          <t>Partially complete — fee figures are university-wide, not Economics-PhD-confirmed; exact Autumn-intake window still needed</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ASA-08</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4251,17 +4251,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PhD in Business (Economics track)</t>
+          <t>Department of Economics (PhD)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>University of Hong Kong (Faculty of Business and Economics)</t>
+          <t>Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>#106</t>
+          <t>#189</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -4271,104 +4271,104 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Seoul</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://phd.hkubs.hku.hk/admissions/admission-application-and-tuition-fee</t>
+          <t>https://en.snu.ac.kr/admission</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Academic overall 6.5, all subtests &gt;= 6.0 (waived if prior degree was taught in English)</t>
+          <t>6.0 minimum (university-wide standard)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>iBT &gt;= 85</t>
+          <t>iBT 80, or TEPS 551 (university-wide standard, alternative to IELTS)</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>GRE or GMAT required, score &lt;5 years old (institution codes: GRE 2482, GMAT FS2-WL-48)</t>
+          <t>Not required (no GRE requirement found in central admissions materials)</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Bachelor's with first-class honours (or equivalent), or Bachelor's + Master's from a recognized university; 3-year track with a research Master's, 4-year track without one; Economics is one of six FBE PhD fields</t>
+          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Fall semester, normally September (matriculates once a year)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Applications open 1 September; Main Round closes 1 December (recurring annual cycle; late applications considered only if places remain)</t>
+          <t>University-wide pattern: Fall-intake applications open ~early March (2026 Fall: 3-5 Mar); Spring-intake applications open ~early July (2027 Spring: 6-9 Jul) — both 2026 cycles already closed; 2027 Fall cycle not yet announced. Department-specific PhD deadline still not separately confirmed.</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>2 (academic referee reports, submitted directly by referees)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>HK$600 (paid online via HKU Graduate School application system)</t>
+          <t>KRW 90,000 (no fee waivers offered)</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>HK$49,500/year (2027-28 rate) for full-time PhD — typically waived/covered for scholarship holders</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Likely (university-wide scholarships only)</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Standard Postgraduate Scholarship (PGS) pays HK$19,135/month (rising to HK$19,655/month once candidature is confirmed), available to essentially all admitted PhD students regardless of HKPFS status. HKPFS awardees instead receive HK$28,700/month plus HK$14,400/year travel allowance for up to 3 years.</t>
+          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Confirmed via direct fetch of the Department of Economics' own PhD page: no department-specific funding scheme exists — funding runs entirely through the university-wide scholarships above.</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; admissions and funding run entirely through the university-wide portal and scholarships</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>Distinct from the cross-institution HKPFS scheme already tracked (ASA-03) — nearly all admitted PhD students get baseline PGS funding here even without winning HKPFS, a broader guarantee than HKPFS alone.</t>
+          <t>Confirmed (Aug 2026) that Economics PhD funding at SNU is university-wide only, with no departmental top-up scheme; department page exists but defers entirely to the central international-admissions portal for deadlines/fees</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4378,17 +4378,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD in Business (Economics track)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>#369 — confirmed via direct fetch of the live RePEc table</t>
+          <t>#106</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -4408,37 +4408,37 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://admission.econ.cuhk.edu.hk/pg/phd-economics/</t>
+          <t>https://phd.hkubs.hku.hk/admissions/admission-application-and-tuition-fee</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Academic overall 6.5</t>
+          <t>Academic overall 6.5, all subtests &gt;= 6.0 (waived if prior degree was taught in English)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>79 iBT (or 4.5-6.0 Home Edition) — see IELTS field for alternatives (GMAT Verbal &gt;=21, or a degree from an English-medium institution, also accepted)</t>
+          <t>iBT &gt;= 85</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Required (institution code 3153, department code 1801); no published hard cutoff, but absence of a score disadvantages applicants</t>
+          <t>GRE or GMAT required, score &lt;5 years old (institution codes: GRE 2482, GMAT FS2-WL-48)</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Master's in economics or a related field with a strong math/stats background expected; strong bachelor's-only applicants can also apply with sufficient research potential. Official transcripts, degree certificates, a 5-page research proposal and/or working papers, resume, and typically an interview all required</t>
+          <t>Bachelor's with first-class honours (or equivalent), or Bachelor's + Master's from a recognized university; 3-year track with a research Master's, 4-year track without one; Economics is one of six FBE PhD fields</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Fall intake (standard)</t>
+          <t>Fall semester, normally September (matriculates once a year)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Applications open 1 Sept 2026; HKPFS-track deadline 1 Dec 2026 (11:59am); non-HKPFS deadline 1 Dec 2026 (11:59pm); referee letters due by 4 Dec 2026</t>
+          <t>Applications open 1 September; Main Round closes 1 December (recurring annual cycle; late applications considered only if places remain)</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -4448,54 +4448,54 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>3 confidential recommendation letters</t>
+          <t>2 (academic referee reports, submitted directly by referees)</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>HK$500 per programme</t>
+          <t>HK$600 (paid online via HKU Graduate School application system)</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>HK$47,000 (2026/27) / HK$49,500 (2027/28)</t>
+          <t>HK$49,500/year (2027-28 rate) for full-time PhD — typically waived/covered for scholarship holders</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Yes — guaranteed assistantship for all admits</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>All successful full-time PhD admits receive a teaching/research assistantship with a monthly stipend of ~HK$19,100. HKPFS awardees additionally receive a full tuition waiver plus HK$40,000 (year 1) / HK$20,000/year (subsequent years) and housing benefits. Local students separately receive a government tuition waiver. Cross-reference the cross-institution HKPFS scheme already tracked (ASA-03).</t>
+          <t>Standard Postgraduate Scholarship (PGS) pays HK$19,135/month (rising to HK$19,655/month once candidature is confirmed), available to essentially all admitted PhD students regardless of HKPFS status. HKPFS awardees instead receive HK$28,700/month plus HK$14,400/year travel allowance for up to 3 years.</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>New find Aug 2026; distinct from HKU (ASA-08) and the cross-institution HKPFS scheme (ASA-03) — CUHK guarantees baseline assistantship funding to all admits independent of HKPFS.</t>
+          <t>Distinct from the cross-institution HKPFS scheme already tracked (ASA-03) — nearly all admitted PhD students get baseline PGS funding here even without winning HKPFS, a broader guarantee than HKPFS alone.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4510,62 +4510,62 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Australian National University (ANU)</t>
+          <t>Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>#124</t>
+          <t>#369 — confirmed via direct fetch of the live RePEc table</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Canberra</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
+          <t>https://admission.econ.cuhk.edu.hk/pg/phd-economics/</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>6.5 overall (no band below 6.0)</t>
+          <t>Academic overall 6.5</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>570 (paper-based; essay ≥4.5)</t>
+          <t>79 iBT (or 4.5-6.0 Home Edition) — see IELTS field for alternatives (GMAT Verbal &gt;=21, or a degree from an English-medium institution, also accepted)</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
+          <t>Required (institution code 3153, department code 1801); no published hard cutoff, but absence of a score disadvantages applicants</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
+          <t>Master's in economics or a related field with a strong math/stats background expected; strong bachelor's-only applicants can also apply with sufficient research potential. Official transcripts, degree certificates, a 5-page research proposal and/or working papers, resume, and typically an interview all required</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>February (Semester 1); Semester 2 entry possible (July)</t>
+          <t>Fall intake (standard)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>For Feb 2027 start: international scholarship deadline (31 Aug 2026) has now closed; the standard/domestic deadline of 31 Oct 2026 is the next live deadline (confirmed via search corroboration, ANU site still returning HTTP 504 to direct fetch); Sem 2 entry deadline (31 Mar) also already closed for this cycle</t>
+          <t>Applications open 1 Sept 2026; HKPFS-track deadline 1 Dec 2026 (11:59am); non-HKPFS deadline 1 Dec 2026 (11:59pm); referee letters due by 4 Dec 2026</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -4575,32 +4575,32 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3 confidential recommendation letters</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$500 per programme</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$47,000 (2026/27) / HK$49,500 (2027/28)</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — guaranteed assistantship for all admits</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>Australian Government RTP Stipend: AUD $39,069/year (2026 full-time base rate, ANU-wide), paid fortnightly, up to 3.5 years. Some HDR supplementary scholarships add AUD $7,000/year on top, for up to 3 years. Domestic candidates pay no tuition (RTP-covered); international candidates can compete for HDR Fee Remission Merit Scholarships covering up to 4 years.</t>
+          <t>All successful full-time PhD admits receive a teaching/research assistantship with a monthly stipend of ~HK$19,100. HKPFS awardees additionally receive a full tuition waiver plus HK$40,000 (year 1) / HK$20,000/year (subsequent years) and housing benefits. Local students separately receive a government tuition waiver. Cross-reference the cross-institution HKPFS scheme already tracked (ASA-03).</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
@@ -4610,19 +4610,19 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline — reset reminder flags for the new date</t>
+          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026 — international-applicant deadline has closed; domestic deadline (31 Oct 2026) is next</t>
+          <t>New find Aug 2026; distinct from HKU (ASA-08) and the cross-institution HKPFS scheme (ASA-03) — CUHK guarantees baseline assistantship funding to all admits independent of HKPFS.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4632,17 +4632,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>University of Melbourne</t>
+          <t>Australian National University (ANU)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>#151</t>
+          <t>#124</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4657,42 +4657,42 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Melbourne</t>
+          <t>Canberra</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
+          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
+          <t>6.5 overall (no band below 6.0)</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>94 iBT (W27/S18/R13/L13)</t>
+          <t>570 (paper-based; essay ≥4.5)</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Not mentioned in entry requirements</t>
+          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
+          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>March intake</t>
+          <t>February (Semester 1); Semester 2 entry possible (July)</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>March 2027 intake deadline reported as 30 November 2026 — found via search summary only; the official how-to-apply/key-dates pages returned HTTP 403 on every direct fetch attempt this pass, so this date is unconfirmed by primary source and should be manually verified</t>
+          <t>For Feb 2027 start: international scholarship deadline (31 Aug 2026) has now closed; the standard/domestic deadline of 31 Oct 2026 is the next live deadline (confirmed via search corroboration, ANU site still returning HTTP 504 to direct fetch); Sem 2 entry deadline (31 Mar) also already closed for this cycle</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -4702,17 +4702,17 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>Not detailed — full tuition fee waiver reported (see funding)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -4722,7 +4722,7 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>Australian Government Research Training Program (RTP) funded places available: RTP stipend reported at AUD $39,500/year (2026 rate) plus full tuition fee waiver and AUD $15,000 research/conference travel funding for confirmed PhD candidates (unconfirmed by primary source — see deadline note). Program structure: 2-year Master of Commerce coursework + 3-year PhD.</t>
+          <t>Australian Government RTP Stipend: AUD $39,069/year (2026 full-time base rate, ANU-wide), paid fortnightly, up to 3.5 years. Some HDR supplementary scholarships add AUD $7,000/year on top, for up to 3 years. Domestic candidates pay no tuition (RTP-covered); international candidates can compete for HDR Fee Remission Merit Scholarships covering up to 4 years.</t>
         </is>
       </c>
       <c r="V33" t="inlineStr">
@@ -4732,24 +4732,24 @@
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>Found a reported deadline and funding figures via search, but could not confirm via direct page fetch (403 blocked) — flagged as lower confidence</t>
+          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline — reset reminder flags for the new date</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches this pass — recommend a manual browser check before relying on the reported 30 Nov 2026 deadline</t>
+          <t>Seed entry Aug 2026 — international-applicant deadline has closed; domestic deadline (31 Oct 2026) is next</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4759,17 +4759,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PhD (Economics)</t>
+          <t>Doctoral Program in Economics</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Monash Business School</t>
+          <t>University of Melbourne</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>#46</t>
+          <t>#151</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4784,42 +4784,42 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Melbourne (Clayton)</t>
+          <t>Melbourne</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
+          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>7.0 minimum reported (third-party source, not confirmed on official Monash page — page returned HTTP 403 to direct fetch)</t>
+          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>94 minimum reported (same caveat as IELTS — unconfirmed by primary source)</t>
+          <t>94 iBT (W27/S18/R13/L13)</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Not mentioned in entry requirements</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
+          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>March intake</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Integrated-pathway Feb/Semester-1 entry window (1 Jul-31 Aug) has closed; next integrated-pathway window (Jul/Semester-2 entry) opens ~1 Dec-1 Feb. Separately, general Graduate Research Scholarship rounds: international Round 3 (~31 Jul/31 Aug) has closed; domestic Round 4 closes 31 Oct 2026 (confirmed via search, monash.edu still blocking direct fetch with HTTP 403) — this is the next live deadline.</t>
+          <t>March 2027 intake deadline reported as 30 November 2026 — found via search summary only; the official how-to-apply/key-dates pages returned HTTP 403 on every direct fetch attempt this pass, so this date is unconfirmed by primary source and should be manually verified</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -4834,12 +4834,12 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>International ~AUD $38,900/yr, domestic ~AUD $37,100/yr reported (third-party aggregator source, not confirmed by official Monash page)</t>
+          <t>Not detailed — full tuition fee waiver reported (see funding)</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -4849,7 +4849,7 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places — general RTP stipend reported at AUD $37,145/yr (2026 rate) plus a $1,500 relocation allowance (not confirmed Economics-specific).</t>
+          <t>Australian Government Research Training Program (RTP) funded places available: RTP stipend reported at AUD $39,500/year (2026 rate) plus full tuition fee waiver and AUD $15,000 research/conference travel funding for confirmed PhD candidates (unconfirmed by primary source — see deadline note). Program structure: 2-year Master of Commerce coursework + 3-year PhD.</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
@@ -4859,24 +4859,24 @@
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>Confirmed the ~31 Aug 2026 integrated-pathway and international-round deadlines have closed; domestic Graduate Research Scholarship Round 4 (31 Oct 2026) is the next live deadline — reset reminder flags for the new date</t>
+          <t>Found a reported deadline and funding figures via search, but could not confirm via direct page fetch (403 blocked) — flagged as lower confidence</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; monash.edu has blocked all automated fetches on every pass so far (scholarships-and-fees, apply, and program pages all 403'd) — every figure in this entry is lower-confidence (search snippets/third-party aggregator only) and needs a manual browser check</t>
+          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches this pass — recommend a manual browser check before relying on the reported 30 Nov 2026 deadline</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4886,17 +4886,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD (Economics)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>University of Sydney</t>
+          <t>Monash Business School</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>#87</t>
+          <t>#46</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4911,32 +4911,32 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Sydney</t>
+          <t>Melbourne (Clayton)</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://www.sydney.edu.au/scholarships/</t>
+          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>7.0 minimum reported (third-party source, not confirmed on official Monash page — page returned HTTP 403 to direct fetch)</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>94 minimum reported (same caveat as IELTS — unconfirmed by primary source)</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP. Material finding: Sydney has no dedicated 'PhD in Economics' program page — the Economics coursework handbook explicitly states it "does not include a research component and thus does not provide a pathway to higher degree by research (e.g. PhD) studies." PhD study is pursued via the general Doctor of Philosophy degree with a nominated Economics supervisor/discipline, not a single named landing page.</t>
+          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -4946,17 +4946,17 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>General Research Training Program (RTP) scholarship rounds for 2027 entry (reconfirmed via search, not a directly-fetched dedicated Economics PhD page): Research Period 1 &amp; 2 — deadline 11 September 2026 (imminent — 6 days away as of 5 Sep 2026); Research Period 3 &amp; 4 — deadline 18 December 2026.</t>
+          <t>Integrated-pathway Feb/Semester-1 entry window (1 Jul-31 Aug) has closed; next integrated-pathway window (Jul/Semester-2 entry) opens ~1 Dec-1 Feb. Separately, general Graduate Research Scholarship rounds: international Round 3 (~31 Jul/31 Aug) has closed; domestic Round 4 closes 31 Oct 2026 (confirmed via search, monash.edu still blocking direct fetch with HTTP 403) — this is the next live deadline.</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>1 (for named scholarship example; general program may differ)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -4966,7 +4966,7 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>International ~AUD $38,900/yr, domestic ~AUD $37,100/yr reported (third-party aggregator source, not confirmed by official Monash page)</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -4976,7 +4976,7 @@
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly.</t>
+          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places — general RTP stipend reported at AUD $37,145/yr (2026 rate) plus a $1,500 relocation allowance (not confirmed Economics-specific).</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
@@ -4991,19 +4991,19 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>Reconfirmed the 11 Sep 2026 Research Period 1 &amp; 2 deadline is still live and now imminent; set 7-day reminder flag</t>
+          <t>Confirmed the ~31 Aug 2026 integrated-pathway and international-round deadlines have closed; domestic Graduate Research Scholarship Round 4 (31 Oct 2026) is the next live deadline — reset reminder flags for the new date</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check; no dedicated Economics-specific PhD admissions page exists at Sydney</t>
+          <t>Seed entry Aug 2026; monash.edu has blocked all automated fetches on every pass so far (scholarships-and-fees, apply, and program pages all 403'd) — every figure in this entry is lower-confidence (search snippets/third-party aggregator only) and needs a manual browser check</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AUS-05</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5018,12 +5018,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>UNSW Sydney</t>
+          <t>University of Sydney</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>#80</t>
+          <t>#87</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -5043,67 +5043,67 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://www.unsw.edu.au/business/study-with-us/postgraduate-research/phd-degrees/doctor-philosophy-phd-economics</t>
+          <t>https://www.sydney.edu.au/scholarships/</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Not listed on this page (exemptions for AU/CA/UK/US/NZ citizens); non-English-speaking-country applicants need IELTS/TOEFL/PTE/Cambridge or the UNSW Global English Course</t>
+          <t>Not specified at general program level</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Not listed on this page — see IELTS field for alternatives</t>
+          <t>Not specified at general program level</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Optional but recommended overall; one source indicates GRE may be specifically required for the Economics stream — this conflicts with the general 'optional' language elsewhere and needs manual confirmation</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course. Program begins with a 1-year Master of Pre-Doctoral Business Studies, followed by 3-3.5 years of doctoral research; direct entry to the 3-year PhD is possible for candidates with first-class Honours/Master's plus independent funding (Stream 2).</t>
+          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP. Material finding: Sydney has no dedicated 'PhD in Economics' program page — the Economics coursework handbook explicitly states it "does not include a research component and thus does not provide a pathway to higher degree by research (e.g. PhD) studies." PhD study is pursued via the general Doctor of Philosophy degree with a nominated Economics supervisor/discipline, not a single named landing page.</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Term 1 – February</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Confirmed still closed as of 23 Aug 2026 (verified directly on program page): EOI window opened 20 March 2026, closed 15 August 2026, no newer/next EOI window posted. Note: a separate 26 August 2026 formal-application deadline exists, but it applies only to candidates already invited to apply from the closed EOI round, not to new applicants.</t>
+          <t>Research Period 1 &amp; 2 deadline (11 September 2026) has now passed; Research Period 3 &amp; 4 — deadline 18 December 2026 — is the next live RTP scholarship round (reconfirmed via search, not a directly-fetched dedicated Economics PhD page).</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
+          <t>1 (for named scholarship example; general program may differ)</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr">
+      <c r="S36" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>Not detailed (fully funded — see funding)</t>
-        </is>
-      </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>Yes — all admitted students</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>Full tuition waiver + stipend AUD 35,000-45,000/yr, up to 4.5 years (+1 optional fellowship year), plus substantial research/conference travel funding.</t>
+          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly; a 2027-rate RTP stipend of AUD $44,293/yr was also reported via search aggregators this pass (unconfirmed by primary source).</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
@@ -5113,142 +5113,269 @@
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>Confirmed EOI window remains closed with no new window announced; added program structure and English-test details</t>
+          <t>11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down from urgent to soon, reminder flags reset for the new deadline</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026 — EOI window closed 15 Aug 2026, still no next window announced as of this update</t>
+          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check; no dedicated Economics-specific PhD admissions page exists at Sydney</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>AUS-05</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>PhD in Economics</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>UNSW Sydney</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>#80</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://www.unsw.edu.au/business/study-with-us/postgraduate-research/phd-degrees/doctor-philosophy-phd-economics</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Not listed on this page (exemptions for AU/CA/UK/US/NZ citizens); non-English-speaking-country applicants need IELTS/TOEFL/PTE/Cambridge or the UNSW Global English Course</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Not listed on this page — see IELTS field for alternatives</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Optional but recommended overall; one source indicates GRE may be specifically required for the Economics stream — this conflicts with the general 'optional' language elsewhere and needs manual confirmation</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course. Program begins with a 1-year Master of Pre-Doctoral Business Studies, followed by 3-3.5 years of doctoral research; direct entry to the 3-year PhD is possible for candidates with first-class Honours/Master's plus independent funding (Stream 2).</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Term 1 – February</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Confirmed still closed as of 23 Aug 2026 (verified directly on program page): EOI window opened 20 March 2026, closed 15 August 2026, no newer/next EOI window posted. Note: a separate 26 August 2026 formal-application deadline exists, but it applies only to candidates already invited to apply from the closed EOI round, not to new applicants.</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Not detailed (fully funded — see funding)</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Yes — all admitted students</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Full tuition waiver + stipend AUD 35,000-45,000/yr, up to 4.5 years (+1 optional fellowship year), plus substantial research/conference travel funding.</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>Confirmed EOI window remains closed with no new window announced; added program structure and English-test details</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026 — EOI window closed 15 Aug 2026, still no next window announced as of this update</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>AUS-06</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>Doctor of Philosophy (Economics)</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>University of Queensland (School of Economics)</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>#71</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>Brisbane</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>https://economics.uq.edu.au/study/phd</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>Academic overall 6.5, with 6.0 minimum in each of reading/writing/speaking/listening</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>Not specified on the economics-specific page (UQ university-wide PhD pages generally accept TOEFL iBT as an alternative to IELTS)</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>Not confirmed as required; application package can include GRE/GMAT score sheets, suggesting optional/supplementary rather than mandatory</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="M38" t="inlineStr">
         <is>
           <t>Academic CV, transcripts; MPhil/research master's options also available; can join a funded project with scholarship support as an alternative entry route</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
+      <c r="N38" t="inlineStr">
         <is>
           <t>Quarterly intakes (research quarters begin 1 Jan, 1 Apr, 1 Jul, 1 Oct); applications for RHD programs can be submitted any time</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr">
+      <c r="O38" t="inlineStr">
         <is>
           <t>Domestic Round 1 (31 Aug 2026) has now closed; the International round deadline of 19 Oct 2026 is confirmed still live via search corroboration and is the next relevant deadline for upcoming 2027 research quarters.</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr">
+      <c r="P38" t="inlineStr">
         <is>
           <t>soon</t>
         </is>
       </c>
-      <c r="Q37" t="inlineStr">
+      <c r="Q38" t="inlineStr">
         <is>
           <t>Minimum 2 referee reports</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr">
+      <c r="R38" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="S37" t="inlineStr">
+      <c r="S38" t="inlineStr">
         <is>
           <t>Not specified (international RTP scholarship recipients typically get a full tuition fee offset)</t>
         </is>
       </c>
-      <c r="T37" t="inlineStr">
+      <c r="T38" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U37" t="inlineStr">
+      <c r="U38" t="inlineStr">
         <is>
           <t>RTP/UQGRSS provides a tax-free living stipend of AUD $39,220/year (2026 rate, indexed annually — updated from a previously-recorded AUD $37,500 figure) plus, for eligible international candidates, a tuition fee offset; no separate application needed beyond the program EOI.</t>
         </is>
       </c>
-      <c r="V37" t="inlineStr">
+      <c r="V38" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="W37" t="inlineStr">
+      <c r="W38" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="X37" t="inlineStr">
+      <c r="X38" t="inlineStr">
         <is>
           <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026) — reset reminder flags for the new date</t>
         </is>
       </c>
-      <c r="Y37" t="inlineStr">
+      <c r="Y38" t="inlineStr">
         <is>
           <t>Scholarship is university-wide (RTP/UQGRSS), not economics-specific, but School of Economics PhD candidates are eligible.</t>
         </is>
@@ -5265,7 +5392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5305,17 +5432,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -5325,88 +5452,88 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline, urgency moved from urgent to soon.</t>
+          <t>The 11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down to soon, reminder flags reset.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Confirmed the integrated-pathway and international scholarship round deadlines have closed; now tracking the domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026), urgency moved from urgent to soon.</t>
+          <t>30-day reminder: the early-round deadline (30 Sep 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7-day reminder: the 11 Sep 2026 Research Period 1 &amp; 2 deadline is confirmed still live and now imminent.</t>
+          <t>Official site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>EUR-22</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>PhD in Economics — University of Cambridge</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026), urgency moved from urgent to soon.</t>
+          <t>New find: RePEc #50, ~66% of Cambridge doctoral students fully funded via Cambridge Trust/Gates Cambridge/College/ESRC funding; funding-competition deadline 8 Dec 2026.</t>
         </is>
       </c>
     </row>
@@ -5418,12 +5545,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EUR-17</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -5433,7 +5560,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#192) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline, urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -5445,12 +5572,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EUR-18</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -5460,7 +5587,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#24) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>Confirmed the integrated-pathway and international scholarship round deadlines have closed; now tracking the domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026), urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -5472,22 +5599,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EUR-19</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#40) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>7-day reminder: the 11 Sep 2026 Research Period 1 &amp; 2 deadline is confirmed still live and now imminent.</t>
         </is>
       </c>
     </row>
@@ -5499,12 +5626,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EUR-20</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -5514,7 +5641,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#164) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026), urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -5526,12 +5653,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -5541,7 +5668,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>Confirmed RePEc rank (#192) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
@@ -5553,12 +5680,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -5568,7 +5695,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Official site remains unreachable (DNS failure, fourth consecutive pass); recommend a manual browser check rather than further automated retries.</t>
+          <t>Confirmed RePEc rank (#24) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
@@ -5580,120 +5707,120 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EUR-21</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>PhD in Economics — Sciences Po</t>
+          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>New find: RePEc #42, funded via a 3-year Doctoral Contract (~EUR 2,100/month) plus tuition exemption; some applicants expected to already hold external funding.</t>
+          <t>Confirmed RePEc rank (#40) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EUR-17</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
+          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>New find: FWF-grant-funded PhD positions at the University of Vienna; admission-round dates inconsistent across sources, recommend a manual spot-check.</t>
+          <t>Confirmed RePEc rank (#164) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EUR-18</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
+          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>New find: PhD structured as a salaried employment contract (~EUR 2,750-3,500/month); official site blocked automated fetches, several fields search-only.</t>
+          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>EUR-19</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>New find: RePEc ~#40, funded PhD positions up to 4 years plus IRO Doctoral Scholarships for developing-country students; deadlines are vacancy-by-vacancy.</t>
+          <t>Official site remains unreachable (DNS failure, fourth consecutive pass); recommend a manual browser check rather than further automated retries.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EUR-20</t>
+          <t>EUR-21</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
+          <t>PhD in Economics — Sciences Po</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -5703,7 +5830,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>New find: joint Berlin-area doctoral school, funded via a EUR 1,650/month qualification-phase stipend then dissertation-phase employment.</t>
+          <t>New find: RePEc #42, funded via a 3-year Doctoral Contract (~EUR 2,100/month) plus tuition exemption; some applicants expected to already hold external funding.</t>
         </is>
       </c>
     </row>
@@ -5715,12 +5842,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -5730,7 +5857,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>New find: guaranteed teaching/research assistantship (~HK$19,100/month) for all admits, independent of the HKPFS scheme already tracked (ASA-03).</t>
+          <t>New find: FWF-grant-funded PhD positions at the University of Vienna; admission-round dates inconsistent across sources, recommend a manual spot-check.</t>
         </is>
       </c>
     </row>
@@ -5742,22 +5869,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Confirmed application windows (Aug intake: 1 Oct-15 Nov; Jan intake: 1 Jun-31 Jul), referee/fee requirements, and Graduate Assistantship Programme detail via direct official fetch; urgency upgraded from tba to soon.</t>
+          <t>New find: PhD structured as a salaried employment contract (~EUR 2,750-3,500/month); official site blocked automated fetches, several fields search-only.</t>
         </is>
       </c>
     </row>
@@ -5769,22 +5896,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Corroborated via search snippets (site unreachable for a third consecutive pass) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad.</t>
+          <t>New find: RePEc ~#40, funded PhD positions up to 4 years plus IRO Doctoral Scholarships for developing-country students; deadlines are vacancy-by-vacancy.</t>
         </is>
       </c>
     </row>
@@ -5796,22 +5923,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration; urgency upgraded from tba to soon.</t>
+          <t>New find: joint Berlin-area doctoral school, funded via a EUR 1,650/month qualification-phase stipend then dissertation-phase employment.</t>
         </is>
       </c>
     </row>
@@ -5823,22 +5950,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; funding runs entirely through university-wide scholarships.</t>
+          <t>New find: guaranteed teaching/research assistantship (~HK$19,100/month) for all admits, independent of the HKPFS scheme already tracked (ASA-03).</t>
         </is>
       </c>
     </row>
@@ -5850,22 +5977,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>7-day reminder: the 31 Aug 2026 international scholarship deadline is confirmed still live via search corroboration (ANU site returned HTTP 504 to direct fetch).</t>
+          <t>Confirmed application windows (Aug intake: 1 Oct-15 Nov; Jan intake: 1 Jun-31 Jul), referee/fee requirements, and Graduate Assistantship Programme detail via direct official fetch; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
@@ -5877,22 +6004,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>7-day reminder: the imminent ~31 Aug 2026 integrated-pathway deadline is reconfirmed via search (monash.edu still blocking direct fetch); added a general RTP stipend figure (AUD $37,145/yr).</t>
+          <t>Corroborated via search snippets (site unreachable for a third consecutive pass) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad.</t>
         </is>
       </c>
     </row>
@@ -5904,39 +6031,39 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>7-day reminder: confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to AUD $39,220/yr (2026 rate).</t>
+          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -5946,88 +6073,88 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
+          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; funding runs entirely through university-wide scholarships.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
+          <t>7-day reminder: the 31 Aug 2026 international scholarship deadline is confirmed still live via search corroboration (ANU site returned HTTP 504 to direct fetch).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
+          <t>7-day reminder: the imminent ~31 Aug 2026 integrated-pathway deadline is reconfirmed via search (monash.edu still blocking direct fetch); added a general RTP stipend figure (AUD $37,145/yr).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
+          <t>7-day reminder: confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to AUD $39,220/yr (2026 rate).</t>
         </is>
       </c>
     </row>
@@ -6039,12 +6166,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -6054,7 +6181,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
+          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
         </is>
       </c>
     </row>
@@ -6066,12 +6193,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -6081,7 +6208,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
+          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
         </is>
       </c>
     </row>
@@ -6093,12 +6220,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -6108,7 +6235,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
+          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
         </is>
       </c>
     </row>
@@ -6120,12 +6247,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -6135,7 +6262,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
+          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
         </is>
       </c>
     </row>
@@ -6147,12 +6274,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -6162,7 +6289,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
+          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
         </is>
       </c>
     </row>
@@ -6174,12 +6301,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -6189,7 +6316,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
         </is>
       </c>
     </row>
@@ -6201,12 +6328,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -6216,7 +6343,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
+          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
         </is>
       </c>
     </row>
@@ -6228,12 +6355,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -6243,7 +6370,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
+          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
         </is>
       </c>
     </row>
@@ -6255,12 +6382,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -6270,7 +6397,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
+          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
         </is>
       </c>
     </row>
@@ -6282,12 +6409,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>AUS-05</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PhD in Economics — UNSW Sydney</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -6297,7 +6424,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
+          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -6309,22 +6436,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>EUR-13</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
+          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
         </is>
       </c>
     </row>
@@ -6336,22 +6463,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EUR-14</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
+          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -6363,22 +6490,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>EUR-15</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
+          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -6390,22 +6517,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EUR-16</t>
+          <t>AUS-05</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
+          <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
+          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
         </is>
       </c>
     </row>
@@ -6417,12 +6544,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ASA-08</t>
+          <t>EUR-13</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
+          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -6432,7 +6559,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
+          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
         </is>
       </c>
     </row>
@@ -6444,12 +6571,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>EUR-14</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -6459,115 +6586,115 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
+          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>EUR-15</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>EUR-16</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>EUR-03</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
+          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EUR-04</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
         </is>
       </c>
     </row>
@@ -6579,12 +6706,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>EUR-05</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PhD in Economics — CEMFI</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -6606,12 +6733,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>EUR-06</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -6633,12 +6760,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>EUR-07</t>
+          <t>EUR-03</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>PhD Program — Paris School of Economics (PSE)</t>
+          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -6660,12 +6787,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>EUR-08</t>
+          <t>EUR-04</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — Stockholm University / IIES</t>
+          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6687,12 +6814,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>EUR-09</t>
+          <t>EUR-05</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>MPhil + DPhil in Economics — University of Oxford</t>
+          <t>PhD in Economics — CEMFI</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6714,12 +6841,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>EUR-06</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6741,12 +6868,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>EUR-07</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>PhD Program — Paris School of Economics (PSE)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6768,12 +6895,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EUR-12</t>
+          <t>EUR-08</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
+          <t>PhD Programme in Economics — Stockholm University / IIES</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -6795,12 +6922,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-09</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>MPhil + DPhil in Economics — University of Oxford</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -6822,12 +6949,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -6849,12 +6976,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -6876,12 +7003,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-12</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -6903,12 +7030,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -6930,12 +7057,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -6957,12 +7084,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-03</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -6984,12 +7111,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -7011,12 +7138,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -7038,12 +7165,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -7065,12 +7192,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -7092,20 +7219,128 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
+          <t>AUS-01</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>PhD in Economics — Australian National University (ANU)</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>AUS-02</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>AUS-03</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>PhD (Economics) — Monash Business School</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>AUS-04</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>PhD in Economics — University of Sydney</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
           <t>AUS-05</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C72" t="inlineStr">
         <is>
           <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="D72" t="inlineStr">
         <is>
           <t>Added (seed)</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="E72" t="inlineStr">
         <is>
           <t>Initial research pass — program added to tracker.</t>
         </is>

</xml_diff>

<commit_message>
Econ ledger update 2026-09-19: 1 added, 2 updated, 2 reminder flags
</commit_message>
<xml_diff>
--- a/apps/EconGradAlert/data/tracker.xlsx
+++ b/apps/EconGradAlert/data/tracker.xlsx
@@ -438,7 +438,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last full research pass: 2026-09-14</t>
+          <t>Last full research pass: 2026-09-19</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Program count: 37</t>
+          <t>Program count: 38</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y38"/>
+  <dimension ref="A1:Y39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3479,7 +3479,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-23</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3489,144 +3489,144 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD in Economics (Quantitative Economics track)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>National University of Singapore (NUS)</t>
+          <t>Goethe University Frankfurt — Graduate School of Economics, Finance, and Management (GSEFM)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>#120</t>
+          <t>#81</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Frankfurt am Main</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
+          <t>https://www.gsefm.eu/degree-programs/economics.html</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>7.0 overall</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>93 iBT (or secondary/university education conducted entirely in English)</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Not mentioned on this page</t>
+          <t>Not mandatory; GRE Quant "strongly encouraged" — upper 20-25th percentile cited as demonstrating strong quantitative skills</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Non-English-medium graduates may need to take a Graduate English Course; good undergraduate honours degree (first class or high 2:1 equivalent) or Master's, in economics or another quantitative subject</t>
+          <t>Joint PhD/MSQ program — MSQ (Master's) students can transition into the PhD track after a successful first year; core training in economic theory, econometrics, and computational methods</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Winter semester (typically October)</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Early: 30 September 2026 (now within 30 days — imminent); Main: 1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
+          <t>Three-stage rolling review: Stage 1 31 January, Stage 2 31 March, Stage 3 31 May (recurring annual, for the following Winter semester intake) — early application recommended for visa processing and financial-aid consideration</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
+          <t>2 (at least one from a university professor)</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Not detailed (fully funded — see funding)</t>
+          <t>None — no tuition fees; administrative/semester fee ~EUR 377/semester (~EUR 754/year), includes public transit and museum access</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Yes — all admitted students</t>
+          <t>Yes — limited, competitive</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
+          <t>Up to three first-year stipends awarded via the IMFS Stipend program (amount not published; targeted at applicants in quantitative macroeconomics, model comparison, or monetary economics); TA/RA positions available after qualifying exams. The school's separate Finance track (SAFE-funded) offers EUR 1,300/month in year 1 plus RA contracts, for reference — not the Economics-track figure.</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>Early-round deadline (30 Sep 2026) is now within 30 days — urgency upgraded from soon to urgent, 30-day reminder flag set</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics</t>
+          <t>New find Sep 2026; stipend funding is limited/competitive (only 'up to three' first-year awards) rather than guaranteed to all admits — verify funding availability directly before relying on it.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MPhil/PhD</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Hong Kong University of Science and Technology (HKUST)</t>
+          <t>National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>#287</t>
+          <t>#120</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3636,52 +3636,52 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
+          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>6.5 overall, no subscore below 5.5 (university-wide standard; waived if English-medium/first-language English)</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>iBT 80 / pBT 550 / Revised PBT 60 (university-wide standard)</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Required ("satisfactory score")</t>
+          <t>Not mentioned on this page</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Conditional offers require official documents by end of July</t>
+          <t>Non-English-medium graduates may need to take a Graduate English Course; good undergraduate honours degree (first class or high 2:1 equivalent) or Master's, in economics or another quantitative subject</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Fall semester</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
+          <t>Early: 30 September 2026 (now within 30 days — imminent); Main: 1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>urgent</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -3691,22 +3691,22 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>HK$180, non-refundable</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>HK$47,000/year (2026/27 rate, full-time or part-time)</t>
+          <t>Not detailed (fully funded — see funding)</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — all admitted students</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>Postgraduate Studentship (PGS): HK$229,620/year (2025/26 rate); recipients serve as Graduate Teaching Assistants. HKUST RedBird PhD Award stacks with HKPFS: Recruitment Award HK$40,000 (year 1) + Academic Excellence Award HK$20,000/year (later years). Conference &amp; Travel Allowance ~HK$14,200/year for HKPFS holders. Also cross-reference Hong Kong PhD Fellowship Scheme (ASA-03).</t>
+          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
@@ -3716,44 +3716,44 @@
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr), fees, and IELTS/TOEFL standards; upgraded funding_status from Likely to Yes</t>
+          <t>Early-round deadline (30 Sep 2026) is now within 30 days — urgency upgraded from soon to urgent, 30-day reminder flag set</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026</t>
+          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PhD (Fellowship, cross-university)</t>
+          <t>MPhil/PhD</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
+          <t>MPhil/PhD in Economics</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Varies by host university (scheme spans multiple HK institutions)</t>
+          <t>#287</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3773,37 +3773,37 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
+          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>6.5 overall, no subscore below 5.5 (university-wide standard; waived if English-medium/first-language English)</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>iBT 80 / pBT 550 / Revised PBT 60 (university-wide standard)</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>Required ("satisfactory score")</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
+          <t>Conditional offers require official documents by end of July</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Typically September (Fall)</t>
+          <t>Fall semester</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
+          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -3813,27 +3813,27 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$180, non-refundable</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Waived (see funding)</t>
+          <t>HK$47,000/year (2026/27 rate, full-time or part-time)</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Yes — major fellowship</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
+          <t>Postgraduate Studentship (PGS): HK$229,620/year (2025/26 rate); recipients serve as Graduate Teaching Assistants. HKUST RedBird PhD Award stacks with HKPFS: Recruitment Award HK$40,000 (year 1) + Academic Excellence Award HK$20,000/year (later years). Conference &amp; Travel Allowance ~HK$14,200/year for HKPFS holders. Also cross-reference Hong Kong PhD Fellowship Scheme (ASA-03).</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
@@ -3843,44 +3843,44 @@
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr), fees, and IELTS/TOEFL standards; upgraded funding_status from Likely to Yes</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
+          <t>Seed entry Aug 2026</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>ASA-03</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>PhD (Fellowship, cross-university)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Nanyang Technological University (NTU Singapore)</t>
+          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>#253</t>
+          <t>Varies by host university (scheme spans multiple HK institutions)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3890,47 +3890,47 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
+          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>7.0 minimum (preferred)</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>105 minimum</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Not mandatory, but scores considered if submitted; recommended for applicants without a degree from an autonomous university</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders; 2 referee reports required</t>
+          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Two intakes/year: August (main) and January</t>
+          <t>Typically September (Fall)</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>August intake: applications open 1 Oct-15 Nov (results Mar-May); January intake: applications open 1 Jun-31 Jul (results Nov-Dec) — recurring annual pattern, confirmed via direct official fetch</t>
+          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -3940,27 +3940,27 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>2 (referee reports)</t>
+          <t>Not specified in scheme rules</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>S$50</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Not specified (MOE-subsidised place)</t>
+          <t>Waived (see funding)</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — major fellowship</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>MOE-subsidised programme; funded via Nanyang President's Graduate Scholarship or Nanyang Research Scholarship, which carries Graduate Assistantship Programme (GAP) teaching/research duties.</t>
+          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
@@ -3970,24 +3970,24 @@
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>Confirmed application windows, referee/fee requirements via direct official fetch; urgency upgraded from tba to soon</t>
+          <t>Added (seed)</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; tuition fee figure still not found</t>
+          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3997,17 +3997,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD)</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>University of Tokyo</t>
+          <t>Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>#110</t>
+          <t>#253</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -4017,77 +4017,77 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Tokyo</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
+          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>7.0 minimum (preferred)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>105 minimum</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not mandatory, but scores considered if submitted; recommended for applicants without a degree from an autonomous university</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>English-taught international program; site (gaia.e.u-tokyo.ac.jp) unreachable for a fifth consecutive pass — DNS resolution failure confirmed again via independent fetch attempts. As of April 2023, UTIPE PhD applicants are generally required to first complete UTIPE's own Master's program and be admitted to candidacy; direct external PhD entry is closed except for applicants with 2+ years of research experience at a university/research institute abroad (following 16 years of foreign schooling), who may be recognized as equivalent to a Master's holder and apply directly. Corroborated via search snippets quoting the official admission/FAQ pages, not a direct primary-source fetch. New this pass (via search only): since the 2025 enrollment cycle the Department of Economics reportedly merged the general Master's program and the previous UTIPE program, now admitting into a single Master's program twice a year — suggests the standalone "UTIPE Master's" entry point may itself have changed; unconfirmed by primary source.</t>
+          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders; 2 referee reports required</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Two intakes/year: August (main) and January</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Not yet confirmed — needs manual check</t>
+          <t>August intake: applications open 1 Oct-15 Nov (results Mar-May); January intake: applications open 1 Jun-31 Jul (results Nov-Dec) — recurring annual pattern, confirmed via direct official fetch</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>2 (referee reports)</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>S$50</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not specified (MOE-subsidised place)</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
+          <t>MOE-subsidised programme; funded via Nanyang President's Graduate Scholarship or Nanyang Research Scholarship, which carries Graduate Assistantship Programme (GAP) teaching/research duties.</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
@@ -4097,24 +4097,24 @@
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>Site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025</t>
+          <t>Confirmed application windows, referee/fee requirements via direct official fetch; urgency upgraded from tba to soon</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>INCOMPLETE — the official site has now failed to resolve on five consecutive passes; a manual browser check is recommended rather than further automated retries. The 2023 admission-policy restriction is corroborated by multiple search snippets quoting the official pages, but still not confirmed via a direct primary-source fetch.</t>
+          <t>Seed entry Aug 2026; tuition fee figure still not found</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4124,17 +4124,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD)</t>
+          <t>International Program in Economics (PhD)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Hitotsubashi University</t>
+          <t>University of Tokyo</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>#390 (confirmed still outside global top 300)</t>
+          <t>#110</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -4149,72 +4149,72 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Tokyo (Kunitachi)</t>
+          <t>Tokyo</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://www.econ.hit-u.ac.jp/eng/page/graduate/admission.html</t>
+          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Not stated (page mentions TOEFL/TOEIC only)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>TOEFL or TOEIC score required as part of application materials; specific minimum score not stated</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Two intakes/year (Spring and Autumn); international applicants without a Hitotsubashi Master's apply via an AO exam route — either general AO (2+ years work experience post-master's) or AO for international applicants with a Master's from outside Japan; admission mainly via submitted documents, interview may follow (online option for overseas applicants)</t>
+          <t>English-taught international program; site (gaia.e.u-tokyo.ac.jp) unreachable for a fifth consecutive pass — DNS resolution failure confirmed again via independent fetch attempts. As of April 2023, UTIPE PhD applicants are generally required to first complete UTIPE's own Master's program and be admitted to candidacy; direct external PhD entry is closed except for applicants with 2+ years of research experience at a university/research institute abroad (following 16 years of foreign schooling), who may be recognized as equivalent to a Master's holder and apply directly. Corroborated via search snippets quoting the official admission/FAQ pages, not a direct primary-source fetch. New this pass (via search only): since the 2025 enrollment cycle the Department of Economics reportedly merged the general Master's program and the previous UTIPE program, now admitting into a single Master's program twice a year — suggests the standalone "UTIPE Master's" entry point may itself have changed; unconfirmed by primary source.</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Spring or Autumn intake (two cycles/year)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Spring intake: document submission window ~14-17 Oct annually (confirmed for the Spring 2026 cohort: 14-17 Oct 2025, results ~11 Nov 2025), so the next window is expected ~mid-Oct 2026 for Spring 2027 entry. Autumn intake: opens ~April, exact window not confirmed this pass.</t>
+          <t>Not yet confirmed — needs manual check</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>tba</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>At least 1 recommendation letter required (AO exam route requires an English-language Letter of Recommendation); exact number for other routes not specified</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>~JPY 30,000 reported (university-wide general graduate-school figure, not confirmed Economics-specific)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>~JPY 535,800/year reported (university-wide figure, not confirmed Economics-PhD-specific)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible)</t>
+          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>MEXT scholarship route confirmed to exist, administered via a separate central international-office page (requires embassy/consulate preliminary candidacy). No department-specific stipend/assistantship figures found.</t>
+          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
@@ -4224,24 +4224,24 @@
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration (official PDF/page blocked direct fetch by an SSL certificate error); urgency upgraded from tba to soon</t>
+          <t>Site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>Partially complete — fee figures are university-wide, not Economics-PhD-confirmed; exact Autumn-intake window still needed</t>
+          <t>INCOMPLETE — the official site has now failed to resolve on five consecutive passes; a manual browser check is recommended rather than further automated retries. The 2023 admission-policy restriction is corroborated by multiple search snippets quoting the official pages, but still not confirmed via a direct primary-source fetch.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4251,17 +4251,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD)</t>
+          <t>Graduate School of Economics (PhD)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Seoul National University (SNU)</t>
+          <t>Hitotsubashi University</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>#189</t>
+          <t>#390 (confirmed still outside global top 300)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -4271,77 +4271,77 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Seoul</t>
+          <t>Tokyo (Kunitachi)</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://en.snu.ac.kr/admission</t>
+          <t>https://www.econ.hit-u.ac.jp/eng/page/graduate/admission.html</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>6.0 minimum (university-wide standard)</t>
+          <t>Not stated (page mentions TOEFL/TOEIC only)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>iBT 80, or TEPS 551 (university-wide standard, alternative to IELTS)</t>
+          <t>TOEFL or TOEIC score required as part of application materials; specific minimum score not stated</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Not required (no GRE requirement found in central admissions materials)</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
+          <t>Two intakes/year (Spring and Autumn); international applicants without a Hitotsubashi Master's apply via an AO exam route — either general AO (2+ years work experience post-master's) or AO for international applicants with a Master's from outside Japan; admission mainly via submitted documents, interview may follow (online option for overseas applicants)</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Spring or Autumn intake (two cycles/year)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>University-wide pattern: Fall-intake applications open ~early March (2026 Fall: 3-5 Mar); Spring-intake applications open ~early July (2027 Spring: 6-9 Jul) — both 2026 cycles already closed; 2027 Fall cycle not yet announced. Department-specific PhD deadline still not separately confirmed.</t>
+          <t>Spring intake: document submission window ~14-17 Oct annually (confirmed for the Spring 2026 cohort: 14-17 Oct 2025, results ~11 Nov 2025), so the next window is expected ~mid-Oct 2026 for Spring 2027 entry. Autumn intake: opens ~April, exact window not confirmed this pass.</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>later</t>
+          <t>urgent</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>At least 1 recommendation letter required (AO exam route requires an English-language Letter of Recommendation); exact number for other routes not specified</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>KRW 90,000 (no fee waivers offered)</t>
+          <t>~JPY 30,000 reported (university-wide general graduate-school figure, not confirmed Economics-specific)</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>~JPY 535,800/year reported (university-wide figure, not confirmed Economics-PhD-specific)</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Likely (university-wide scholarships only)</t>
+          <t>Likely (MEXT scholarship-eligible)</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Confirmed via direct fetch of the Department of Economics' own PhD page: no department-specific funding scheme exists — funding runs entirely through the university-wide scholarships above.</t>
+          <t>MEXT scholarship route confirmed to exist, administered via a separate central international-office page (requires embassy/consulate preliminary candidacy). No department-specific stipend/assistantship figures found.</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
@@ -4351,24 +4351,24 @@
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; admissions and funding run entirely through the university-wide portal and scholarships</t>
+          <t>Spring-intake submission window (expected ~14-17 Oct 2026) is now within 30 days — urgency upgraded from soon to urgent, 30-day reminder flag set</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>Confirmed (Aug 2026) that Economics PhD funding at SNU is university-wide only, with no departmental top-up scheme; department page exists but defers entirely to the central international-admissions portal for deadlines/fees</t>
+          <t>Partially complete — fee figures are university-wide, not Economics-PhD-confirmed; the 14-17 Oct 2026 window is an estimate based on the recurring annual pattern (confirmed dates were for the Spring 2026 cohort), not yet directly reconfirmed for this cycle — recommend a manual spot-check closer to the date</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ASA-08</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4378,17 +4378,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PhD in Business (Economics track)</t>
+          <t>Department of Economics (PhD)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>University of Hong Kong (Faculty of Business and Economics)</t>
+          <t>Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>#106</t>
+          <t>#189</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -4398,104 +4398,104 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Seoul</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://phd.hkubs.hku.hk/admissions/admission-application-and-tuition-fee</t>
+          <t>https://en.snu.ac.kr/admission</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Academic overall 6.5, all subtests &gt;= 6.0 (waived if prior degree was taught in English)</t>
+          <t>6.0 minimum (university-wide standard)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>iBT &gt;= 85</t>
+          <t>iBT 80, or TEPS 551 (university-wide standard, alternative to IELTS)</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>GRE or GMAT required, score &lt;5 years old (institution codes: GRE 2482, GMAT FS2-WL-48)</t>
+          <t>Not required (no GRE requirement found in central admissions materials)</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Bachelor's with first-class honours (or equivalent), or Bachelor's + Master's from a recognized university; 3-year track with a research Master's, 4-year track without one; Economics is one of six FBE PhD fields</t>
+          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Fall semester, normally September (matriculates once a year)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Applications open 1 September; Main Round closes 1 December (recurring annual cycle; late applications considered only if places remain)</t>
+          <t>University-wide pattern: Fall-intake applications open ~early March (2026 Fall: 3-5 Mar); Spring-intake applications open ~early July (2027 Spring: 6-9 Jul) — both 2026 cycles already closed; 2027 Fall cycle not yet announced. Department-specific PhD deadline still not separately confirmed.</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2 (academic referee reports, submitted directly by referees)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>HK$600 (paid online via HKU Graduate School application system)</t>
+          <t>KRW 90,000 (no fee waivers offered)</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>HK$49,500/year (2027-28 rate) for full-time PhD — typically waived/covered for scholarship holders</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Likely (university-wide scholarships only)</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>Standard Postgraduate Scholarship (PGS) pays HK$19,135/month (rising to HK$19,655/month once candidature is confirmed), available to essentially all admitted PhD students regardless of HKPFS status. HKPFS awardees instead receive HK$28,700/month plus HK$14,400/year travel allowance for up to 3 years.</t>
+          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Confirmed via direct fetch of the Department of Economics' own PhD page: no department-specific funding scheme exists — funding runs entirely through the university-wide scholarships above.</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; admissions and funding run entirely through the university-wide portal and scholarships</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>Distinct from the cross-institution HKPFS scheme already tracked (ASA-03) — nearly all admitted PhD students get baseline PGS funding here even without winning HKPFS, a broader guarantee than HKPFS alone.</t>
+          <t>Confirmed (Aug 2026) that Economics PhD funding at SNU is university-wide only, with no departmental top-up scheme; department page exists but defers entirely to the central international-admissions portal for deadlines/fees</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4505,17 +4505,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD in Business (Economics track)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>#369 — confirmed via direct fetch of the live RePEc table</t>
+          <t>#106</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -4535,37 +4535,37 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://admission.econ.cuhk.edu.hk/pg/phd-economics/</t>
+          <t>https://phd.hkubs.hku.hk/admissions/admission-application-and-tuition-fee</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Academic overall 6.5</t>
+          <t>Academic overall 6.5, all subtests &gt;= 6.0 (waived if prior degree was taught in English)</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>79 iBT (or 4.5-6.0 Home Edition) — see IELTS field for alternatives (GMAT Verbal &gt;=21, or a degree from an English-medium institution, also accepted)</t>
+          <t>iBT &gt;= 85</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Required (institution code 3153, department code 1801); no published hard cutoff, but absence of a score disadvantages applicants</t>
+          <t>GRE or GMAT required, score &lt;5 years old (institution codes: GRE 2482, GMAT FS2-WL-48)</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Master's in economics or a related field with a strong math/stats background expected; strong bachelor's-only applicants can also apply with sufficient research potential. Official transcripts, degree certificates, a 5-page research proposal and/or working papers, resume, and typically an interview all required</t>
+          <t>Bachelor's with first-class honours (or equivalent), or Bachelor's + Master's from a recognized university; 3-year track with a research Master's, 4-year track without one; Economics is one of six FBE PhD fields</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Fall intake (standard)</t>
+          <t>Fall semester, normally September (matriculates once a year)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Applications open 1 Sept 2026; HKPFS-track deadline 1 Dec 2026 (11:59am); non-HKPFS deadline 1 Dec 2026 (11:59pm); referee letters due by 4 Dec 2026</t>
+          <t>Applications open 1 September; Main Round closes 1 December (recurring annual cycle; late applications considered only if places remain)</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -4575,54 +4575,54 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>3 confidential recommendation letters</t>
+          <t>2 (academic referee reports, submitted directly by referees)</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>HK$500 per programme</t>
+          <t>HK$600 (paid online via HKU Graduate School application system)</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>HK$47,000 (2026/27) / HK$49,500 (2027/28)</t>
+          <t>HK$49,500/year (2027-28 rate) for full-time PhD — typically waived/covered for scholarship holders</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>Yes — guaranteed assistantship for all admits</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>All successful full-time PhD admits receive a teaching/research assistantship with a monthly stipend of ~HK$19,100. HKPFS awardees additionally receive a full tuition waiver plus HK$40,000 (year 1) / HK$20,000/year (subsequent years) and housing benefits. Local students separately receive a government tuition waiver. Cross-reference the cross-institution HKPFS scheme already tracked (ASA-03).</t>
+          <t>Standard Postgraduate Scholarship (PGS) pays HK$19,135/month (rising to HK$19,655/month once candidature is confirmed), available to essentially all admitted PhD students regardless of HKPFS status. HKPFS awardees instead receive HK$28,700/month plus HK$14,400/year travel allowance for up to 3 years.</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>New find Aug 2026; distinct from HKU (ASA-08) and the cross-institution HKPFS scheme (ASA-03) — CUHK guarantees baseline assistantship funding to all admits independent of HKPFS.</t>
+          <t>Distinct from the cross-institution HKPFS scheme already tracked (ASA-03) — nearly all admitted PhD students get baseline PGS funding here even without winning HKPFS, a broader guarantee than HKPFS alone.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4637,62 +4637,62 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Australian National University (ANU)</t>
+          <t>Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>#124</t>
+          <t>#369 — confirmed via direct fetch of the live RePEc table</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Canberra</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
+          <t>https://admission.econ.cuhk.edu.hk/pg/phd-economics/</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>6.5 overall (no band below 6.0)</t>
+          <t>Academic overall 6.5</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>570 (paper-based; essay ≥4.5)</t>
+          <t>79 iBT (or 4.5-6.0 Home Edition) — see IELTS field for alternatives (GMAT Verbal &gt;=21, or a degree from an English-medium institution, also accepted)</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
+          <t>Required (institution code 3153, department code 1801); no published hard cutoff, but absence of a score disadvantages applicants</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
+          <t>Master's in economics or a related field with a strong math/stats background expected; strong bachelor's-only applicants can also apply with sufficient research potential. Official transcripts, degree certificates, a 5-page research proposal and/or working papers, resume, and typically an interview all required</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>February (Semester 1); Semester 2 entry possible (July)</t>
+          <t>Fall intake (standard)</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>For Feb 2027 start: international scholarship deadline (31 Aug 2026) has now closed; the standard/domestic deadline of 31 Oct 2026 is the next live deadline (confirmed via search corroboration, ANU site still returning HTTP 504 to direct fetch); Sem 2 entry deadline (31 Mar) also already closed for this cycle</t>
+          <t>Applications open 1 Sept 2026; HKPFS-track deadline 1 Dec 2026 (11:59am); non-HKPFS deadline 1 Dec 2026 (11:59pm); referee letters due by 4 Dec 2026</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -4702,32 +4702,32 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3 confidential recommendation letters</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$500 per programme</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$47,000 (2026/27) / HK$49,500 (2027/28)</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — guaranteed assistantship for all admits</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>Australian Government RTP Stipend: AUD $39,069/year (2026 full-time base rate, ANU-wide), paid fortnightly, up to 3.5 years. Some HDR supplementary scholarships add AUD $7,000/year on top, for up to 3 years. Domestic candidates pay no tuition (RTP-covered); international candidates can compete for HDR Fee Remission Merit Scholarships covering up to 4 years.</t>
+          <t>All successful full-time PhD admits receive a teaching/research assistantship with a monthly stipend of ~HK$19,100. HKPFS awardees additionally receive a full tuition waiver plus HK$40,000 (year 1) / HK$20,000/year (subsequent years) and housing benefits. Local students separately receive a government tuition waiver. Cross-reference the cross-institution HKPFS scheme already tracked (ASA-03).</t>
         </is>
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
@@ -4737,19 +4737,19 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline — reset reminder flags for the new date</t>
+          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026 — international-applicant deadline has closed; domestic deadline (31 Oct 2026) is next</t>
+          <t>New find Aug 2026; distinct from HKU (ASA-08) and the cross-institution HKPFS scheme (ASA-03) — CUHK guarantees baseline assistantship funding to all admits independent of HKPFS.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4759,17 +4759,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>University of Melbourne</t>
+          <t>Australian National University (ANU)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>#151</t>
+          <t>#124</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4784,42 +4784,42 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Melbourne</t>
+          <t>Canberra</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
+          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
+          <t>6.5 overall (no band below 6.0)</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>94 iBT (W27/S18/R13/L13)</t>
+          <t>570 (paper-based; essay ≥4.5)</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Not mentioned in entry requirements</t>
+          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
+          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>March intake</t>
+          <t>February (Semester 1); Semester 2 entry possible (July)</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>March 2027 intake deadline reported as 30 November 2026 — found via search summary only; the official how-to-apply/key-dates pages returned HTTP 403 on every direct fetch attempt this pass, so this date is unconfirmed by primary source and should be manually verified</t>
+          <t>For Feb 2027 start: international scholarship deadline (31 Aug 2026) has now closed; the standard/domestic deadline of 31 Oct 2026 is the next live deadline (confirmed via search corroboration, ANU site still returning HTTP 504 to direct fetch); Sem 2 entry deadline (31 Mar) also already closed for this cycle</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -4829,17 +4829,17 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Not detailed — full tuition fee waiver reported (see funding)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -4849,7 +4849,7 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>Australian Government Research Training Program (RTP) funded places available: RTP stipend reported at AUD $39,500/year (2026 rate) plus full tuition fee waiver and AUD $15,000 research/conference travel funding for confirmed PhD candidates (unconfirmed by primary source — see deadline note). Program structure: 2-year Master of Commerce coursework + 3-year PhD.</t>
+          <t>Australian Government RTP Stipend: AUD $39,069/year (2026 full-time base rate, ANU-wide), paid fortnightly, up to 3.5 years. Some HDR supplementary scholarships add AUD $7,000/year on top, for up to 3 years. Domestic candidates pay no tuition (RTP-covered); international candidates can compete for HDR Fee Remission Merit Scholarships covering up to 4 years.</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
@@ -4859,24 +4859,24 @@
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>Found a reported deadline and funding figures via search, but could not confirm via direct page fetch (403 blocked) — flagged as lower confidence</t>
+          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline — reset reminder flags for the new date</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches this pass — recommend a manual browser check before relying on the reported 30 Nov 2026 deadline</t>
+          <t>Seed entry Aug 2026 — international-applicant deadline has closed; domestic deadline (31 Oct 2026) is next</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4886,17 +4886,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PhD (Economics)</t>
+          <t>Doctoral Program in Economics</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Monash Business School</t>
+          <t>University of Melbourne</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>#46</t>
+          <t>#151</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4911,42 +4911,42 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Melbourne (Clayton)</t>
+          <t>Melbourne</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
+          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>7.0 minimum reported (third-party source, not confirmed on official Monash page — page returned HTTP 403 to direct fetch)</t>
+          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>94 minimum reported (same caveat as IELTS — unconfirmed by primary source)</t>
+          <t>94 iBT (W27/S18/R13/L13)</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Not mentioned in entry requirements</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
+          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>March intake</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Integrated-pathway Feb/Semester-1 entry window (1 Jul-31 Aug) has closed; next integrated-pathway window (Jul/Semester-2 entry) opens ~1 Dec-1 Feb. Separately, general Graduate Research Scholarship rounds: international Round 3 (~31 Jul/31 Aug) has closed; domestic Round 4 closes 31 Oct 2026 (confirmed via search, monash.edu still blocking direct fetch with HTTP 403) — this is the next live deadline.</t>
+          <t>March 2027 intake deadline reported as 30 November 2026 — found via search summary only; the official how-to-apply/key-dates pages returned HTTP 403 on every direct fetch attempt this pass, so this date is unconfirmed by primary source and should be manually verified</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -4961,12 +4961,12 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>International ~AUD $38,900/yr, domestic ~AUD $37,100/yr reported (third-party aggregator source, not confirmed by official Monash page)</t>
+          <t>Not detailed — full tuition fee waiver reported (see funding)</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -4976,7 +4976,7 @@
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places — general RTP stipend reported at AUD $37,145/yr (2026 rate) plus a $1,500 relocation allowance (not confirmed Economics-specific).</t>
+          <t>Australian Government Research Training Program (RTP) funded places available: RTP stipend reported at AUD $39,500/year (2026 rate) plus full tuition fee waiver and AUD $15,000 research/conference travel funding for confirmed PhD candidates (unconfirmed by primary source — see deadline note). Program structure: 2-year Master of Commerce coursework + 3-year PhD.</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
@@ -4986,24 +4986,24 @@
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>Confirmed the ~31 Aug 2026 integrated-pathway and international-round deadlines have closed; domestic Graduate Research Scholarship Round 4 (31 Oct 2026) is the next live deadline — reset reminder flags for the new date</t>
+          <t>Found a reported deadline and funding figures via search, but could not confirm via direct page fetch (403 blocked) — flagged as lower confidence</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; monash.edu has blocked all automated fetches on every pass so far (scholarships-and-fees, apply, and program pages all 403'd) — every figure in this entry is lower-confidence (search snippets/third-party aggregator only) and needs a manual browser check</t>
+          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches this pass — recommend a manual browser check before relying on the reported 30 Nov 2026 deadline</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5013,17 +5013,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD (Economics)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>University of Sydney</t>
+          <t>Monash Business School</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>#87</t>
+          <t>#46</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -5038,32 +5038,32 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Sydney</t>
+          <t>Melbourne (Clayton)</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://www.sydney.edu.au/scholarships/</t>
+          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>7.0 minimum reported (third-party source, not confirmed on official Monash page — page returned HTTP 403 to direct fetch)</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>94 minimum reported (same caveat as IELTS — unconfirmed by primary source)</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP. Material finding: Sydney has no dedicated 'PhD in Economics' program page — the Economics coursework handbook explicitly states it "does not include a research component and thus does not provide a pathway to higher degree by research (e.g. PhD) studies." PhD study is pursued via the general Doctor of Philosophy degree with a nominated Economics supervisor/discipline, not a single named landing page.</t>
+          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -5073,7 +5073,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Research Period 1 &amp; 2 deadline (11 September 2026) has now passed; Research Period 3 &amp; 4 — deadline 18 December 2026 — is the next live RTP scholarship round (reconfirmed via search, not a directly-fetched dedicated Economics PhD page).</t>
+          <t>Integrated-pathway Feb/Semester-1 entry window (1 Jul-31 Aug) has closed; next integrated-pathway window (Jul/Semester-2 entry) opens ~1 Dec-1 Feb. Separately, general Graduate Research Scholarship rounds: international Round 3 (~31 Jul/31 Aug) has closed; domestic Round 4 closes 31 Oct 2026 (confirmed via search, monash.edu still blocking direct fetch with HTTP 403) — this is the next live deadline.</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -5083,7 +5083,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>1 (for named scholarship example; general program may differ)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>International ~AUD $38,900/yr, domestic ~AUD $37,100/yr reported (third-party aggregator source, not confirmed by official Monash page)</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -5103,7 +5103,7 @@
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly; a 2027-rate RTP stipend of AUD $44,293/yr was also reported via search aggregators this pass (unconfirmed by primary source).</t>
+          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places — general RTP stipend reported at AUD $37,145/yr (2026 rate) plus a $1,500 relocation allowance (not confirmed Economics-specific).</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
@@ -5113,24 +5113,24 @@
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down from urgent to soon, reminder flags reset for the new deadline</t>
+          <t>Confirmed the ~31 Aug 2026 integrated-pathway and international-round deadlines have closed; domestic Graduate Research Scholarship Round 4 (31 Oct 2026) is the next live deadline — reset reminder flags for the new date</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check; no dedicated Economics-specific PhD admissions page exists at Sydney</t>
+          <t>Seed entry Aug 2026; monash.edu has blocked all automated fetches on every pass so far (scholarships-and-fees, apply, and program pages all 403'd) — every figure in this entry is lower-confidence (search snippets/third-party aggregator only) and needs a manual browser check</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AUS-05</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -5145,12 +5145,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>UNSW Sydney</t>
+          <t>University of Sydney</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>#80</t>
+          <t>#87</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -5170,67 +5170,67 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://www.unsw.edu.au/business/study-with-us/postgraduate-research/phd-degrees/doctor-philosophy-phd-economics</t>
+          <t>https://www.sydney.edu.au/scholarships/</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Not listed on this page (exemptions for AU/CA/UK/US/NZ citizens); non-English-speaking-country applicants need IELTS/TOEFL/PTE/Cambridge or the UNSW Global English Course</t>
+          <t>Not specified at general program level</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Not listed on this page — see IELTS field for alternatives</t>
+          <t>Not specified at general program level</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Optional but recommended overall; one source indicates GRE may be specifically required for the Economics stream — this conflicts with the general 'optional' language elsewhere and needs manual confirmation</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course. Program begins with a 1-year Master of Pre-Doctoral Business Studies, followed by 3-3.5 years of doctoral research; direct entry to the 3-year PhD is possible for candidates with first-class Honours/Master's plus independent funding (Stream 2).</t>
+          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP. Material finding: Sydney has no dedicated 'PhD in Economics' program page — the Economics coursework handbook explicitly states it "does not include a research component and thus does not provide a pathway to higher degree by research (e.g. PhD) studies." PhD study is pursued via the general Doctor of Philosophy degree with a nominated Economics supervisor/discipline, not a single named landing page.</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Term 1 – February</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Confirmed still closed as of 23 Aug 2026 (verified directly on program page): EOI window opened 20 March 2026, closed 15 August 2026, no newer/next EOI window posted. Note: a separate 26 August 2026 formal-application deadline exists, but it applies only to candidates already invited to apply from the closed EOI round, not to new applicants.</t>
+          <t>Research Period 1 &amp; 2 deadline (11 September 2026) has now passed; Research Period 3 &amp; 4 — deadline 18 December 2026 — is the next live RTP scholarship round (reconfirmed via search, not a directly-fetched dedicated Economics PhD page).</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
+          <t>1 (for named scholarship example; general program may differ)</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr">
+      <c r="S37" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t>Not detailed (fully funded — see funding)</t>
-        </is>
-      </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>Yes — all admitted students</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>Full tuition waiver + stipend AUD 35,000-45,000/yr, up to 4.5 years (+1 optional fellowship year), plus substantial research/conference travel funding.</t>
+          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly; a 2027-rate RTP stipend of AUD $44,293/yr was also reported via search aggregators this pass (unconfirmed by primary source).</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
@@ -5240,142 +5240,269 @@
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>Confirmed EOI window remains closed with no new window announced; added program structure and English-test details</t>
+          <t>11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down from urgent to soon, reminder flags reset for the new deadline</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026 — EOI window closed 15 Aug 2026, still no next window announced as of this update</t>
+          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check; no dedicated Economics-specific PhD admissions page exists at Sydney</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>AUS-05</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>PhD in Economics</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>UNSW Sydney</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>#80</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://www.unsw.edu.au/business/study-with-us/postgraduate-research/phd-degrees/doctor-philosophy-phd-economics</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Not listed on this page (exemptions for AU/CA/UK/US/NZ citizens); non-English-speaking-country applicants need IELTS/TOEFL/PTE/Cambridge or the UNSW Global English Course</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Not listed on this page — see IELTS field for alternatives</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Optional but recommended overall; one source indicates GRE may be specifically required for the Economics stream — this conflicts with the general 'optional' language elsewhere and needs manual confirmation</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course. Program begins with a 1-year Master of Pre-Doctoral Business Studies, followed by 3-3.5 years of doctoral research; direct entry to the 3-year PhD is possible for candidates with first-class Honours/Master's plus independent funding (Stream 2).</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Term 1 – February</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Confirmed still closed as of 23 Aug 2026 (verified directly on program page): EOI window opened 20 March 2026, closed 15 August 2026, no newer/next EOI window posted. Note: a separate 26 August 2026 formal-application deadline exists, but it applies only to candidates already invited to apply from the closed EOI round, not to new applicants.</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Not detailed (fully funded — see funding)</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Yes — all admitted students</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Full tuition waiver + stipend AUD 35,000-45,000/yr, up to 4.5 years (+1 optional fellowship year), plus substantial research/conference travel funding.</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>Confirmed EOI window remains closed with no new window announced; added program structure and English-test details</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026 — EOI window closed 15 Aug 2026, still no next window announced as of this update</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>AUS-06</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>Doctor of Philosophy (Economics)</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>University of Queensland (School of Economics)</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>#71</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>Brisbane</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>https://economics.uq.edu.au/study/phd</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>Academic overall 6.5, with 6.0 minimum in each of reading/writing/speaking/listening</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>Not specified on the economics-specific page (UQ university-wide PhD pages generally accept TOEFL iBT as an alternative to IELTS)</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>Not confirmed as required; application package can include GRE/GMAT score sheets, suggesting optional/supplementary rather than mandatory</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="M39" t="inlineStr">
         <is>
           <t>Academic CV, transcripts; MPhil/research master's options also available; can join a funded project with scholarship support as an alternative entry route</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
+      <c r="N39" t="inlineStr">
         <is>
           <t>Quarterly intakes (research quarters begin 1 Jan, 1 Apr, 1 Jul, 1 Oct); applications for RHD programs can be submitted any time</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr">
+      <c r="O39" t="inlineStr">
         <is>
           <t>Domestic Round 1 (31 Aug 2026) has now closed; the International round deadline of 19 Oct 2026 is confirmed still live via search corroboration and is the next relevant deadline for upcoming 2027 research quarters.</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr">
+      <c r="P39" t="inlineStr">
         <is>
           <t>soon</t>
         </is>
       </c>
-      <c r="Q38" t="inlineStr">
+      <c r="Q39" t="inlineStr">
         <is>
           <t>Minimum 2 referee reports</t>
         </is>
       </c>
-      <c r="R38" t="inlineStr">
+      <c r="R39" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="S38" t="inlineStr">
+      <c r="S39" t="inlineStr">
         <is>
           <t>Not specified (international RTP scholarship recipients typically get a full tuition fee offset)</t>
         </is>
       </c>
-      <c r="T38" t="inlineStr">
+      <c r="T39" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
+      <c r="U39" t="inlineStr">
         <is>
           <t>RTP/UQGRSS provides a tax-free living stipend of AUD $39,220/year (2026 rate, indexed annually — updated from a previously-recorded AUD $37,500 figure) plus, for eligible international candidates, a tuition fee offset; no separate application needed beyond the program EOI.</t>
         </is>
       </c>
-      <c r="V38" t="inlineStr">
+      <c r="V39" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="W38" t="inlineStr">
-        <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
-      <c r="X38" t="inlineStr">
-        <is>
-          <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026) — reset reminder flags for the new date</t>
-        </is>
-      </c>
-      <c r="Y38" t="inlineStr">
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>International round deadline (19 Oct 2026) is now within 30 days — 30-day reminder flag set</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
         <is>
           <t>Scholarship is university-wide (RTP/UQGRSS), not economics-specific, but School of Economics PhD candidates are eligible.</t>
         </is>
@@ -5392,7 +5519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5432,44 +5559,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>EUR-23</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>PhD in Economics (Quantitative Economics track) — Goethe University Frankfurt (GSEFM)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>The 11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down to soon, reminder flags reset.</t>
+          <t>New find: RePEc #81, up to three competitive first-year IMFS stipends plus post-qualifying-exam TA/RA positions; no tuition fees.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -5479,34 +5606,34 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>30-day reminder: the early-round deadline (30 Sep 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
+          <t>30-day reminder: the Spring-intake submission window (expected ~14-17 Oct 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Official site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025.</t>
+          <t>30-day reminder: the international round deadline (19 Oct 2026) is now within 30 days.</t>
         </is>
       </c>
     </row>
@@ -5518,66 +5645,66 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>EUR-22</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Cambridge</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>New find: RePEc #50, ~66% of Cambridge doctoral students fully funded via Cambridge Trust/Gates Cambridge/College/ESRC funding; funding-competition deadline 8 Dec 2026.</t>
+          <t>The 11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down to soon, reminder flags reset.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline, urgency moved from urgent to soon.</t>
+          <t>30-day reminder: the early-round deadline (30 Sep 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -5587,34 +5714,34 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Confirmed the integrated-pathway and international scholarship round deadlines have closed; now tracking the domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026), urgency moved from urgent to soon.</t>
+          <t>Official site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>EUR-22</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>PhD in Economics — University of Cambridge</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>7-day reminder: the 11 Sep 2026 Research Period 1 &amp; 2 deadline is confirmed still live and now imminent.</t>
+          <t>New find: RePEc #50, ~66% of Cambridge doctoral students fully funded via Cambridge Trust/Gates Cambridge/College/ESRC funding; funding-competition deadline 8 Dec 2026.</t>
         </is>
       </c>
     </row>
@@ -5626,12 +5753,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -5641,7 +5768,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026), urgency moved from urgent to soon.</t>
+          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline, urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -5653,12 +5780,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EUR-17</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -5668,7 +5795,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#192) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>Confirmed the integrated-pathway and international scholarship round deadlines have closed; now tracking the domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026), urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -5680,22 +5807,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EUR-18</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#24) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>7-day reminder: the 11 Sep 2026 Research Period 1 &amp; 2 deadline is confirmed still live and now imminent.</t>
         </is>
       </c>
     </row>
@@ -5707,12 +5834,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EUR-19</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -5722,7 +5849,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#40) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026), urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -5734,12 +5861,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EUR-20</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -5749,7 +5876,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#164) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>Confirmed RePEc rank (#192) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
@@ -5761,12 +5888,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -5776,7 +5903,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>Confirmed RePEc rank (#24) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
@@ -5788,12 +5915,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -5803,7 +5930,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Official site remains unreachable (DNS failure, fourth consecutive pass); recommend a manual browser check rather than further automated retries.</t>
+          <t>Confirmed RePEc rank (#40) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
@@ -5815,93 +5942,93 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EUR-21</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PhD in Economics — Sciences Po</t>
+          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>New find: RePEc #42, funded via a 3-year Doctoral Contract (~EUR 2,100/month) plus tuition exemption; some applicants expected to already hold external funding.</t>
+          <t>Confirmed RePEc rank (#164) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>EUR-17</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
+          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>New find: FWF-grant-funded PhD positions at the University of Vienna; admission-round dates inconsistent across sources, recommend a manual spot-check.</t>
+          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>EUR-18</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>New find: PhD structured as a salaried employment contract (~EUR 2,750-3,500/month); official site blocked automated fetches, several fields search-only.</t>
+          <t>Official site remains unreachable (DNS failure, fourth consecutive pass); recommend a manual browser check rather than further automated retries.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>EUR-19</t>
+          <t>EUR-21</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
+          <t>PhD in Economics — Sciences Po</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -5911,7 +6038,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>New find: RePEc ~#40, funded PhD positions up to 4 years plus IRO Doctoral Scholarships for developing-country students; deadlines are vacancy-by-vacancy.</t>
+          <t>New find: RePEc #42, funded via a 3-year Doctoral Contract (~EUR 2,100/month) plus tuition exemption; some applicants expected to already hold external funding.</t>
         </is>
       </c>
     </row>
@@ -5923,12 +6050,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>EUR-20</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -5938,7 +6065,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>New find: joint Berlin-area doctoral school, funded via a EUR 1,650/month qualification-phase stipend then dissertation-phase employment.</t>
+          <t>New find: FWF-grant-funded PhD positions at the University of Vienna; admission-round dates inconsistent across sources, recommend a manual spot-check.</t>
         </is>
       </c>
     </row>
@@ -5950,12 +6077,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -5965,7 +6092,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>New find: guaranteed teaching/research assistantship (~HK$19,100/month) for all admits, independent of the HKPFS scheme already tracked (ASA-03).</t>
+          <t>New find: PhD structured as a salaried employment contract (~EUR 2,750-3,500/month); official site blocked automated fetches, several fields search-only.</t>
         </is>
       </c>
     </row>
@@ -5977,22 +6104,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Confirmed application windows (Aug intake: 1 Oct-15 Nov; Jan intake: 1 Jun-31 Jul), referee/fee requirements, and Graduate Assistantship Programme detail via direct official fetch; urgency upgraded from tba to soon.</t>
+          <t>New find: RePEc ~#40, funded PhD positions up to 4 years plus IRO Doctoral Scholarships for developing-country students; deadlines are vacancy-by-vacancy.</t>
         </is>
       </c>
     </row>
@@ -6004,22 +6131,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Corroborated via search snippets (site unreachable for a third consecutive pass) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad.</t>
+          <t>New find: joint Berlin-area doctoral school, funded via a EUR 1,650/month qualification-phase stipend then dissertation-phase employment.</t>
         </is>
       </c>
     </row>
@@ -6031,22 +6158,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration; urgency upgraded from tba to soon.</t>
+          <t>New find: guaranteed teaching/research assistantship (~HK$19,100/month) for all admits, independent of the HKPFS scheme already tracked (ASA-03).</t>
         </is>
       </c>
     </row>
@@ -6058,12 +6185,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -6073,7 +6200,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; funding runs entirely through university-wide scholarships.</t>
+          <t>Confirmed application windows (Aug intake: 1 Oct-15 Nov; Jan intake: 1 Jun-31 Jul), referee/fee requirements, and Graduate Assistantship Programme detail via direct official fetch; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
@@ -6085,22 +6212,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>7-day reminder: the 31 Aug 2026 international scholarship deadline is confirmed still live via search corroboration (ANU site returned HTTP 504 to direct fetch).</t>
+          <t>Corroborated via search snippets (site unreachable for a third consecutive pass) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad.</t>
         </is>
       </c>
     </row>
@@ -6112,22 +6239,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>7-day reminder: the imminent ~31 Aug 2026 integrated-pathway deadline is reconfirmed via search (monash.edu still blocking direct fetch); added a general RTP stipend figure (AUD $37,145/yr).</t>
+          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
@@ -6139,103 +6266,103 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>7-day reminder: confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to AUD $39,220/yr (2026 rate).</t>
+          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; funding runs entirely through university-wide scholarships.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
+          <t>7-day reminder: the 31 Aug 2026 international scholarship deadline is confirmed still live via search corroboration (ANU site returned HTTP 504 to direct fetch).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
+          <t>7-day reminder: the imminent ~31 Aug 2026 integrated-pathway deadline is reconfirmed via search (monash.edu still blocking direct fetch); added a general RTP stipend figure (AUD $37,145/yr).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
+          <t>7-day reminder: confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to AUD $39,220/yr (2026 rate).</t>
         </is>
       </c>
     </row>
@@ -6247,12 +6374,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -6262,7 +6389,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
+          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
         </is>
       </c>
     </row>
@@ -6274,12 +6401,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -6289,7 +6416,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
+          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
         </is>
       </c>
     </row>
@@ -6301,12 +6428,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -6316,7 +6443,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
+          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
         </is>
       </c>
     </row>
@@ -6328,12 +6455,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -6343,7 +6470,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
+          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
         </is>
       </c>
     </row>
@@ -6355,12 +6482,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -6370,7 +6497,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
+          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
         </is>
       </c>
     </row>
@@ -6382,12 +6509,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -6397,7 +6524,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
         </is>
       </c>
     </row>
@@ -6409,12 +6536,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -6424,7 +6551,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
+          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
         </is>
       </c>
     </row>
@@ -6436,12 +6563,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -6451,7 +6578,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
+          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
         </is>
       </c>
     </row>
@@ -6463,12 +6590,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -6478,7 +6605,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
+          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
         </is>
       </c>
     </row>
@@ -6490,12 +6617,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -6505,7 +6632,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
+          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -6517,12 +6644,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>AUS-05</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>PhD in Economics — UNSW Sydney</t>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -6532,7 +6659,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
+          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
         </is>
       </c>
     </row>
@@ -6544,22 +6671,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>EUR-13</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
+          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -6571,22 +6698,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>EUR-14</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
+          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -6598,22 +6725,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>EUR-15</t>
+          <t>AUS-05</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
+          <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
+          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
         </is>
       </c>
     </row>
@@ -6625,12 +6752,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>EUR-16</t>
+          <t>EUR-13</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
+          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -6640,7 +6767,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
+          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
         </is>
       </c>
     </row>
@@ -6652,12 +6779,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ASA-08</t>
+          <t>EUR-14</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
+          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -6667,7 +6794,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
+          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
         </is>
       </c>
     </row>
@@ -6679,12 +6806,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>EUR-15</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -6694,88 +6821,88 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
+          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>EUR-16</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>EUR-03</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
         </is>
       </c>
     </row>
@@ -6787,12 +6914,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>EUR-04</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6814,12 +6941,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>EUR-05</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PhD in Economics — CEMFI</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6841,12 +6968,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>EUR-06</t>
+          <t>EUR-03</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
+          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6868,12 +6995,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>EUR-07</t>
+          <t>EUR-04</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PhD Program — Paris School of Economics (PSE)</t>
+          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6895,12 +7022,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EUR-08</t>
+          <t>EUR-05</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — Stockholm University / IIES</t>
+          <t>PhD in Economics — CEMFI</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -6922,12 +7049,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EUR-09</t>
+          <t>EUR-06</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>MPhil + DPhil in Economics — University of Oxford</t>
+          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -6949,12 +7076,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>EUR-07</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>PhD Program — Paris School of Economics (PSE)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -6976,12 +7103,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>EUR-08</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>PhD Programme in Economics — Stockholm University / IIES</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -7003,12 +7130,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>EUR-12</t>
+          <t>EUR-09</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
+          <t>MPhil + DPhil in Economics — University of Oxford</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -7030,12 +7157,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -7057,12 +7184,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -7084,12 +7211,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>EUR-12</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -7111,12 +7238,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -7138,12 +7265,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -7165,12 +7292,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-03</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -7192,12 +7319,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -7219,12 +7346,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -7246,12 +7373,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -7273,12 +7400,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -7300,12 +7427,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -7327,20 +7454,101 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
+          <t>AUS-02</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>AUS-03</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>PhD (Economics) — Monash Business School</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>AUS-04</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>PhD in Economics — University of Sydney</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
           <t>AUS-05</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D75" t="inlineStr">
         <is>
           <t>Added (seed)</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
+      <c r="E75" t="inlineStr">
         <is>
           <t>Initial research pass — program added to tracker.</t>
         </is>

</xml_diff>

<commit_message>
Econ ledger update 2026-09-26: 2 added, 7 updated, 0 reminder flags
Includes a correction to ASA-01 (NUS): the 30 Sep 2026 'early round' deadline
recorded on 14 Sep could not be re-substantiated and appears to have been an
error. Reset to the corroborated 1 Dec 2026 department deadline, urgency
stepped back to soon, reminder flag reset, and a correction notice posted to
the channel.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/EconGradAlert/data/tracker.xlsx
+++ b/apps/EconGradAlert/data/tracker.xlsx
@@ -438,7 +438,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last full research pass: 2026-09-19</t>
+          <t>Last full research pass: 2026-09-26</t>
         </is>
       </c>
     </row>
@@ -479,14 +479,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RePEc snapshot: July 2026</t>
+          <t>RePEc snapshot: August 2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Program count: 38</t>
+          <t>Program count: 40</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y39"/>
+  <dimension ref="A1:Y41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -755,7 +755,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1 Dec (scholarship/non-EEA) / 1 Feb (partner non-EEA &amp; EEA scholarship) / 1 May (EEA) — recurring; page also notes Cohort 2027-2029 admissions open in Studielink 1 Oct 2026, which is hard to reconcile with the Dec/Feb/May dates shown — cohort-year labeling on the official page is ambiguous, recommend a manual spot-check</t>
+          <t>Cohort 2027-2029 (confirmed directly on the official admissions page): admissions open in Studielink 1 Oct 2026; Round 1 deadline 1 Dec 2026 (open to all applicants, strongly recommended for scholarship consideration); Round 2 deadline 1 Feb 2027 (final deadline for non-EEA applicants not at partner institutions); Round 3 deadline 1 May 2027 (EEA citizens and non-EEA students at partner schools); rolling admissions until 15 Jun 2027 if places remain</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts</t>
+          <t>Resolved the long-standing cohort-year ambiguity: confirmed the Dec/Feb/May rounds belong to Cohort 2027-2029, which opens in Studielink 1 Oct 2026</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; deadline year-labeling on official page is internally inconsistent (Dec/Feb/May dates vs. an Oct 2026 Studielink-opening note) — verify manually before relying on exact cohort year</t>
+          <t>Seed entry Aug 2026; the prior caveat about internally inconsistent cohort-year labeling is now resolved — a direct fetch of the admissions page (26 Sep 2026) confirms the Dec 2026 / Feb 2027 / May 2027 rounds are the Cohort 2027-2029 rounds and that Studielink opens 1 Oct 2026, so the two sets of dates are consistent after all</t>
         </is>
       </c>
     </row>
@@ -1009,12 +1009,12 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>~15 January (recurring annual pattern; 2026-27 cycle deadline was 15 Jan 2026 — 2027-28 date TBA)</t>
+          <t>15 January 2027, 14:00 CET — confirmed for the 2027-28 cycle via direct fetch of the official apply page; the call for applications opens early November 2026 (applications not yet open as of 26 Sep 2026)</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>later</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -1049,17 +1049,17 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>2027-28 cycle deadline now confirmed as 15 Jan 2027 14:00 CET (was TBA); call opens early Nov 2026 — urgency raised from later to soon</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; watch for 2027-28 deadline announcement</t>
+          <t>Seed entry Aug 2026; the 2027-28 deadline that was pending announcement is now confirmed (15 Jan 2027, 14:00 CET), so this entry no longer needs watching for a date. IELTS/TOEFL, references and application fee are still not stated on the pages checked.</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Closed for 2026-27 entry; ~January annual deadline pattern — register for 2027-28 notification</t>
+          <t>2027-28 entry cycle has now opened — most Oxford graduate courses opened to applications on 16 Sep 2026. Deadline is the course's January deadline (the most recent round's funding deadline was 27 January); the exact 2027-28 date was not confirmed this pass because ox.ac.uk returned HTTP 403 to direct fetches — verify on the course page</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>1,100+ full/partial graduate scholarships for 2026-27, merit-based. Automatic consideration for most scholarships if course offer received by January deadline.</t>
+          <t>Over 1,200 full/partial graduate scholarships expected across all courses for 2027-28 entry (up from the 1,100+ figure published for 2026-27), merit-based. Automatic consideration for most Oxford scholarships — assessed against eligibility criteria without a separate application — if a course offer is received by the January deadline.</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1811,17 +1811,17 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>2027-28 entry cycle has opened (courses opened 16 Sep 2026); scholarship count updated to the 1,200+ figure published for 2027-28</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; watch for 2027-28 cycle opening</t>
+          <t>Seed entry Aug 2026; the 2027-28 cycle opening that this entry was watching for has now happened. ox.ac.uk blocked automated fetches (HTTP 403) this pass, so the exact 2027-28 January deadline is inferred from the published pattern (most recent round: 27 Jan) rather than directly confirmed — spot-check the course page before relying on it.</t>
         </is>
       </c>
     </row>
@@ -2025,12 +2025,12 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Both the 42nd-cycle (2026-27) ordinary call and the special FIS-funded call (deadline was 18 May 2026) have now closed; the 43rd cycle (2027-28) has not yet been announced as of 23 Aug 2026 — recurring annual pattern (ordinary call ~October, FIS-funded call ~spring), check back autumn/winter 2026</t>
+          <t>43rd cycle (a.y. 2027-28) is now announced: the Call for Applications opens 3 November 2026 (confirmed via direct fetch of the official PhD admissions page). The submission deadline for that call has not yet been published — expected to follow Bocconi's usual pattern of a winter/early-spring closing. The 42nd-cycle (2026-27) ordinary call and FIS-funded call (18 May 2026) are both closed.</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -2065,17 +2065,17 @@
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>Confirmed 2026-27 cycle (ordinary + FIS call) is fully closed and 2027-28 cycle not yet announced; added test-requirement and application-fee detail</t>
+          <t>43rd cycle (2027-28) is now announced — call opens 3 Nov 2026; urgency moved from closed to later now that a next cycle exists</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; watch for 43rd-cycle (2027-28) announcement in autumn/winter 2026</t>
+          <t>Seed entry Aug 2026; the 43rd-cycle announcement this entry was waiting on has arrived (call opens 3 Nov 2026), so it is no longer a dead cycle. The closing date for that call is still unpublished — re-check once the call actually opens in November.</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2152,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>~20 Oct – 13 Jan recurring window (dates shown were for Oct 2026 entry, already closed) — next application window expected to open ~Oct 2026 for Oct 2027 entry</t>
+          <t>Corrected this pass: the most recent confirmed cycle (Sept/Oct 2026 entry) closed 23 January 2026 at 17:00 UK time, with late applications considered up to 27 March 2026 — so the recurring pattern is a ~late-January deadline, not the '13 Jan' previously recorded. A separate 2027/28-entry course page exists but UCL returned HTTP 403 to every direct fetch this pass, so the exact 2027 entry deadline is not yet confirmed — expect ~late Jan 2027.</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -2192,17 +2192,17 @@
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Corrected the deadline pattern — the confirmed recent-cycle deadline was 23 Jan 2026 17:00 (late applications to 27 Mar 2026), replacing the previously recorded '~20 Oct – 13 Jan' window</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026</t>
+          <t>Seed entry Aug 2026; the previously recorded '~20 Oct – 13 Jan' application window did not match UCL's published dates for this course and has been corrected to the confirmed late-January pattern. ucl.ac.uk blocks automated fetches (HTTP 403) on both the current and 2027-entry course pages, so the 2027 date is inferred, not confirmed — manual browser check recommended.</t>
         </is>
       </c>
     </row>
@@ -3606,7 +3606,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3621,139 +3621,139 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>National University of Singapore (NUS)</t>
+          <t>Central European University (CEU)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>#120</t>
+          <t>#268</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Vienna</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
+          <t>https://www.ceu.edu/academics/degrees/phd-economics</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>7.0 overall; waived for applicants whose Bachelor's and/or Master's was taught exclusively in English</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>100 iBT overall; same English-medium-degree waiver as IELTS</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Not mentioned on this page</t>
+          <t>Required for most applicants; waived for CEU Master of Arts in Economics, Data and Policy students applying to the program</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Non-English-medium graduates may need to take a Graduate English Course; good undergraduate honours degree (first class or high 2:1 equivalent) or Master's, in economics or another quantitative subject</t>
+          <t>Master's degree or equivalent in economics or a related field with GPA 3.33+; solid foundations in micro, macro and econometrics; research proposal of max 500 words; part of the Vienna Economics Graduate Center (VEGC), a cooperation between CEU, University of Vienna and WU Vienna</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Not stated on the program page (CEU's academic year conventionally begins in late September)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Early: 30 September 2026 (now within 30 days — imminent); Main: 1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
+          <t>15 January 2027 — the current application round's closing date, confirmed via direct fetch of the official program page</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>3 letters of recommendation from professors</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not stated on the pages checked (an application fee payment is referenced as required, but no amount is published)</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Not detailed (fully funded — see funding)</t>
+          <t>Not published as a figure; tuition is fully covered for students on the CEU Doctoral Scholarship</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Yes — all admitted students</t>
+          <t>Yes — full tuition plus stipend for the standard 4 years</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
+          <t>Full tuition coverage plus stipend support for the standard 48-month duration. The doctoral stipend is EUR 2,002 gross/month, awarded for 48 months. Applicants who apply by the financial-aid deadline are automatically considered for the CEU Doctoral Scholarship — no separate scholarship application is needed. Field research grants are available in year two, plus doctoral research and travel funds. Note that PhD stipends are taxable in Austria and are treated as self-employed income, so they must be declared to the tax authorities.</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>Early-round deadline (30 Sep 2026) is now within 30 days — urgency upgraded from soon to urgent, 30-day reminder flag set</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics</t>
+          <t>New find Sep 2026; distinct from EUR-17 (Vienna Graduate School of Economics, University of Vienna / WU Vienna) even though CEU's Economics PhD sits inside the same Vienna Economics Graduate Center cooperation — CEU is a separate degree-awarding institution with its own admissions round and its own scholarship. Funding is unusually clean for Europe: full tuition plus a stated monthly stipend figure for the full 48 months, awarded automatically from the admissions round rather than via a separate competition. The gross-vs-net distinction matters here because the stipend is taxable in Austria. Start date and application fee are still unconfirmed.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MPhil/PhD</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Hong Kong University of Science and Technology (HKUST)</t>
+          <t>National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>#287</t>
+          <t>#120</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3763,47 +3763,47 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
+          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>6.5 overall, no subscore below 5.5 (university-wide standard; waived if English-medium/first-language English)</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>iBT 80 / pBT 550 / Revised PBT 60 (university-wide standard)</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Required ("satisfactory score")</t>
+          <t>Not mentioned on this page</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Conditional offers require official documents by end of July</t>
+          <t>Non-English-medium graduates may need to take a Graduate English Course; good undergraduate honours degree (first class or high 2:1 equivalent) or Master's, in economics or another quantitative subject</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Fall semester</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
+          <t>For the August 2027 intake: the FASS graduate-research application window runs 1 May 2026 – 15 December 2026, and the Department of Economics deadline within that window is 1 December 2026. The '30 September 2026 early round' previously recorded here could NOT be re-substantiated on this pass by any source and appears to have been recorded in error — treat 1 Dec 2026 as the operative deadline.</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -3818,22 +3818,22 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>HK$180, non-refundable</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>HK$47,000/year (2026/27 rate, full-time or part-time)</t>
+          <t>Not detailed (fully funded — see funding)</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — all admitted students</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>Postgraduate Studentship (PGS): HK$229,620/year (2025/26 rate); recipients serve as Graduate Teaching Assistants. HKUST RedBird PhD Award stacks with HKPFS: Recruitment Award HK$40,000 (year 1) + Academic Excellence Award HK$20,000/year (later years). Conference &amp; Travel Allowance ~HK$14,200/year for HKPFS holders. Also cross-reference Hong Kong PhD Fellowship Scheme (ASA-03).</t>
+          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
@@ -3843,44 +3843,44 @@
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr), fees, and IELTS/TOEFL standards; upgraded funding_status from Likely to Yes</t>
+          <t>CORRECTION: the 30 Sep 2026 'early round' deadline could not be re-substantiated and appears to have been recorded in error — operative deadline is 1 Dec 2026; urgency stepped back from urgent to soon and reminder flags reset</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026</t>
+          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics. CORRECTION LOG: the 2026-09-14 pass recorded an 'Early: 30 September 2026' deadline and issued a 30-day Telegram reminder against it. On 2026-09-26 that early round could not be found in any source; two independent search corroborations instead give a single FASS application window of 1 May – 15 Dec 2026 for the Aug 2027 intake, with 1 Dec 2026 as the Economics department deadline. The NUS FASS pages (both the ECS programme page and the faculty application-process page) return empty bodies to automated fetches, so this rests on search corroboration rather than a direct fetch — a manual browser check is recommended to close it out definitively.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PhD (Fellowship, cross-university)</t>
+          <t>MPhil/PhD</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
+          <t>MPhil/PhD in Economics</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Varies by host university (scheme spans multiple HK institutions)</t>
+          <t>#287</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3900,37 +3900,37 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
+          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>6.5 overall, no subscore below 5.5 (university-wide standard; waived if English-medium/first-language English)</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>iBT 80 / pBT 550 / Revised PBT 60 (university-wide standard)</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>Required ("satisfactory score")</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
+          <t>Conditional offers require official documents by end of July</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Typically September (Fall)</t>
+          <t>Fall semester</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
+          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -3940,27 +3940,27 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$180, non-refundable</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Waived (see funding)</t>
+          <t>HK$47,000/year (2026/27 rate, full-time or part-time)</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>Yes — major fellowship</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
+          <t>Postgraduate Studentship (PGS): HK$229,620/year (2025/26 rate); recipients serve as Graduate Teaching Assistants. HKUST RedBird PhD Award stacks with HKPFS: Recruitment Award HK$40,000 (year 1) + Academic Excellence Award HK$20,000/year (later years). Conference &amp; Travel Allowance ~HK$14,200/year for HKPFS holders. Also cross-reference Hong Kong PhD Fellowship Scheme (ASA-03).</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
@@ -3970,44 +3970,44 @@
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr), fees, and IELTS/TOEFL standards; upgraded funding_status from Likely to Yes</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
+          <t>Seed entry Aug 2026</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>ASA-03</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>PhD (Fellowship, cross-university)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Nanyang Technological University (NTU Singapore)</t>
+          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>#253</t>
+          <t>Varies by host university (scheme spans multiple HK institutions)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -4017,47 +4017,47 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
+          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>7.0 minimum (preferred)</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>105 minimum</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Not mandatory, but scores considered if submitted; recommended for applicants without a degree from an autonomous university</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders; 2 referee reports required</t>
+          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Two intakes/year: August (main) and January</t>
+          <t>Typically September (Fall)</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>August intake: applications open 1 Oct-15 Nov (results Mar-May); January intake: applications open 1 Jun-31 Jul (results Nov-Dec) — recurring annual pattern, confirmed via direct official fetch</t>
+          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -4067,27 +4067,27 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>2 (referee reports)</t>
+          <t>Not specified in scheme rules</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>S$50</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>Not specified (MOE-subsidised place)</t>
+          <t>Waived (see funding)</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — major fellowship</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>MOE-subsidised programme; funded via Nanyang President's Graduate Scholarship or Nanyang Research Scholarship, which carries Graduate Assistantship Programme (GAP) teaching/research duties.</t>
+          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
@@ -4097,24 +4097,24 @@
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>Confirmed application windows, referee/fee requirements via direct official fetch; urgency upgraded from tba to soon</t>
+          <t>Added (seed)</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; tuition fee figure still not found</t>
+          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4124,17 +4124,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD)</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>University of Tokyo</t>
+          <t>Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>#110</t>
+          <t>#253</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -4144,77 +4144,77 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Tokyo</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
+          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>7.0 minimum (preferred)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>105 minimum</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not mandatory, but scores considered if submitted; recommended for applicants without a degree from an autonomous university</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>English-taught international program; site (gaia.e.u-tokyo.ac.jp) unreachable for a fifth consecutive pass — DNS resolution failure confirmed again via independent fetch attempts. As of April 2023, UTIPE PhD applicants are generally required to first complete UTIPE's own Master's program and be admitted to candidacy; direct external PhD entry is closed except for applicants with 2+ years of research experience at a university/research institute abroad (following 16 years of foreign schooling), who may be recognized as equivalent to a Master's holder and apply directly. Corroborated via search snippets quoting the official admission/FAQ pages, not a direct primary-source fetch. New this pass (via search only): since the 2025 enrollment cycle the Department of Economics reportedly merged the general Master's program and the previous UTIPE program, now admitting into a single Master's program twice a year — suggests the standalone "UTIPE Master's" entry point may itself have changed; unconfirmed by primary source.</t>
+          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders; 2 referee reports required</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Two intakes/year: August (main) and January</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Not yet confirmed — needs manual check</t>
+          <t>August intake: applications open 1 Oct-15 Nov (results Mar-May); January intake: applications open 1 Jun-31 Jul (results Nov-Dec) — recurring annual pattern, confirmed via direct official fetch</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>2 (referee reports)</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>S$50</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not specified (MOE-subsidised place)</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
+          <t>MOE-subsidised programme; funded via Nanyang President's Graduate Scholarship or Nanyang Research Scholarship, which carries Graduate Assistantship Programme (GAP) teaching/research duties.</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
@@ -4224,24 +4224,24 @@
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>Site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025</t>
+          <t>Confirmed application windows, referee/fee requirements via direct official fetch; urgency upgraded from tba to soon</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>INCOMPLETE — the official site has now failed to resolve on five consecutive passes; a manual browser check is recommended rather than further automated retries. The 2023 admission-policy restriction is corroborated by multiple search snippets quoting the official pages, but still not confirmed via a direct primary-source fetch.</t>
+          <t>Seed entry Aug 2026; tuition fee figure still not found</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4251,17 +4251,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD)</t>
+          <t>International Program in Economics (PhD)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Hitotsubashi University</t>
+          <t>University of Tokyo</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>#390 (confirmed still outside global top 300)</t>
+          <t>#110</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -4276,72 +4276,72 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Tokyo (Kunitachi)</t>
+          <t>Tokyo</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://www.econ.hit-u.ac.jp/eng/page/graduate/admission.html</t>
+          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Not stated (page mentions TOEFL/TOEIC only)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>TOEFL or TOEIC score required as part of application materials; specific minimum score not stated</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Two intakes/year (Spring and Autumn); international applicants without a Hitotsubashi Master's apply via an AO exam route — either general AO (2+ years work experience post-master's) or AO for international applicants with a Master's from outside Japan; admission mainly via submitted documents, interview may follow (online option for overseas applicants)</t>
+          <t>English-taught international program; site (gaia.e.u-tokyo.ac.jp) unreachable for a fifth consecutive pass — DNS resolution failure confirmed again via independent fetch attempts. As of April 2023, UTIPE PhD applicants are generally required to first complete UTIPE's own Master's program and be admitted to candidacy; direct external PhD entry is closed except for applicants with 2+ years of research experience at a university/research institute abroad (following 16 years of foreign schooling), who may be recognized as equivalent to a Master's holder and apply directly. Corroborated via search snippets quoting the official admission/FAQ pages, not a direct primary-source fetch. New this pass (via search only): since the 2025 enrollment cycle the Department of Economics reportedly merged the general Master's program and the previous UTIPE program, now admitting into a single Master's program twice a year — suggests the standalone "UTIPE Master's" entry point may itself have changed; unconfirmed by primary source.</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Spring or Autumn intake (two cycles/year)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Spring intake: document submission window ~14-17 Oct annually (confirmed for the Spring 2026 cohort: 14-17 Oct 2025, results ~11 Nov 2025), so the next window is expected ~mid-Oct 2026 for Spring 2027 entry. Autumn intake: opens ~April, exact window not confirmed this pass.</t>
+          <t>Not yet confirmed — needs manual check</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>tba</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>At least 1 recommendation letter required (AO exam route requires an English-language Letter of Recommendation); exact number for other routes not specified</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>~JPY 30,000 reported (university-wide general graduate-school figure, not confirmed Economics-specific)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>~JPY 535,800/year reported (university-wide figure, not confirmed Economics-PhD-specific)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible)</t>
+          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>MEXT scholarship route confirmed to exist, administered via a separate central international-office page (requires embassy/consulate preliminary candidacy). No department-specific stipend/assistantship figures found.</t>
+          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
@@ -4351,24 +4351,24 @@
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>Spring-intake submission window (expected ~14-17 Oct 2026) is now within 30 days — urgency upgraded from soon to urgent, 30-day reminder flag set</t>
+          <t>Site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>Partially complete — fee figures are university-wide, not Economics-PhD-confirmed; the 14-17 Oct 2026 window is an estimate based on the recurring annual pattern (confirmed dates were for the Spring 2026 cohort), not yet directly reconfirmed for this cycle — recommend a manual spot-check closer to the date</t>
+          <t>INCOMPLETE — the official site has now failed to resolve on five consecutive passes; a manual browser check is recommended rather than further automated retries. The 2023 admission-policy restriction is corroborated by multiple search snippets quoting the official pages, but still not confirmed via a direct primary-source fetch.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4378,17 +4378,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD)</t>
+          <t>Graduate School of Economics (PhD)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Seoul National University (SNU)</t>
+          <t>Hitotsubashi University</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>#189</t>
+          <t>#390 (confirmed still outside global top 300)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -4398,77 +4398,77 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Seoul</t>
+          <t>Tokyo (Kunitachi)</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://en.snu.ac.kr/admission</t>
+          <t>https://www.econ.hit-u.ac.jp/eng/page/graduate/admission.html</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>6.0 minimum (university-wide standard)</t>
+          <t>Not stated (page mentions TOEFL/TOEIC only)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>iBT 80, or TEPS 551 (university-wide standard, alternative to IELTS)</t>
+          <t>TOEFL or TOEIC score required as part of application materials; specific minimum score not stated</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Not required (no GRE requirement found in central admissions materials)</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
+          <t>Two intakes/year (Spring and Autumn); international applicants without a Hitotsubashi Master's apply via an AO exam route — either general AO (2+ years work experience post-master's) or AO for international applicants with a Master's from outside Japan; admission mainly via submitted documents, interview may follow (online option for overseas applicants)</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Spring or Autumn intake (two cycles/year)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>University-wide pattern: Fall-intake applications open ~early March (2026 Fall: 3-5 Mar); Spring-intake applications open ~early July (2027 Spring: 6-9 Jul) — both 2026 cycles already closed; 2027 Fall cycle not yet announced. Department-specific PhD deadline still not separately confirmed.</t>
+          <t>Spring intake: document submission window ~14-17 Oct annually (confirmed for the Spring 2026 cohort: 14-17 Oct 2025, results ~11 Nov 2025), so the next window is expected ~mid-Oct 2026 for Spring 2027 entry. Autumn intake: opens ~April, exact window not confirmed this pass.</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>later</t>
+          <t>urgent</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>At least 1 recommendation letter required (AO exam route requires an English-language Letter of Recommendation); exact number for other routes not specified</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>KRW 90,000 (no fee waivers offered)</t>
+          <t>~JPY 30,000 reported (university-wide general graduate-school figure, not confirmed Economics-specific)</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>~JPY 535,800/year reported (university-wide figure, not confirmed Economics-PhD-specific)</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Likely (university-wide scholarships only)</t>
+          <t>Likely (MEXT scholarship-eligible)</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Confirmed via direct fetch of the Department of Economics' own PhD page: no department-specific funding scheme exists — funding runs entirely through the university-wide scholarships above.</t>
+          <t>MEXT scholarship route confirmed to exist, administered via a separate central international-office page (requires embassy/consulate preliminary candidacy). No department-specific stipend/assistantship figures found.</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
@@ -4478,24 +4478,24 @@
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; admissions and funding run entirely through the university-wide portal and scholarships</t>
+          <t>Spring-intake submission window (expected ~14-17 Oct 2026) is now within 30 days — urgency upgraded from soon to urgent, 30-day reminder flag set</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>Confirmed (Aug 2026) that Economics PhD funding at SNU is university-wide only, with no departmental top-up scheme; department page exists but defers entirely to the central international-admissions portal for deadlines/fees</t>
+          <t>Partially complete — fee figures are university-wide, not Economics-PhD-confirmed; the 14-17 Oct 2026 window is an estimate based on the recurring annual pattern (confirmed dates were for the Spring 2026 cohort), not yet directly reconfirmed for this cycle — recommend a manual spot-check closer to the date</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ASA-08</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4505,17 +4505,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PhD in Business (Economics track)</t>
+          <t>Department of Economics (PhD)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>University of Hong Kong (Faculty of Business and Economics)</t>
+          <t>Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>#106</t>
+          <t>#189</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -4525,104 +4525,104 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Seoul</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://phd.hkubs.hku.hk/admissions/admission-application-and-tuition-fee</t>
+          <t>https://en.snu.ac.kr/admission</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Academic overall 6.5, all subtests &gt;= 6.0 (waived if prior degree was taught in English)</t>
+          <t>6.0 minimum (university-wide standard)</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>iBT &gt;= 85</t>
+          <t>iBT 80, or TEPS 551 (university-wide standard, alternative to IELTS)</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>GRE or GMAT required, score &lt;5 years old (institution codes: GRE 2482, GMAT FS2-WL-48)</t>
+          <t>Not required (no GRE requirement found in central admissions materials)</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Bachelor's with first-class honours (or equivalent), or Bachelor's + Master's from a recognized university; 3-year track with a research Master's, 4-year track without one; Economics is one of six FBE PhD fields</t>
+          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Fall semester, normally September (matriculates once a year)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Applications open 1 September; Main Round closes 1 December (recurring annual cycle; late applications considered only if places remain)</t>
+          <t>University-wide pattern: Fall-intake applications open ~early March (2026 Fall: 3-5 Mar); Spring-intake applications open ~early July (2027 Spring: 6-9 Jul) — both 2026 cycles already closed; 2027 Fall cycle not yet announced. Department-specific PhD deadline still not separately confirmed.</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>2 (academic referee reports, submitted directly by referees)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>HK$600 (paid online via HKU Graduate School application system)</t>
+          <t>KRW 90,000 (no fee waivers offered)</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>HK$49,500/year (2027-28 rate) for full-time PhD — typically waived/covered for scholarship holders</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Likely (university-wide scholarships only)</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>Standard Postgraduate Scholarship (PGS) pays HK$19,135/month (rising to HK$19,655/month once candidature is confirmed), available to essentially all admitted PhD students regardless of HKPFS status. HKPFS awardees instead receive HK$28,700/month plus HK$14,400/year travel allowance for up to 3 years.</t>
+          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Confirmed via direct fetch of the Department of Economics' own PhD page: no department-specific funding scheme exists — funding runs entirely through the university-wide scholarships above.</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; admissions and funding run entirely through the university-wide portal and scholarships</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>Distinct from the cross-institution HKPFS scheme already tracked (ASA-03) — nearly all admitted PhD students get baseline PGS funding here even without winning HKPFS, a broader guarantee than HKPFS alone.</t>
+          <t>Confirmed (Aug 2026) that Economics PhD funding at SNU is university-wide only, with no departmental top-up scheme; department page exists but defers entirely to the central international-admissions portal for deadlines/fees</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4632,17 +4632,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD in Business (Economics track)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>#369 — confirmed via direct fetch of the live RePEc table</t>
+          <t>#106</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4662,37 +4662,37 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://admission.econ.cuhk.edu.hk/pg/phd-economics/</t>
+          <t>https://phd.hkubs.hku.hk/admissions/admission-application-and-tuition-fee</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Academic overall 6.5</t>
+          <t>Academic overall 6.5, all subtests &gt;= 6.0 (waived if prior degree was taught in English)</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>79 iBT (or 4.5-6.0 Home Edition) — see IELTS field for alternatives (GMAT Verbal &gt;=21, or a degree from an English-medium institution, also accepted)</t>
+          <t>iBT &gt;= 85</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Required (institution code 3153, department code 1801); no published hard cutoff, but absence of a score disadvantages applicants</t>
+          <t>GRE or GMAT required, score &lt;5 years old (institution codes: GRE 2482, GMAT FS2-WL-48)</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Master's in economics or a related field with a strong math/stats background expected; strong bachelor's-only applicants can also apply with sufficient research potential. Official transcripts, degree certificates, a 5-page research proposal and/or working papers, resume, and typically an interview all required</t>
+          <t>Bachelor's with first-class honours (or equivalent), or Bachelor's + Master's from a recognized university; 3-year track with a research Master's, 4-year track without one; Economics is one of six FBE PhD fields</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Fall intake (standard)</t>
+          <t>Fall semester, normally September (matriculates once a year)</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Applications open 1 Sept 2026; HKPFS-track deadline 1 Dec 2026 (11:59am); non-HKPFS deadline 1 Dec 2026 (11:59pm); referee letters due by 4 Dec 2026</t>
+          <t>Applications open 1 September; Main Round closes 1 December (recurring annual cycle; late applications considered only if places remain)</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -4702,54 +4702,54 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>3 confidential recommendation letters</t>
+          <t>2 (academic referee reports, submitted directly by referees)</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>HK$500 per programme</t>
+          <t>HK$600 (paid online via HKU Graduate School application system)</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>HK$47,000 (2026/27) / HK$49,500 (2027/28)</t>
+          <t>HK$49,500/year (2027-28 rate) for full-time PhD — typically waived/covered for scholarship holders</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>Yes — guaranteed assistantship for all admits</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>All successful full-time PhD admits receive a teaching/research assistantship with a monthly stipend of ~HK$19,100. HKPFS awardees additionally receive a full tuition waiver plus HK$40,000 (year 1) / HK$20,000/year (subsequent years) and housing benefits. Local students separately receive a government tuition waiver. Cross-reference the cross-institution HKPFS scheme already tracked (ASA-03).</t>
+          <t>Standard Postgraduate Scholarship (PGS) pays HK$19,135/month (rising to HK$19,655/month once candidature is confirmed), available to essentially all admitted PhD students regardless of HKPFS status. HKPFS awardees instead receive HK$28,700/month plus HK$14,400/year travel allowance for up to 3 years.</t>
         </is>
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>New find Aug 2026; distinct from HKU (ASA-08) and the cross-institution HKPFS scheme (ASA-03) — CUHK guarantees baseline assistantship funding to all admits independent of HKPFS.</t>
+          <t>Distinct from the cross-institution HKPFS scheme already tracked (ASA-03) — nearly all admitted PhD students get baseline PGS funding here even without winning HKPFS, a broader guarantee than HKPFS alone.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4764,62 +4764,62 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Australian National University (ANU)</t>
+          <t>Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>#124</t>
+          <t>#369 — confirmed via direct fetch of the live RePEc table</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Canberra</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
+          <t>https://admission.econ.cuhk.edu.hk/pg/phd-economics/</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>6.5 overall (no band below 6.0)</t>
+          <t>Academic overall 6.5</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>570 (paper-based; essay ≥4.5)</t>
+          <t>79 iBT (or 4.5-6.0 Home Edition) — see IELTS field for alternatives (GMAT Verbal &gt;=21, or a degree from an English-medium institution, also accepted)</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
+          <t>Required (institution code 3153, department code 1801); no published hard cutoff, but absence of a score disadvantages applicants</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
+          <t>Master's in economics or a related field with a strong math/stats background expected; strong bachelor's-only applicants can also apply with sufficient research potential. Official transcripts, degree certificates, a 5-page research proposal and/or working papers, resume, and typically an interview all required</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>February (Semester 1); Semester 2 entry possible (July)</t>
+          <t>Fall intake (standard)</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>For Feb 2027 start: international scholarship deadline (31 Aug 2026) has now closed; the standard/domestic deadline of 31 Oct 2026 is the next live deadline (confirmed via search corroboration, ANU site still returning HTTP 504 to direct fetch); Sem 2 entry deadline (31 Mar) also already closed for this cycle</t>
+          <t>Applications open 1 Sept 2026; HKPFS-track deadline 1 Dec 2026 (11:59am); non-HKPFS deadline 1 Dec 2026 (11:59pm); referee letters due by 4 Dec 2026</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -4829,32 +4829,32 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3 confidential recommendation letters</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$500 per programme</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$47,000 (2026/27) / HK$49,500 (2027/28)</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — guaranteed assistantship for all admits</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>Australian Government RTP Stipend: AUD $39,069/year (2026 full-time base rate, ANU-wide), paid fortnightly, up to 3.5 years. Some HDR supplementary scholarships add AUD $7,000/year on top, for up to 3 years. Domestic candidates pay no tuition (RTP-covered); international candidates can compete for HDR Fee Remission Merit Scholarships covering up to 4 years.</t>
+          <t>All successful full-time PhD admits receive a teaching/research assistantship with a monthly stipend of ~HK$19,100. HKPFS awardees additionally receive a full tuition waiver plus HK$40,000 (year 1) / HK$20,000/year (subsequent years) and housing benefits. Local students separately receive a government tuition waiver. Cross-reference the cross-institution HKPFS scheme already tracked (ASA-03).</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
@@ -4864,89 +4864,89 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline — reset reminder flags for the new date</t>
+          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026 — international-applicant deadline has closed; domestic deadline (31 Oct 2026) is next</t>
+          <t>New find Aug 2026; distinct from HKU (ASA-08) and the cross-institution HKPFS scheme (ASA-03) — CUHK guarantees baseline assistantship funding to all admits independent of HKPFS.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>ASA-10</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>MPhil/PhD</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>University of Melbourne</t>
+          <t>Singapore Management University (SMU), School of Economics</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>#151</t>
+          <t>#198</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Melbourne</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
+          <t>https://economics.smu.edu.sg/phd-economics</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
+          <t>Required if the medium of instruction at Bachelor's/Master's level was not English; no minimum score is published — SMU states each applicant is assessed on all credentials together. Results must be from within the last 2 years.</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>94 iBT (W27/S18/R13/L13)</t>
+          <t>Same policy as IELTS — required for non-English-medium degrees, no published minimum, valid within 2 years. SMU TOEFL institution code 9014.</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Not mentioned in entry requirements</t>
+          <t>GRE or GMAT required, but may be waived for SMU, NTU and NUS graduates; scores must be less than 5 years old at the proposed date of admission. SMU GRE code 2861; GMAT code for PhD Economics F8D-KD-38.</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
+          <t>Referees receive an auto-generated email to complete an online referee report once the application is submitted</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>March intake</t>
+          <t>August intake</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>March 2027 intake deadline reported as 30 November 2026 — found via search summary only; the official how-to-apply/key-dates pages returned HTTP 403 on every direct fetch attempt this pass, so this date is unconfirmed by primary source and should be manually verified</t>
+          <t>Applications run 1 August – 31 December each year (recurring annual window), so 31 December 2026 is the operative deadline for the August 2027 intake</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -4956,54 +4956,54 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>2 referee reports (submitted online by the referees)</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>SGD 15 (non-refundable)</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Not detailed — full tuition fee waiver reported (see funding)</t>
+          <t>Covered in full for scholarship holders — the scholarship pays registration and tuition fees; no separate self-funded figure located</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — full scholarship for outstanding candidates</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>Australian Government Research Training Program (RTP) funded places available: RTP stipend reported at AUD $39,500/year (2026 rate) plus full tuition fee waiver and AUD $15,000 research/conference travel funding for confirmed PhD candidates (unconfirmed by primary source — see deadline note). Program structure: 2-year Master of Commerce coursework + 3-year PhD.</t>
+          <t>Full scholarships covering registration and tuition fees plus a monthly stipend, awarded to outstanding candidates. Stipend rates (from 1 Jan 2024) are tiered by citizenship and rise after the qualifying examination: Singapore Citizens SGD 3,200/month before and SGD 3,700 after; Permanent Residents SGD 2,800 before and SGD 3,300 after; foreign students SGD 2,500 before and SGD 3,000 after. Renewable yearly subject to good academic performance for the first 4 years of candidature; beyond that, continued support is available via research or teaching assistantships or industry grants.</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>Found a reported deadline and funding figures via search, but could not confirm via direct page fetch (403 blocked) — flagged as lower confidence</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches this pass — recommend a manual browser check before relying on the reported 30 Nov 2026 deadline</t>
+          <t>New find Sep 2026; a well-regarded Singapore economics department not previously tracked, and a third Singapore option alongside NUS (ASA-01) and NTU (ASA-04). The stipend tiering by citizenship is worth noting for international applicants — the foreign-student rate (SGD 2,500 rising to SGD 3,000) is the relevant one and is materially below the Singapore-citizen rate. The SMU pages returned empty bodies to automated fetches, so the figures here rest on search corroboration of the official scholarship and admissions pages rather than a direct fetch; the RePEc rank (#198) was confirmed against the live August 2026 table.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5013,17 +5013,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PhD (Economics)</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Monash Business School</t>
+          <t>Australian National University (ANU)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>#46</t>
+          <t>#124</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -5038,42 +5038,42 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Melbourne (Clayton)</t>
+          <t>Canberra</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
+          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>7.0 minimum reported (third-party source, not confirmed on official Monash page — page returned HTTP 403 to direct fetch)</t>
+          <t>6.5 overall (no band below 6.0)</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>94 minimum reported (same caveat as IELTS — unconfirmed by primary source)</t>
+          <t>570 (paper-based; essay ≥4.5)</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
+          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>February (Semester 1); Semester 2 entry possible (July)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Integrated-pathway Feb/Semester-1 entry window (1 Jul-31 Aug) has closed; next integrated-pathway window (Jul/Semester-2 entry) opens ~1 Dec-1 Feb. Separately, general Graduate Research Scholarship rounds: international Round 3 (~31 Jul/31 Aug) has closed; domestic Round 4 closes 31 Oct 2026 (confirmed via search, monash.edu still blocking direct fetch with HTTP 403) — this is the next live deadline.</t>
+          <t>For Feb 2027 start: international scholarship deadline (31 Aug 2026) has now closed; the standard/domestic deadline of 31 Oct 2026 is the next live deadline (confirmed via search corroboration, ANU site still returning HTTP 504 to direct fetch); Sem 2 entry deadline (31 Mar) also already closed for this cycle</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -5083,19 +5083,19 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr">
+      <c r="S36" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>International ~AUD $38,900/yr, domestic ~AUD $37,100/yr reported (third-party aggregator source, not confirmed by official Monash page)</t>
-        </is>
-      </c>
       <c r="T36" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -5103,7 +5103,7 @@
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places — general RTP stipend reported at AUD $37,145/yr (2026 rate) plus a $1,500 relocation allowance (not confirmed Economics-specific).</t>
+          <t>Australian Government RTP Stipend: AUD $39,069/year (2026 full-time base rate, ANU-wide), paid fortnightly, up to 3.5 years. Some HDR supplementary scholarships add AUD $7,000/year on top, for up to 3 years. Domestic candidates pay no tuition (RTP-covered); international candidates can compete for HDR Fee Remission Merit Scholarships covering up to 4 years.</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
@@ -5118,19 +5118,19 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>Confirmed the ~31 Aug 2026 integrated-pathway and international-round deadlines have closed; domestic Graduate Research Scholarship Round 4 (31 Oct 2026) is the next live deadline — reset reminder flags for the new date</t>
+          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline — reset reminder flags for the new date</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; monash.edu has blocked all automated fetches on every pass so far (scholarships-and-fees, apply, and program pages all 403'd) — every figure in this entry is lower-confidence (search snippets/third-party aggregator only) and needs a manual browser check</t>
+          <t>Seed entry Aug 2026 — international-applicant deadline has closed; domestic deadline (31 Oct 2026) is next</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -5140,17 +5140,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>Doctoral Program in Economics</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>University of Sydney</t>
+          <t>University of Melbourne</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>#87</t>
+          <t>#151</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -5165,62 +5165,62 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Sydney</t>
+          <t>Melbourne</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://www.sydney.edu.au/scholarships/</t>
+          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>94 iBT (W27/S18/R13/L13)</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
+          <t>Not mentioned in entry requirements</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>March intake</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>March 2027 intake deadline reported as 30 November 2026 — found via search summary only; the official how-to-apply/key-dates pages returned HTTP 403 on every direct fetch attempt this pass, so this date is unconfirmed by primary source and should be manually verified</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>soon</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
           <t>Not mentioned</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP. Material finding: Sydney has no dedicated 'PhD in Economics' program page — the Economics coursework handbook explicitly states it "does not include a research component and thus does not provide a pathway to higher degree by research (e.g. PhD) studies." PhD study is pursued via the general Doctor of Philosophy degree with a nominated Economics supervisor/discipline, not a single named landing page.</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>Not specified on this page</t>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>Research Period 1 &amp; 2 deadline (11 September 2026) has now passed; Research Period 3 &amp; 4 — deadline 18 December 2026 — is the next live RTP scholarship round (reconfirmed via search, not a directly-fetched dedicated Economics PhD page).</t>
-        </is>
-      </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>soon</t>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>1 (for named scholarship example; general program may differ)</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not detailed — full tuition fee waiver reported (see funding)</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly; a 2027-rate RTP stipend of AUD $44,293/yr was also reported via search aggregators this pass (unconfirmed by primary source).</t>
+          <t>Australian Government Research Training Program (RTP) funded places available: RTP stipend reported at AUD $39,500/year (2026 rate) plus full tuition fee waiver and AUD $15,000 research/conference travel funding for confirmed PhD candidates (unconfirmed by primary source — see deadline note). Program structure: 2-year Master of Commerce coursework + 3-year PhD.</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
@@ -5240,24 +5240,24 @@
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down from urgent to soon, reminder flags reset for the new deadline</t>
+          <t>Found a reported deadline and funding figures via search, but could not confirm via direct page fetch (403 blocked) — flagged as lower confidence</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check; no dedicated Economics-specific PhD admissions page exists at Sydney</t>
+          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches this pass — recommend a manual browser check before relying on the reported 30 Nov 2026 deadline</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>AUS-05</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -5267,17 +5267,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD (Economics)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>UNSW Sydney</t>
+          <t>Monash Business School</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>#80</t>
+          <t>#46</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -5292,47 +5292,47 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Sydney</t>
+          <t>Melbourne (Clayton)</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://www.unsw.edu.au/business/study-with-us/postgraduate-research/phd-degrees/doctor-philosophy-phd-economics</t>
+          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Not listed on this page (exemptions for AU/CA/UK/US/NZ citizens); non-English-speaking-country applicants need IELTS/TOEFL/PTE/Cambridge or the UNSW Global English Course</t>
+          <t>7.0 minimum reported (third-party source, not confirmed on official Monash page — page returned HTTP 403 to direct fetch)</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Not listed on this page — see IELTS field for alternatives</t>
+          <t>94 minimum reported (same caveat as IELTS — unconfirmed by primary source)</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Optional but recommended overall; one source indicates GRE may be specifically required for the Economics stream — this conflicts with the general 'optional' language elsewhere and needs manual confirmation</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course. Program begins with a 1-year Master of Pre-Doctoral Business Studies, followed by 3-3.5 years of doctoral research; direct entry to the 3-year PhD is possible for candidates with first-class Honours/Master's plus independent funding (Stream 2).</t>
+          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Term 1 – February</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Confirmed still closed as of 23 Aug 2026 (verified directly on program page): EOI window opened 20 March 2026, closed 15 August 2026, no newer/next EOI window posted. Note: a separate 26 August 2026 formal-application deadline exists, but it applies only to candidates already invited to apply from the closed EOI round, not to new applicants.</t>
+          <t>Integrated-pathway Feb/Semester-1 entry window (1 Jul-31 Aug) has closed; next integrated-pathway window (Jul/Semester-2 entry) opens ~1 Dec-1 Feb. Separately, general Graduate Research Scholarship rounds: international Round 3 (~31 Jul/31 Aug) has closed; domestic Round 4 closes 31 Oct 2026 (confirmed via search, monash.edu still blocking direct fetch with HTTP 403) — this is the next live deadline.</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -5347,17 +5347,17 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>Not detailed (fully funded — see funding)</t>
+          <t>International ~AUD $38,900/yr, domestic ~AUD $37,100/yr reported (third-party aggregator source, not confirmed by official Monash page)</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>Yes — all admitted students</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>Full tuition waiver + stipend AUD 35,000-45,000/yr, up to 4.5 years (+1 optional fellowship year), plus substantial research/conference travel funding.</t>
+          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places — general RTP stipend reported at AUD $37,145/yr (2026 rate) plus a $1,500 relocation allowance (not confirmed Economics-specific).</t>
         </is>
       </c>
       <c r="V38" t="inlineStr">
@@ -5367,144 +5367,398 @@
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>Confirmed EOI window remains closed with no new window announced; added program structure and English-test details</t>
+          <t>Confirmed the ~31 Aug 2026 integrated-pathway and international-round deadlines have closed; domestic Graduate Research Scholarship Round 4 (31 Oct 2026) is the next live deadline — reset reminder flags for the new date</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026 — EOI window closed 15 Aug 2026, still no next window announced as of this update</t>
+          <t>Seed entry Aug 2026; monash.edu has blocked all automated fetches on every pass so far (scholarships-and-fees, apply, and program pages all 403'd) — every figure in this entry is lower-confidence (search snippets/third-party aggregator only) and needs a manual browser check</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>AUS-04</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>PhD in Economics</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>University of Sydney</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>#87</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://www.sydney.edu.au/scholarships/</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Not specified at general program level</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Not specified at general program level</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Not mentioned</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP. Material finding: Sydney has no dedicated 'PhD in Economics' program page — the Economics coursework handbook explicitly states it "does not include a research component and thus does not provide a pathway to higher degree by research (e.g. PhD) studies." PhD study is pursued via the general Doctor of Philosophy degree with a nominated Economics supervisor/discipline, not a single named landing page.</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Not specified on this page</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Research Period 1 &amp; 2 deadline (11 September 2026) has now passed; Research Period 3 &amp; 4 — deadline 18 December 2026 — is the next live RTP scholarship round (reconfirmed via search, not a directly-fetched dedicated Economics PhD page).</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>soon</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>1 (for named scholarship example; general program may differ)</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly; a 2027-rate RTP stipend of AUD $44,293/yr was also reported via search aggregators this pass (unconfirmed by primary source).</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down from urgent to soon, reminder flags reset for the new deadline</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check; no dedicated Economics-specific PhD admissions page exists at Sydney</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>AUS-05</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>PhD in Economics</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>UNSW Sydney</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>#80</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://www.unsw.edu.au/business/study-with-us/postgraduate-research/phd-degrees/doctor-philosophy-phd-economics</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Not listed on this page (exemptions for AU/CA/UK/US/NZ citizens); non-English-speaking-country applicants need IELTS/TOEFL/PTE/Cambridge or the UNSW Global English Course</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Not listed on this page — see IELTS field for alternatives</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Optional but recommended overall; one source indicates GRE may be specifically required for the Economics stream — this conflicts with the general 'optional' language elsewhere and needs manual confirmation</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course. Program begins with a 1-year Master of Pre-Doctoral Business Studies, followed by 3-3.5 years of doctoral research; direct entry to the 3-year PhD is possible for candidates with first-class Honours/Master's plus independent funding (Stream 2).</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Term 1 – February</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Confirmed still closed as of 23 Aug 2026 (verified directly on program page): EOI window opened 20 March 2026, closed 15 August 2026, no newer/next EOI window posted. Note: a separate 26 August 2026 formal-application deadline exists, but it applies only to candidates already invited to apply from the closed EOI round, not to new applicants.</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Not detailed (fully funded — see funding)</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Yes — all admitted students</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Full tuition waiver + stipend AUD 35,000-45,000/yr, up to 4.5 years (+1 optional fellowship year), plus substantial research/conference travel funding.</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>Confirmed EOI window remains closed with no new window announced; added program structure and English-test details</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026 — EOI window closed 15 Aug 2026, still no next window announced as of this update</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>AUS-06</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>Doctor of Philosophy (Economics)</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>University of Queensland (School of Economics)</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>#71</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>Brisbane</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>https://economics.uq.edu.au/study/phd</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>Academic overall 6.5, with 6.0 minimum in each of reading/writing/speaking/listening</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>Not specified on the economics-specific page (UQ university-wide PhD pages generally accept TOEFL iBT as an alternative to IELTS)</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>Not confirmed as required; application package can include GRE/GMAT score sheets, suggesting optional/supplementary rather than mandatory</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="M41" t="inlineStr">
         <is>
           <t>Academic CV, transcripts; MPhil/research master's options also available; can join a funded project with scholarship support as an alternative entry route</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
+      <c r="N41" t="inlineStr">
         <is>
           <t>Quarterly intakes (research quarters begin 1 Jan, 1 Apr, 1 Jul, 1 Oct); applications for RHD programs can be submitted any time</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr">
+      <c r="O41" t="inlineStr">
         <is>
           <t>Domestic Round 1 (31 Aug 2026) has now closed; the International round deadline of 19 Oct 2026 is confirmed still live via search corroboration and is the next relevant deadline for upcoming 2027 research quarters.</t>
         </is>
       </c>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>soon</t>
-        </is>
-      </c>
-      <c r="Q39" t="inlineStr">
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>urgent</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
         <is>
           <t>Minimum 2 referee reports</t>
         </is>
       </c>
-      <c r="R39" t="inlineStr">
+      <c r="R41" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="S39" t="inlineStr">
+      <c r="S41" t="inlineStr">
         <is>
           <t>Not specified (international RTP scholarship recipients typically get a full tuition fee offset)</t>
         </is>
       </c>
-      <c r="T39" t="inlineStr">
+      <c r="T41" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr">
+      <c r="U41" t="inlineStr">
         <is>
           <t>RTP/UQGRSS provides a tax-free living stipend of AUD $39,220/year (2026 rate, indexed annually — updated from a previously-recorded AUD $37,500 figure) plus, for eligible international candidates, a tuition fee offset; no separate application needed beyond the program EOI.</t>
         </is>
       </c>
-      <c r="V39" t="inlineStr">
+      <c r="V41" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="W39" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="X39" t="inlineStr">
-        <is>
-          <t>International round deadline (19 Oct 2026) is now within 30 days — 30-day reminder flag set</t>
-        </is>
-      </c>
-      <c r="Y39" t="inlineStr">
-        <is>
-          <t>Scholarship is university-wide (RTP/UQGRSS), not economics-specific, but School of Economics PhD candidates are eligible.</t>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>International round deadline (19 Oct 2026) is now 23 days out, inside the ~4-week threshold — urgency upgraded from soon to urgent</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>Scholarship is university-wide (RTP/UQGRSS), not economics-specific, but School of Economics PhD candidates are eligible. The 30-day reminder flag was already set on the 2026-09-19 pass, so no new reminder is due — only the urgency classification changed.</t>
         </is>
       </c>
     </row>
@@ -5519,7 +5773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5559,98 +5813,98 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>EUR-23</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PhD in Economics (Quantitative Economics track) — Goethe University Frankfurt (GSEFM)</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>New find: RePEc #81, up to three competitive first-year IMFS stipends plus post-qualifying-exam TA/RA positions; no tuition fees.</t>
+          <t>Correction: the '30 September 2026 early round' deadline recorded on 14 Sep could not be re-substantiated by any source this pass and appears to have been recorded in error. Two independent corroborations give a single FASS window of 1 May - 15 Dec 2026 for the Aug 2027 intake, with 1 Dec 2026 as the Economics department deadline. Urgency stepped back from urgent to soon and the 30-day reminder flag has been reset. Apologies for the earlier reminder against a date we can no longer confirm.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>30-day reminder: the Spring-intake submission window (expected ~14-17 Oct 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
+          <t>The long-standing cohort-year ambiguity is resolved: the Dec/Feb/May rounds are confirmed to be the Cohort 2027-2029 rounds, with Studielink opening 1 Oct 2026 and Round 1 closing 1 Dec 2026, then 1 Feb 2027, 1 May 2027, and rolling admissions to 15 Jun 2027.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>EUR-03</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>30-day reminder: the international round deadline (19 Oct 2026) is now within 30 days.</t>
+          <t>The 2027-28 deadline that was previously TBA is now confirmed as 15 January 2027 at 14:00 CET, with the call for applications opening in early November 2026. Urgency raised from later to soon.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>EUR-09</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>MPhil + DPhil in Economics — University of Oxford</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -5660,51 +5914,51 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>The 11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down to soon, reminder flags reset.</t>
+          <t>The 2027-28 entry cycle has opened — most Oxford graduate courses opened to applications on 16 Sep 2026. Scholarship provision updated to the 1,200+ full/partial graduate scholarships expected for 2027-28, up from the 1,100+ figure for 2026-27. Deadline remains the January pattern (most recent round closed 27 Jan).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>30-day reminder: the early-round deadline (30 Sep 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
+          <t>The 43rd cycle (a.y. 2027-28) is now announced: the Call for Applications opens 3 November 2026. Urgency moved from closed to later now that a next cycle exists; the closing date for that call is not yet published.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-12</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -5714,186 +5968,186 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Official site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025.</t>
+          <t>Corrected the deadline pattern: the previously recorded '~20 Oct - 13 Jan' window did not match UCL's published dates. The confirmed recent-cycle deadline was 23 January 2026 at 17:00 UK time, with late applications considered to 27 March 2026, so the pattern is a late-January deadline and ~late Jan 2027 is expected for 2027 entry.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EUR-22</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Cambridge</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>New find: RePEc #50, ~66% of Cambridge doctoral students fully funded via Cambridge Trust/Gates Cambridge/College/ESRC funding; funding-competition deadline 8 Dec 2026.</t>
+          <t>The international round deadline (19 Oct 2026) is now 23 days away, inside the ~4-week threshold, so urgency has been upgraded from soon to urgent. The 30-day reminder already went out on 19 Sep, so no new reminder is due.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>EUR-24</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD in Economics — Central European University (CEU)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline, urgency moved from urgent to soon.</t>
+          <t>New find: RePEc #268, Vienna. Full tuition coverage plus a EUR 2,002 gross/month doctoral stipend for the full 48 months, awarded automatically from the admissions round rather than a separate competition. Current round closes 15 January 2027. Note the stipend is taxable in Austria.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-10</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>PhD in Economics — Singapore Management University (SMU), School of Economics</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Confirmed the integrated-pathway and international scholarship round deadlines have closed; now tracking the domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026), urgency moved from urgent to soon.</t>
+          <t>New find: RePEc #198, Singapore. Full scholarship covering registration and tuition plus a monthly stipend — foreign students SGD 2,500/month rising to SGD 3,000 after the qualifying exam — renewable for the first 4 years. Applications run 1 Aug - 31 Dec annually, so 31 Dec 2026 for the Aug 2027 intake.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>EUR-23</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>PhD in Economics (Quantitative Economics track) — Goethe University Frankfurt (GSEFM)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>7-day reminder: the 11 Sep 2026 Research Period 1 &amp; 2 deadline is confirmed still live and now imminent.</t>
+          <t>New find: RePEc #81, up to three competitive first-year IMFS stipends plus post-qualifying-exam TA/RA positions; no tuition fees.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026), urgency moved from urgent to soon.</t>
+          <t>30-day reminder: the Spring-intake submission window (expected ~14-17 Oct 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EUR-17</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#192) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>30-day reminder: the international round deadline (19 Oct 2026) is now within 30 days.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EUR-18</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -5903,51 +6157,51 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#24) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>The 11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down to soon, reminder flags reset.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>EUR-19</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#40) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>30-day reminder: the early-round deadline (30 Sep 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EUR-20</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -5957,34 +6211,34 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#164) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>Official site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>EUR-22</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>PhD in Economics — University of Cambridge</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>New find: RePEc #50, ~66% of Cambridge doctoral students fully funded via Cambridge Trust/Gates Cambridge/College/ESRC funding; funding-competition deadline 8 Dec 2026.</t>
         </is>
       </c>
     </row>
@@ -5996,12 +6250,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -6011,7 +6265,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Official site remains unreachable (DNS failure, fourth consecutive pass); recommend a manual browser check rather than further automated retries.</t>
+          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline, urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -6023,174 +6277,174 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>EUR-21</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>PhD in Economics — Sciences Po</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>New find: RePEc #42, funded via a 3-year Doctoral Contract (~EUR 2,100/month) plus tuition exemption; some applicants expected to already hold external funding.</t>
+          <t>Confirmed the integrated-pathway and international scholarship round deadlines have closed; now tracking the domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026), urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>EUR-17</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>New find: FWF-grant-funded PhD positions at the University of Vienna; admission-round dates inconsistent across sources, recommend a manual spot-check.</t>
+          <t>7-day reminder: the 11 Sep 2026 Research Period 1 &amp; 2 deadline is confirmed still live and now imminent.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>EUR-18</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>New find: PhD structured as a salaried employment contract (~EUR 2,750-3,500/month); official site blocked automated fetches, several fields search-only.</t>
+          <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026), urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>EUR-19</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>New find: RePEc ~#40, funded PhD positions up to 4 years plus IRO Doctoral Scholarships for developing-country students; deadlines are vacancy-by-vacancy.</t>
+          <t>Confirmed RePEc rank (#192) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EUR-20</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
+          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>New find: joint Berlin-area doctoral school, funded via a EUR 1,650/month qualification-phase stipend then dissertation-phase employment.</t>
+          <t>Confirmed RePEc rank (#24) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>New find: guaranteed teaching/research assistantship (~HK$19,100/month) for all admits, independent of the HKPFS scheme already tracked (ASA-03).</t>
+          <t>Confirmed RePEc rank (#40) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -6200,24 +6454,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Confirmed application windows (Aug intake: 1 Oct-15 Nov; Jan intake: 1 Jun-31 Jul), referee/fee requirements, and Graduate Assistantship Programme detail via direct official fetch; urgency upgraded from tba to soon.</t>
+          <t>Confirmed RePEc rank (#164) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -6227,24 +6481,24 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Corroborated via search snippets (site unreachable for a third consecutive pass) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad.</t>
+          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -6254,34 +6508,34 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration; urgency upgraded from tba to soon.</t>
+          <t>Official site remains unreachable (DNS failure, fourth consecutive pass); recommend a manual browser check rather than further automated retries.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>EUR-21</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD in Economics — Sciences Po</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; funding runs entirely through university-wide scholarships.</t>
+          <t>New find: RePEc #42, funded via a 3-year Doctoral Contract (~EUR 2,100/month) plus tuition exemption; some applicants expected to already hold external funding.</t>
         </is>
       </c>
     </row>
@@ -6293,22 +6547,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>7-day reminder: the 31 Aug 2026 international scholarship deadline is confirmed still live via search corroboration (ANU site returned HTTP 504 to direct fetch).</t>
+          <t>New find: FWF-grant-funded PhD positions at the University of Vienna; admission-round dates inconsistent across sources, recommend a manual spot-check.</t>
         </is>
       </c>
     </row>
@@ -6320,22 +6574,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>7-day reminder: the imminent ~31 Aug 2026 integrated-pathway deadline is reconfirmed via search (monash.edu still blocking direct fetch); added a general RTP stipend figure (AUD $37,145/yr).</t>
+          <t>New find: PhD structured as a salaried employment contract (~EUR 2,750-3,500/month); official site blocked automated fetches, several fields search-only.</t>
         </is>
       </c>
     </row>
@@ -6347,93 +6601,93 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>7-day reminder: confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to AUD $39,220/yr (2026 rate).</t>
+          <t>New find: RePEc ~#40, funded PhD positions up to 4 years plus IRO Doctoral Scholarships for developing-country students; deadlines are vacancy-by-vacancy.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
+          <t>New find: joint Berlin-area doctoral school, funded via a EUR 1,650/month qualification-phase stipend then dissertation-phase employment.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
+          <t>New find: guaranteed teaching/research assistantship (~HK$19,100/month) for all admits, independent of the HKPFS scheme already tracked (ASA-03).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -6443,24 +6697,24 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
+          <t>Confirmed application windows (Aug intake: 1 Oct-15 Nov; Jan intake: 1 Jun-31 Jul), referee/fee requirements, and Graduate Assistantship Programme detail via direct official fetch; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -6470,24 +6724,24 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
+          <t>Corroborated via search snippets (site unreachable for a third consecutive pass) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -6497,24 +6751,24 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
+          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -6524,88 +6778,88 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
+          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; funding runs entirely through university-wide scholarships.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
+          <t>7-day reminder: the 31 Aug 2026 international scholarship deadline is confirmed still live via search corroboration (ANU site returned HTTP 504 to direct fetch).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
+          <t>7-day reminder: the imminent ~31 Aug 2026 integrated-pathway deadline is reconfirmed via search (monash.edu still blocking direct fetch); added a general RTP stipend figure (AUD $37,145/yr).</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
+          <t>7-day reminder: confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to AUD $39,220/yr (2026 rate).</t>
         </is>
       </c>
     </row>
@@ -6617,12 +6871,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -6632,7 +6886,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
+          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
         </is>
       </c>
     </row>
@@ -6644,12 +6898,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -6659,7 +6913,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
+          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
         </is>
       </c>
     </row>
@@ -6671,12 +6925,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -6686,7 +6940,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
+          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
         </is>
       </c>
     </row>
@@ -6698,12 +6952,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -6713,7 +6967,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
+          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
         </is>
       </c>
     </row>
@@ -6725,12 +6979,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>AUS-05</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PhD in Economics — UNSW Sydney</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -6740,7 +6994,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
+          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
         </is>
       </c>
     </row>
@@ -6752,22 +7006,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>EUR-13</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
         </is>
       </c>
     </row>
@@ -6779,22 +7033,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>EUR-14</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
+          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
         </is>
       </c>
     </row>
@@ -6806,22 +7060,22 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EUR-15</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
+          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
         </is>
       </c>
     </row>
@@ -6833,22 +7087,22 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>EUR-16</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
+          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
         </is>
       </c>
     </row>
@@ -6860,22 +7114,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ASA-08</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
+          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -6887,265 +7141,265 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
+          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>EUR-03</t>
+          <t>AUS-05</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
+          <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>EUR-04</t>
+          <t>EUR-13</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
+          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EUR-05</t>
+          <t>EUR-14</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>PhD in Economics — CEMFI</t>
+          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EUR-06</t>
+          <t>EUR-15</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
+          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>EUR-07</t>
+          <t>EUR-16</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>PhD Program — Paris School of Economics (PSE)</t>
+          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>EUR-08</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — Stockholm University / IIES</t>
+          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>EUR-09</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>MPhil + DPhil in Economics — University of Oxford</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
         </is>
       </c>
     </row>
@@ -7157,12 +7411,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -7184,12 +7438,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -7211,12 +7465,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EUR-12</t>
+          <t>EUR-03</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
+          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -7238,12 +7492,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-04</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -7265,12 +7519,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>EUR-05</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>PhD in Economics — CEMFI</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -7292,12 +7546,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>EUR-06</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -7319,12 +7573,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-07</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>PhD Program — Paris School of Economics (PSE)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -7346,12 +7600,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-08</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD Programme in Economics — Stockholm University / IIES</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -7373,12 +7627,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-09</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>MPhil + DPhil in Economics — University of Oxford</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -7400,12 +7654,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -7427,12 +7681,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -7454,12 +7708,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>EUR-12</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -7481,12 +7735,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -7508,12 +7762,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -7535,20 +7789,263 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
+          <t>ASA-03</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ASA-04</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>ASA-05</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>ASA-06</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>ASA-07</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>AUS-01</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>PhD in Economics — Australian National University (ANU)</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>AUS-02</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>AUS-03</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>PhD (Economics) — Monash Business School</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>AUS-04</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>PhD in Economics — University of Sydney</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
           <t>AUS-05</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D84" t="inlineStr">
         <is>
           <t>Added (seed)</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="E84" t="inlineStr">
         <is>
           <t>Initial research pass — program added to tracker.</t>
         </is>

</xml_diff>

<commit_message>
Econ ledger update 2026-10-03: 1 added, 4 updated, 2 reminder flags
</commit_message>
<xml_diff>
--- a/apps/EconGradAlert/data/tracker.xlsx
+++ b/apps/EconGradAlert/data/tracker.xlsx
@@ -438,7 +438,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last full research pass: 2026-09-26</t>
+          <t>Last full research pass: 2026-10-03</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Program count: 40</t>
+          <t>Program count: 41</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y41"/>
+  <dimension ref="A1:Y42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2787,7 +2787,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Two admission rounds reported — roughly 1 Dec-15 Feb and 1 Mar-30 Apr on one page, vs. a single 1 Feb-15 Jun window on the VGSE-specific page; exact current-cycle dates are inconsistent across the university's own sources, recommend a manual spot-check</t>
+          <t>Two admission rounds, confirmed via direct fetch of the official VGSE site on 2026-10-03: Round 1, 1 Dec – 31 Jan; Round 2, 1 Mar – 30 Apr (recurring annual). This supersedes the previously-reported inconsistency across other university pages — vgse.at is the authoritative source for this entry.</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -2827,17 +2827,17 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#192) via direct fetch of the live table, removing the prior unverified caveat</t>
+          <t>Resolved the previously-flagged admission-round date inconsistency via direct fetch of vgse.at: Round 1 1 Dec–31 Jan, Round 2 1 Mar–30 Apr</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>New find Aug 2026; admission-round dates are inconsistent across the university's own pages — verify the current-cycle deadline directly before relying on it; stipend amount unconfirmed.</t>
+          <t>New find Aug 2026; stipend amount via FWF grant still unconfirmed. Admission-round date inconsistency (flagged since Sept 2026) resolved 2026-10-03 via direct fetch of the authoritative vgse.at page.</t>
         </is>
       </c>
     </row>
@@ -3733,7 +3733,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-25</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3743,144 +3743,144 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>Rome Economics Doctorate (RED)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>National University of Singapore (NUS)</t>
+          <t>Einaudi Institute for Economics and Finance (EIEF), in partnership with Luiss, Sapienza University of Rome, and Tor Vergata University of Rome</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>#120</t>
+          <t>#152 (Istituto Einaudi per l'Economia e la Finanza (EIEF), RePEc top-level institutions)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Rome</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
+          <t>https://www.redphd.it/</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Not mentioned on this page</t>
+          <t>GRE General Test required</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Non-English-medium graduates may need to take a Graduate English Course; good undergraduate honours degree (first class or high 2:1 equivalent) or Master's, in economics or another quantitative subject</t>
+          <t>MSc degree in Economics or equivalent required before enrollment; offers are made sequentially, pending formal admission from one of the three partner universities (confirmed May/June).</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Not specified on pages checked (program enrollment tied to partner-university admission decisions)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>For the August 2027 intake: the FASS graduate-research application window runs 1 May 2026 – 15 December 2026, and the Department of Economics deadline within that window is 1 December 2026. The '30 September 2026 early round' previously recorded here could NOT be re-substantiated on this pass by any source and appears to have been recorded in error — treat 1 Dec 2026 as the operative deadline.</t>
+          <t>15 January (recurring annual pattern, confirmed via direct fetch of redphd.it) — the a.y. 2026/27 call closed 15 Jan 2026 and the site now shows that round as CLOSED; the call for the 2027/28 cycle is expected to open on a similar annual cycle, likely around late 2026</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
+          <t>At least 2, from professors who have closely followed the applicant's studies</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Not detailed (fully funded — see funding)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Yes — all admitted students</t>
+          <t>Fully funded — tuition waiver + stipend</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
+          <t>Four-year scholarship (plus a possible one-year extension for promising students): tuition waiver and a stipend reported as EUR 16,243 gross/year for students on a university scholarship and EUR 22,171.88 gross/year for international candidates, plus research-trip funding and a grant increment for visiting periods at a partner international university. These figures come from a secondary aggregator (wemakescholars.com), not yet directly confirmed on redphd.it — verify before relying on them.</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>CORRECTION: the 30 Sep 2026 'early round' deadline could not be re-substantiated and appears to have been recorded in error — operative deadline is 1 Dec 2026; urgency stepped back from urgent to soon and reminder flags reset</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics. CORRECTION LOG: the 2026-09-14 pass recorded an 'Early: 30 September 2026' deadline and issued a 30-day Telegram reminder against it. On 2026-09-26 that early round could not be found in any source; two independent search corroborations instead give a single FASS application window of 1 May – 15 Dec 2026 for the Aug 2027 intake, with 1 Dec 2026 as the Economics department deadline. The NUS FASS pages (both the ECS programme page and the faculty application-process page) return empty bodies to automated fetches, so this rests on search corroboration rather than a direct fetch — a manual browser check is recommended to close it out definitively.</t>
+          <t>New find Oct 2026 — the 'Rome Economics Doctorate', a joint PhD program across EIEF (a Bank of Italy-funded research institute) and three Rome universities (Luiss, Sapienza, Tor Vergata). Funding appears genuine and well-documented, but exact current-cycle stipend figures, program duration, and start date were not confirmed directly on the official site this pass — verify before relying on specifics. Official site shows the 2026/27 cycle as CLOSED (deadline was 15 Jan 2026); treat the 15 Jan recurrence as a pattern, not a confirmed 2027/28 date.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MPhil/PhD</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Hong Kong University of Science and Technology (HKUST)</t>
+          <t>National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>#287</t>
+          <t>#120</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3890,47 +3890,47 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
+          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>6.5 overall, no subscore below 5.5 (university-wide standard; waived if English-medium/first-language English)</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>iBT 80 / pBT 550 / Revised PBT 60 (university-wide standard)</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Required ("satisfactory score")</t>
+          <t>Not mentioned on this page</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Conditional offers require official documents by end of July</t>
+          <t>Non-English-medium graduates may need to take a Graduate English Course; good undergraduate honours degree (first class or high 2:1 equivalent) or Master's, in economics or another quantitative subject</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Fall semester</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
+          <t>For the August 2027 intake: the FASS graduate-research application window runs 1 May 2026 – 15 December 2026, and the Department of Economics deadline within that window is 1 December 2026. The '30 September 2026 early round' previously recorded here could NOT be re-substantiated on this pass by any source and appears to have been recorded in error — treat 1 Dec 2026 as the operative deadline.</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -3945,22 +3945,22 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>HK$180, non-refundable</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>HK$47,000/year (2026/27 rate, full-time or part-time)</t>
+          <t>Not detailed (fully funded — see funding)</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — all admitted students</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>Postgraduate Studentship (PGS): HK$229,620/year (2025/26 rate); recipients serve as Graduate Teaching Assistants. HKUST RedBird PhD Award stacks with HKPFS: Recruitment Award HK$40,000 (year 1) + Academic Excellence Award HK$20,000/year (later years). Conference &amp; Travel Allowance ~HK$14,200/year for HKPFS holders. Also cross-reference Hong Kong PhD Fellowship Scheme (ASA-03).</t>
+          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
@@ -3970,44 +3970,44 @@
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr), fees, and IELTS/TOEFL standards; upgraded funding_status from Likely to Yes</t>
+          <t>CORRECTION: the 30 Sep 2026 'early round' deadline could not be re-substantiated and appears to have been recorded in error — operative deadline is 1 Dec 2026; urgency stepped back from urgent to soon and reminder flags reset</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026</t>
+          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics. CORRECTION LOG: the 2026-09-14 pass recorded an 'Early: 30 September 2026' deadline and issued a 30-day Telegram reminder against it. On 2026-09-26 that early round could not be found in any source; two independent search corroborations instead give a single FASS application window of 1 May – 15 Dec 2026 for the Aug 2027 intake, with 1 Dec 2026 as the Economics department deadline. The NUS FASS pages (both the ECS programme page and the faculty application-process page) return empty bodies to automated fetches, so this rests on search corroboration rather than a direct fetch — a manual browser check is recommended to close it out definitively.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PhD (Fellowship, cross-university)</t>
+          <t>MPhil/PhD</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
+          <t>MPhil/PhD in Economics</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Varies by host university (scheme spans multiple HK institutions)</t>
+          <t>#287</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -4027,37 +4027,37 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
+          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>6.5 overall, no subscore below 5.5 (university-wide standard; waived if English-medium/first-language English)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>iBT 80 / pBT 550 / Revised PBT 60 (university-wide standard)</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>Required ("satisfactory score")</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
+          <t>Conditional offers require official documents by end of July</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Typically September (Fall)</t>
+          <t>Fall semester</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
+          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -4067,27 +4067,27 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$180, non-refundable</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>Waived (see funding)</t>
+          <t>HK$47,000/year (2026/27 rate, full-time or part-time)</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Yes — major fellowship</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
+          <t>Postgraduate Studentship (PGS): HK$229,620/year (2025/26 rate); recipients serve as Graduate Teaching Assistants. HKUST RedBird PhD Award stacks with HKPFS: Recruitment Award HK$40,000 (year 1) + Academic Excellence Award HK$20,000/year (later years). Conference &amp; Travel Allowance ~HK$14,200/year for HKPFS holders. Also cross-reference Hong Kong PhD Fellowship Scheme (ASA-03).</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
@@ -4097,44 +4097,44 @@
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr), fees, and IELTS/TOEFL standards; upgraded funding_status from Likely to Yes</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
+          <t>Seed entry Aug 2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>ASA-03</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>PhD (Fellowship, cross-university)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Nanyang Technological University (NTU Singapore)</t>
+          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>#253</t>
+          <t>Varies by host university (scheme spans multiple HK institutions)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -4144,47 +4144,47 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
+          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>7.0 minimum (preferred)</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>105 minimum</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Not mandatory, but scores considered if submitted; recommended for applicants without a degree from an autonomous university</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders; 2 referee reports required</t>
+          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Two intakes/year: August (main) and January</t>
+          <t>Typically September (Fall)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>August intake: applications open 1 Oct-15 Nov (results Mar-May); January intake: applications open 1 Jun-31 Jul (results Nov-Dec) — recurring annual pattern, confirmed via direct official fetch</t>
+          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -4194,27 +4194,27 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2 (referee reports)</t>
+          <t>Not specified in scheme rules</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>S$50</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Not specified (MOE-subsidised place)</t>
+          <t>Waived (see funding)</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — major fellowship</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>MOE-subsidised programme; funded via Nanyang President's Graduate Scholarship or Nanyang Research Scholarship, which carries Graduate Assistantship Programme (GAP) teaching/research duties.</t>
+          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
@@ -4224,24 +4224,24 @@
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>Confirmed application windows, referee/fee requirements via direct official fetch; urgency upgraded from tba to soon</t>
+          <t>Added (seed)</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; tuition fee figure still not found</t>
+          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4251,17 +4251,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD)</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>University of Tokyo</t>
+          <t>Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>#110</t>
+          <t>#253</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -4271,77 +4271,77 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Tokyo</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
+          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>7.0 minimum (preferred)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>105 minimum</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not mandatory, but scores considered if submitted; recommended for applicants without a degree from an autonomous university</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>English-taught international program; site (gaia.e.u-tokyo.ac.jp) unreachable for a fifth consecutive pass — DNS resolution failure confirmed again via independent fetch attempts. As of April 2023, UTIPE PhD applicants are generally required to first complete UTIPE's own Master's program and be admitted to candidacy; direct external PhD entry is closed except for applicants with 2+ years of research experience at a university/research institute abroad (following 16 years of foreign schooling), who may be recognized as equivalent to a Master's holder and apply directly. Corroborated via search snippets quoting the official admission/FAQ pages, not a direct primary-source fetch. New this pass (via search only): since the 2025 enrollment cycle the Department of Economics reportedly merged the general Master's program and the previous UTIPE program, now admitting into a single Master's program twice a year — suggests the standalone "UTIPE Master's" entry point may itself have changed; unconfirmed by primary source.</t>
+          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders; 2 referee reports required</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Two intakes/year: August (main) and January</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Not yet confirmed — needs manual check</t>
+          <t>August intake: applications open 1 Oct-15 Nov (results Mar-May); January intake: applications open 1 Jun-31 Jul (results Nov-Dec) — recurring annual pattern, confirmed via direct official fetch</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>2 (referee reports)</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>S$50</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not specified (MOE-subsidised place)</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
+          <t>MOE-subsidised programme; funded via Nanyang President's Graduate Scholarship or Nanyang Research Scholarship, which carries Graduate Assistantship Programme (GAP) teaching/research duties.</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
@@ -4351,24 +4351,24 @@
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>Site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025</t>
+          <t>Confirmed application windows, referee/fee requirements via direct official fetch; urgency upgraded from tba to soon</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>INCOMPLETE — the official site has now failed to resolve on five consecutive passes; a manual browser check is recommended rather than further automated retries. The 2023 admission-policy restriction is corroborated by multiple search snippets quoting the official pages, but still not confirmed via a direct primary-source fetch.</t>
+          <t>Seed entry Aug 2026; tuition fee figure still not found</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4378,17 +4378,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD)</t>
+          <t>International Program in Economics (PhD)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Hitotsubashi University</t>
+          <t>University of Tokyo</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>#390 (confirmed still outside global top 300)</t>
+          <t>#110</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -4403,72 +4403,72 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Tokyo (Kunitachi)</t>
+          <t>Tokyo</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://www.econ.hit-u.ac.jp/eng/page/graduate/admission.html</t>
+          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Not stated (page mentions TOEFL/TOEIC only)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>TOEFL or TOEIC score required as part of application materials; specific minimum score not stated</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Two intakes/year (Spring and Autumn); international applicants without a Hitotsubashi Master's apply via an AO exam route — either general AO (2+ years work experience post-master's) or AO for international applicants with a Master's from outside Japan; admission mainly via submitted documents, interview may follow (online option for overseas applicants)</t>
+          <t>English-taught international program; site (gaia.e.u-tokyo.ac.jp) unreachable for a fifth consecutive pass — DNS resolution failure confirmed again via independent fetch attempts. As of April 2023, UTIPE PhD applicants are generally required to first complete UTIPE's own Master's program and be admitted to candidacy; direct external PhD entry is closed except for applicants with 2+ years of research experience at a university/research institute abroad (following 16 years of foreign schooling), who may be recognized as equivalent to a Master's holder and apply directly. Corroborated via search snippets quoting the official admission/FAQ pages, not a direct primary-source fetch. New this pass (via search only): since the 2025 enrollment cycle the Department of Economics reportedly merged the general Master's program and the previous UTIPE program, now admitting into a single Master's program twice a year — suggests the standalone "UTIPE Master's" entry point may itself have changed; unconfirmed by primary source.</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Spring or Autumn intake (two cycles/year)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Spring intake: document submission window ~14-17 Oct annually (confirmed for the Spring 2026 cohort: 14-17 Oct 2025, results ~11 Nov 2025), so the next window is expected ~mid-Oct 2026 for Spring 2027 entry. Autumn intake: opens ~April, exact window not confirmed this pass.</t>
+          <t>Not yet confirmed — needs manual check</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>tba</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>At least 1 recommendation letter required (AO exam route requires an English-language Letter of Recommendation); exact number for other routes not specified</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>~JPY 30,000 reported (university-wide general graduate-school figure, not confirmed Economics-specific)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>~JPY 535,800/year reported (university-wide figure, not confirmed Economics-PhD-specific)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible)</t>
+          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>MEXT scholarship route confirmed to exist, administered via a separate central international-office page (requires embassy/consulate preliminary candidacy). No department-specific stipend/assistantship figures found.</t>
+          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
@@ -4478,24 +4478,24 @@
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>Spring-intake submission window (expected ~14-17 Oct 2026) is now within 30 days — urgency upgraded from soon to urgent, 30-day reminder flag set</t>
+          <t>Site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>Partially complete — fee figures are university-wide, not Economics-PhD-confirmed; the 14-17 Oct 2026 window is an estimate based on the recurring annual pattern (confirmed dates were for the Spring 2026 cohort), not yet directly reconfirmed for this cycle — recommend a manual spot-check closer to the date</t>
+          <t>INCOMPLETE — the official site has now failed to resolve on five consecutive passes; a manual browser check is recommended rather than further automated retries. The 2023 admission-policy restriction is corroborated by multiple search snippets quoting the official pages, but still not confirmed via a direct primary-source fetch.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4505,17 +4505,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD)</t>
+          <t>Graduate School of Economics (PhD)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Seoul National University (SNU)</t>
+          <t>Hitotsubashi University</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>#189</t>
+          <t>#390 (confirmed still outside global top 300)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -4525,77 +4525,77 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Seoul</t>
+          <t>Tokyo (Kunitachi)</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://en.snu.ac.kr/admission</t>
+          <t>https://www.econ.hit-u.ac.jp/eng/page/graduate/admission.html</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>6.0 minimum (university-wide standard)</t>
+          <t>Not stated (page mentions TOEFL/TOEIC only)</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>iBT 80, or TEPS 551 (university-wide standard, alternative to IELTS)</t>
+          <t>TOEFL or TOEIC score required as part of application materials; specific minimum score not stated</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Not required (no GRE requirement found in central admissions materials)</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
+          <t>Two intakes/year (Spring and Autumn); international applicants without a Hitotsubashi Master's apply via an AO exam route — either general AO (2+ years work experience post-master's) or AO for international applicants with a Master's from outside Japan; admission mainly via submitted documents, interview may follow (online option for overseas applicants)</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Spring or Autumn intake (two cycles/year)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>University-wide pattern: Fall-intake applications open ~early March (2026 Fall: 3-5 Mar); Spring-intake applications open ~early July (2027 Spring: 6-9 Jul) — both 2026 cycles already closed; 2027 Fall cycle not yet announced. Department-specific PhD deadline still not separately confirmed.</t>
+          <t>Spring intake: document submission window ~14-17 Oct annually (confirmed for the Spring 2026 cohort: 14-17 Oct 2025, results ~11 Nov 2025), so the next window is expected ~mid-Oct 2026 for Spring 2027 entry. Autumn intake: opens ~April, exact window not confirmed this pass.</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>later</t>
+          <t>urgent</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>At least 1 recommendation letter required (AO exam route requires an English-language Letter of Recommendation); exact number for other routes not specified</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>KRW 90,000 (no fee waivers offered)</t>
+          <t>~JPY 30,000 reported (university-wide general graduate-school figure, not confirmed Economics-specific)</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>~JPY 535,800/year reported (university-wide figure, not confirmed Economics-PhD-specific)</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>Likely (university-wide scholarships only)</t>
+          <t>Likely (MEXT scholarship-eligible)</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Confirmed via direct fetch of the Department of Economics' own PhD page: no department-specific funding scheme exists — funding runs entirely through the university-wide scholarships above.</t>
+          <t>MEXT scholarship route confirmed to exist, administered via a separate central international-office page (requires embassy/consulate preliminary candidacy). No department-specific stipend/assistantship figures found.</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
@@ -4605,24 +4605,24 @@
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; admissions and funding run entirely through the university-wide portal and scholarships</t>
+          <t>Reconfirmation attempted again — official site unreachable (TLS certificate verification error, distinct from the earlier 403-blocked sites); search also could not pin down the exact 2026 window. Deadline estimate unchanged.</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>Confirmed (Aug 2026) that Economics PhD funding at SNU is university-wide only, with no departmental top-up scheme; department page exists but defers entirely to the central international-admissions portal for deadlines/fees</t>
+          <t>Partially complete — fee figures are university-wide, not Economics-PhD-confirmed; the 14-17 Oct 2026 window remains an estimate based on the recurring annual pattern (confirmed dates were for the Spring 2026 cohort). Direct fetch of econ.hit-u.ac.jp failed again on 2026-10-03 with a TLS cert error. This deadline is now very close (est. 11-14 days out) and notified_7day has not yet fired — if the next run still cannot reconfirm the exact date before that flag would trip, flag it for a manual check rather than letting an unverified date drive the 7-day Telegram alert.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ASA-08</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4632,17 +4632,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PhD in Business (Economics track)</t>
+          <t>Department of Economics (PhD)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>University of Hong Kong (Faculty of Business and Economics)</t>
+          <t>Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>#106</t>
+          <t>#189</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4652,104 +4652,104 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Seoul</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://phd.hkubs.hku.hk/admissions/admission-application-and-tuition-fee</t>
+          <t>https://en.snu.ac.kr/admission</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Academic overall 6.5, all subtests &gt;= 6.0 (waived if prior degree was taught in English)</t>
+          <t>6.0 minimum (university-wide standard)</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>iBT &gt;= 85</t>
+          <t>iBT 80, or TEPS 551 (university-wide standard, alternative to IELTS)</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>GRE or GMAT required, score &lt;5 years old (institution codes: GRE 2482, GMAT FS2-WL-48)</t>
+          <t>Not required (no GRE requirement found in central admissions materials)</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Bachelor's with first-class honours (or equivalent), or Bachelor's + Master's from a recognized university; 3-year track with a research Master's, 4-year track without one; Economics is one of six FBE PhD fields</t>
+          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Fall semester, normally September (matriculates once a year)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Applications open 1 September; Main Round closes 1 December (recurring annual cycle; late applications considered only if places remain)</t>
+          <t>University-wide pattern: Fall-intake applications open ~early March (2026 Fall: 3-5 Mar); Spring-intake applications open ~early July (2027 Spring: 6-9 Jul) — both 2026 cycles already closed; 2027 Fall cycle not yet announced. Department-specific PhD deadline still not separately confirmed.</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2 (academic referee reports, submitted directly by referees)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>HK$600 (paid online via HKU Graduate School application system)</t>
+          <t>KRW 90,000 (no fee waivers offered)</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>HK$49,500/year (2027-28 rate) for full-time PhD — typically waived/covered for scholarship holders</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Likely (university-wide scholarships only)</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>Standard Postgraduate Scholarship (PGS) pays HK$19,135/month (rising to HK$19,655/month once candidature is confirmed), available to essentially all admitted PhD students regardless of HKPFS status. HKPFS awardees instead receive HK$28,700/month plus HK$14,400/year travel allowance for up to 3 years.</t>
+          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Confirmed via direct fetch of the Department of Economics' own PhD page: no department-specific funding scheme exists — funding runs entirely through the university-wide scholarships above.</t>
         </is>
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; admissions and funding run entirely through the university-wide portal and scholarships</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>Distinct from the cross-institution HKPFS scheme already tracked (ASA-03) — nearly all admitted PhD students get baseline PGS funding here even without winning HKPFS, a broader guarantee than HKPFS alone.</t>
+          <t>Confirmed (Aug 2026) that Economics PhD funding at SNU is university-wide only, with no departmental top-up scheme; department page exists but defers entirely to the central international-admissions portal for deadlines/fees</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4759,17 +4759,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD in Business (Economics track)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>#369 — confirmed via direct fetch of the live RePEc table</t>
+          <t>#106</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4789,37 +4789,37 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://admission.econ.cuhk.edu.hk/pg/phd-economics/</t>
+          <t>https://phd.hkubs.hku.hk/admissions/admission-application-and-tuition-fee</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Academic overall 6.5</t>
+          <t>Academic overall 6.5, all subtests &gt;= 6.0 (waived if prior degree was taught in English)</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>79 iBT (or 4.5-6.0 Home Edition) — see IELTS field for alternatives (GMAT Verbal &gt;=21, or a degree from an English-medium institution, also accepted)</t>
+          <t>iBT &gt;= 85</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Required (institution code 3153, department code 1801); no published hard cutoff, but absence of a score disadvantages applicants</t>
+          <t>GRE or GMAT required, score &lt;5 years old (institution codes: GRE 2482, GMAT FS2-WL-48)</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Master's in economics or a related field with a strong math/stats background expected; strong bachelor's-only applicants can also apply with sufficient research potential. Official transcripts, degree certificates, a 5-page research proposal and/or working papers, resume, and typically an interview all required</t>
+          <t>Bachelor's with first-class honours (or equivalent), or Bachelor's + Master's from a recognized university; 3-year track with a research Master's, 4-year track without one; Economics is one of six FBE PhD fields</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Fall intake (standard)</t>
+          <t>Fall semester, normally September (matriculates once a year)</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Applications open 1 Sept 2026; HKPFS-track deadline 1 Dec 2026 (11:59am); non-HKPFS deadline 1 Dec 2026 (11:59pm); referee letters due by 4 Dec 2026</t>
+          <t>Applications open 1 September; Main Round closes 1 December (recurring annual cycle; late applications considered only if places remain)</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -4829,59 +4829,59 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>3 confidential recommendation letters</t>
+          <t>2 (academic referee reports, submitted directly by referees)</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>HK$500 per programme</t>
+          <t>HK$600 (paid online via HKU Graduate School application system)</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>HK$47,000 (2026/27) / HK$49,500 (2027/28)</t>
+          <t>HK$49,500/year (2027-28 rate) for full-time PhD — typically waived/covered for scholarship holders</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>Yes — guaranteed assistantship for all admits</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>All successful full-time PhD admits receive a teaching/research assistantship with a monthly stipend of ~HK$19,100. HKPFS awardees additionally receive a full tuition waiver plus HK$40,000 (year 1) / HK$20,000/year (subsequent years) and housing benefits. Local students separately receive a government tuition waiver. Cross-reference the cross-institution HKPFS scheme already tracked (ASA-03).</t>
+          <t>Standard Postgraduate Scholarship (PGS) pays HK$19,135/month (rising to HK$19,655/month once candidature is confirmed), available to essentially all admitted PhD students regardless of HKPFS status. HKPFS awardees instead receive HK$28,700/month plus HK$14,400/year travel allowance for up to 3 years.</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>New find Aug 2026; distinct from HKU (ASA-08) and the cross-institution HKPFS scheme (ASA-03) — CUHK guarantees baseline assistantship funding to all admits independent of HKPFS.</t>
+          <t>Distinct from the cross-institution HKPFS scheme already tracked (ASA-03) — nearly all admitted PhD students get baseline PGS funding here even without winning HKPFS, a broader guarantee than HKPFS alone.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ASA-10</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MPhil/PhD</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -4891,12 +4891,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Singapore Management University (SMU), School of Economics</t>
+          <t>Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>#198</t>
+          <t>#369 — confirmed via direct fetch of the live RePEc table</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4906,47 +4906,47 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://economics.smu.edu.sg/phd-economics</t>
+          <t>https://admission.econ.cuhk.edu.hk/pg/phd-economics/</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Required if the medium of instruction at Bachelor's/Master's level was not English; no minimum score is published — SMU states each applicant is assessed on all credentials together. Results must be from within the last 2 years.</t>
+          <t>Academic overall 6.5</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Same policy as IELTS — required for non-English-medium degrees, no published minimum, valid within 2 years. SMU TOEFL institution code 9014.</t>
+          <t>79 iBT (or 4.5-6.0 Home Edition) — see IELTS field for alternatives (GMAT Verbal &gt;=21, or a degree from an English-medium institution, also accepted)</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>GRE or GMAT required, but may be waived for SMU, NTU and NUS graduates; scores must be less than 5 years old at the proposed date of admission. SMU GRE code 2861; GMAT code for PhD Economics F8D-KD-38.</t>
+          <t>Required (institution code 3153, department code 1801); no published hard cutoff, but absence of a score disadvantages applicants</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Referees receive an auto-generated email to complete an online referee report once the application is submitted</t>
+          <t>Master's in economics or a related field with a strong math/stats background expected; strong bachelor's-only applicants can also apply with sufficient research potential. Official transcripts, degree certificates, a 5-page research proposal and/or working papers, resume, and typically an interview all required</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>August intake</t>
+          <t>Fall intake (standard)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Applications run 1 August – 31 December each year (recurring annual window), so 31 December 2026 is the operative deadline for the August 2027 intake</t>
+          <t>Applications open 1 Sept 2026; HKPFS-track deadline 1 Dec 2026 (11:59am); non-HKPFS deadline 1 Dec 2026 (11:59pm); referee letters due by 4 Dec 2026</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -4956,59 +4956,59 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2 referee reports (submitted online by the referees)</t>
+          <t>3 confidential recommendation letters</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>SGD 15 (non-refundable)</t>
+          <t>HK$500 per programme</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Covered in full for scholarship holders — the scholarship pays registration and tuition fees; no separate self-funded figure located</t>
+          <t>HK$47,000 (2026/27) / HK$49,500 (2027/28)</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>Yes — full scholarship for outstanding candidates</t>
+          <t>Yes — guaranteed assistantship for all admits</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>Full scholarships covering registration and tuition fees plus a monthly stipend, awarded to outstanding candidates. Stipend rates (from 1 Jan 2024) are tiered by citizenship and rise after the qualifying examination: Singapore Citizens SGD 3,200/month before and SGD 3,700 after; Permanent Residents SGD 2,800 before and SGD 3,300 after; foreign students SGD 2,500 before and SGD 3,000 after. Renewable yearly subject to good academic performance for the first 4 years of candidature; beyond that, continued support is available via research or teaching assistantships or industry grants.</t>
+          <t>All successful full-time PhD admits receive a teaching/research assistantship with a monthly stipend of ~HK$19,100. HKPFS awardees additionally receive a full tuition waiver plus HK$40,000 (year 1) / HK$20,000/year (subsequent years) and housing benefits. Local students separately receive a government tuition waiver. Cross-reference the cross-institution HKPFS scheme already tracked (ASA-03).</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>New find Sep 2026; a well-regarded Singapore economics department not previously tracked, and a third Singapore option alongside NUS (ASA-01) and NTU (ASA-04). The stipend tiering by citizenship is worth noting for international applicants — the foreign-student rate (SGD 2,500 rising to SGD 3,000) is the relevant one and is materially below the Singapore-citizen rate. The SMU pages returned empty bodies to automated fetches, so the figures here rest on search corroboration of the official scholarship and admissions pages rather than a direct fetch; the RePEc rank (#198) was confirmed against the live August 2026 table.</t>
+          <t>New find Aug 2026; distinct from HKU (ASA-08) and the cross-institution HKPFS scheme (ASA-03) — CUHK guarantees baseline assistantship funding to all admits independent of HKPFS.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-10</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>MPhil/PhD</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5018,62 +5018,62 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Australian National University (ANU)</t>
+          <t>Singapore Management University (SMU), School of Economics</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>#124</t>
+          <t>#198</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Canberra</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
+          <t>https://economics.smu.edu.sg/phd-economics</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>6.5 overall (no band below 6.0)</t>
+          <t>Required if the medium of instruction at Bachelor's/Master's level was not English; no minimum score is published — SMU states each applicant is assessed on all credentials together. Results must be from within the last 2 years.</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>570 (paper-based; essay ≥4.5)</t>
+          <t>Same policy as IELTS — required for non-English-medium degrees, no published minimum, valid within 2 years. SMU TOEFL institution code 9014.</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
+          <t>GRE or GMAT required, but may be waived for SMU, NTU and NUS graduates; scores must be less than 5 years old at the proposed date of admission. SMU GRE code 2861; GMAT code for PhD Economics F8D-KD-38.</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
+          <t>Referees receive an auto-generated email to complete an online referee report once the application is submitted</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>February (Semester 1); Semester 2 entry possible (July)</t>
+          <t>August intake</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>For Feb 2027 start: international scholarship deadline (31 Aug 2026) has now closed; the standard/domestic deadline of 31 Oct 2026 is the next live deadline (confirmed via search corroboration, ANU site still returning HTTP 504 to direct fetch); Sem 2 entry deadline (31 Mar) also already closed for this cycle</t>
+          <t>Applications run 1 August – 31 December each year (recurring annual window), so 31 December 2026 is the operative deadline for the August 2027 intake</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -5083,54 +5083,54 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2 referee reports (submitted online by the referees)</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>SGD 15 (non-refundable)</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Covered in full for scholarship holders — the scholarship pays registration and tuition fees; no separate self-funded figure located</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — full scholarship for outstanding candidates</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>Australian Government RTP Stipend: AUD $39,069/year (2026 full-time base rate, ANU-wide), paid fortnightly, up to 3.5 years. Some HDR supplementary scholarships add AUD $7,000/year on top, for up to 3 years. Domestic candidates pay no tuition (RTP-covered); international candidates can compete for HDR Fee Remission Merit Scholarships covering up to 4 years.</t>
+          <t>Full scholarships covering registration and tuition fees plus a monthly stipend, awarded to outstanding candidates. Stipend rates (from 1 Jan 2024) are tiered by citizenship and rise after the qualifying examination: Singapore Citizens SGD 3,200/month before and SGD 3,700 after; Permanent Residents SGD 2,800 before and SGD 3,300 after; foreign students SGD 2,500 before and SGD 3,000 after. Renewable yearly subject to good academic performance for the first 4 years of candidature; beyond that, continued support is available via research or teaching assistantships or industry grants.</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline — reset reminder flags for the new date</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026 — international-applicant deadline has closed; domestic deadline (31 Oct 2026) is next</t>
+          <t>New find Sep 2026; a well-regarded Singapore economics department not previously tracked, and a third Singapore option alongside NUS (ASA-01) and NTU (ASA-04). The stipend tiering by citizenship is worth noting for international applicants — the foreign-student rate (SGD 2,500 rising to SGD 3,000) is the relevant one and is materially below the Singapore-citizen rate. The SMU pages returned empty bodies to automated fetches, so the figures here rest on search corroboration of the official scholarship and admissions pages rather than a direct fetch; the RePEc rank (#198) was confirmed against the live August 2026 table.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -5140,17 +5140,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>University of Melbourne</t>
+          <t>Australian National University (ANU)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>#151</t>
+          <t>#124</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -5165,62 +5165,62 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Melbourne</t>
+          <t>Canberra</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
+          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
+          <t>6.5 overall (no band below 6.0)</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>94 iBT (W27/S18/R13/L13)</t>
+          <t>570 (paper-based; essay ≥4.5)</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Not mentioned in entry requirements</t>
+          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
+          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>March intake</t>
+          <t>February (Semester 1); Semester 2 entry possible (July)</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>March 2027 intake deadline reported as 30 November 2026 — found via search summary only; the official how-to-apply/key-dates pages returned HTTP 403 on every direct fetch attempt this pass, so this date is unconfirmed by primary source and should be manually verified</t>
+          <t>For Feb 2027 start: international scholarship deadline (31 Aug 2026) has now closed; the standard/domestic deadline of 31 Oct 2026 is the next live deadline (confirmed via search corroboration, ANU site still returning HTTP 504 to direct fetch); Sem 2 entry deadline (31 Mar) also already closed for this cycle</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>urgent</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Not detailed — full tuition fee waiver reported (see funding)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>Australian Government Research Training Program (RTP) funded places available: RTP stipend reported at AUD $39,500/year (2026 rate) plus full tuition fee waiver and AUD $15,000 research/conference travel funding for confirmed PhD candidates (unconfirmed by primary source — see deadline note). Program structure: 2-year Master of Commerce coursework + 3-year PhD.</t>
+          <t>Australian Government RTP Stipend: AUD $39,069/year (2026 full-time base rate, ANU-wide), paid fortnightly, up to 3.5 years. Some HDR supplementary scholarships add AUD $7,000/year on top, for up to 3 years. Domestic candidates pay no tuition (RTP-covered); international candidates can compete for HDR Fee Remission Merit Scholarships covering up to 4 years.</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
@@ -5240,24 +5240,24 @@
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>Found a reported deadline and funding figures via search, but could not confirm via direct page fetch (403 blocked) — flagged as lower confidence</t>
+          <t>Domestic deadline (31 Oct 2026) is now within 30 days (28 days out) — urgency upgraded from soon to urgent, 30-day reminder flag set</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches this pass — recommend a manual browser check before relying on the reported 30 Nov 2026 deadline</t>
+          <t>Seed entry Aug 2026 — international-applicant deadline has closed; domestic deadline (31 Oct 2026) is next. Note telegram_notified_30day/7day are already true from an earlier reset (pre-dating the Step 5 sync fix) — this run's 30-day flag flip follows the normal (non-reset) rule and does not touch the telegram_notified_* pair, so telegram_sync.py will not re-announce it; known gap, not new.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -5267,17 +5267,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PhD (Economics)</t>
+          <t>Doctoral Program in Economics</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Monash Business School</t>
+          <t>University of Melbourne</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>#46</t>
+          <t>#151</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -5292,42 +5292,42 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Melbourne (Clayton)</t>
+          <t>Melbourne</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
+          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>7.0 minimum reported (third-party source, not confirmed on official Monash page — page returned HTTP 403 to direct fetch)</t>
+          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>94 minimum reported (same caveat as IELTS — unconfirmed by primary source)</t>
+          <t>94 iBT (W27/S18/R13/L13)</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Not mentioned in entry requirements</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
+          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>March intake</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Integrated-pathway Feb/Semester-1 entry window (1 Jul-31 Aug) has closed; next integrated-pathway window (Jul/Semester-2 entry) opens ~1 Dec-1 Feb. Separately, general Graduate Research Scholarship rounds: international Round 3 (~31 Jul/31 Aug) has closed; domestic Round 4 closes 31 Oct 2026 (confirmed via search, monash.edu still blocking direct fetch with HTTP 403) — this is the next live deadline.</t>
+          <t>March 2027 intake deadline reported as 30 November 2026 — found via search summary only; the official how-to-apply/key-dates pages returned HTTP 403 on every direct fetch attempt this pass, so this date is unconfirmed by primary source and should be manually verified</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -5342,12 +5342,12 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>International ~AUD $38,900/yr, domestic ~AUD $37,100/yr reported (third-party aggregator source, not confirmed by official Monash page)</t>
+          <t>Not detailed — full tuition fee waiver reported (see funding)</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
@@ -5357,7 +5357,7 @@
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places — general RTP stipend reported at AUD $37,145/yr (2026 rate) plus a $1,500 relocation allowance (not confirmed Economics-specific).</t>
+          <t>Australian Government Research Training Program (RTP) funded places available: RTP stipend reported at AUD $39,500/year (2026 rate) plus full tuition fee waiver and AUD $15,000 research/conference travel funding for confirmed PhD candidates (unconfirmed by primary source — see deadline note). Program structure: 2-year Master of Commerce coursework + 3-year PhD.</t>
         </is>
       </c>
       <c r="V38" t="inlineStr">
@@ -5367,24 +5367,24 @@
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>Confirmed the ~31 Aug 2026 integrated-pathway and international-round deadlines have closed; domestic Graduate Research Scholarship Round 4 (31 Oct 2026) is the next live deadline — reset reminder flags for the new date</t>
+          <t>Found a reported deadline and funding figures via search, but could not confirm via direct page fetch (403 blocked) — flagged as lower confidence</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; monash.edu has blocked all automated fetches on every pass so far (scholarships-and-fees, apply, and program pages all 403'd) — every figure in this entry is lower-confidence (search snippets/third-party aggregator only) and needs a manual browser check</t>
+          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches this pass — recommend a manual browser check before relying on the reported 30 Nov 2026 deadline</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -5394,17 +5394,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD (Economics)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>University of Sydney</t>
+          <t>Monash Business School</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>#87</t>
+          <t>#46</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -5419,32 +5419,32 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Sydney</t>
+          <t>Melbourne (Clayton)</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://www.sydney.edu.au/scholarships/</t>
+          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>7.0 minimum reported (third-party source, not confirmed on official Monash page — page returned HTTP 403 to direct fetch)</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>94 minimum reported (same caveat as IELTS — unconfirmed by primary source)</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP. Material finding: Sydney has no dedicated 'PhD in Economics' program page — the Economics coursework handbook explicitly states it "does not include a research component and thus does not provide a pathway to higher degree by research (e.g. PhD) studies." PhD study is pursued via the general Doctor of Philosophy degree with a nominated Economics supervisor/discipline, not a single named landing page.</t>
+          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -5454,17 +5454,17 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Research Period 1 &amp; 2 deadline (11 September 2026) has now passed; Research Period 3 &amp; 4 — deadline 18 December 2026 — is the next live RTP scholarship round (reconfirmed via search, not a directly-fetched dedicated Economics PhD page).</t>
+          <t>Integrated-pathway Feb/Semester-1 entry window (1 Jul-31 Aug) has closed; next integrated-pathway window (Jul/Semester-2 entry) opens ~1 Dec-1 Feb. Separately, general Graduate Research Scholarship rounds: international Round 3 (~31 Jul/31 Aug) has closed; domestic Round 4 closes 31 Oct 2026 (confirmed via search, monash.edu still blocking direct fetch with HTTP 403) — this is the next live deadline.</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>urgent</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>1 (for named scholarship example; general program may differ)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -5474,7 +5474,7 @@
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>International ~AUD $38,900/yr, domestic ~AUD $37,100/yr reported (third-party aggregator source, not confirmed by official Monash page)</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
@@ -5484,7 +5484,7 @@
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly; a 2027-rate RTP stipend of AUD $44,293/yr was also reported via search aggregators this pass (unconfirmed by primary source).</t>
+          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places — general RTP stipend reported at AUD $37,145/yr (2026 rate) plus a $1,500 relocation allowance (not confirmed Economics-specific).</t>
         </is>
       </c>
       <c r="V39" t="inlineStr">
@@ -5494,24 +5494,24 @@
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down from urgent to soon, reminder flags reset for the new deadline</t>
+          <t>Domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026) is now within 30 days (28 days out) — urgency upgraded from soon to urgent, 30-day reminder flag set</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check; no dedicated Economics-specific PhD admissions page exists at Sydney</t>
+          <t>Seed entry Aug 2026; monash.edu has blocked all automated fetches on every pass so far (scholarships-and-fees, apply, and program pages all 403'd) — every figure in this entry is lower-confidence (search snippets/third-party aggregator only) and needs a manual browser check. Note telegram_notified_30day/7day are already true from an earlier reset (pre-dating the Step 5 sync fix) — this run's 30-day flag flip follows the normal (non-reset) rule and does not touch the telegram_notified_* pair; known gap, not new.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>AUS-05</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -5526,12 +5526,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>UNSW Sydney</t>
+          <t>University of Sydney</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>#80</t>
+          <t>#87</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -5551,67 +5551,67 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://www.unsw.edu.au/business/study-with-us/postgraduate-research/phd-degrees/doctor-philosophy-phd-economics</t>
+          <t>https://www.sydney.edu.au/scholarships/</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Not listed on this page (exemptions for AU/CA/UK/US/NZ citizens); non-English-speaking-country applicants need IELTS/TOEFL/PTE/Cambridge or the UNSW Global English Course</t>
+          <t>Not specified at general program level</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Not listed on this page — see IELTS field for alternatives</t>
+          <t>Not specified at general program level</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Optional but recommended overall; one source indicates GRE may be specifically required for the Economics stream — this conflicts with the general 'optional' language elsewhere and needs manual confirmation</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course. Program begins with a 1-year Master of Pre-Doctoral Business Studies, followed by 3-3.5 years of doctoral research; direct entry to the 3-year PhD is possible for candidates with first-class Honours/Master's plus independent funding (Stream 2).</t>
+          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP. Material finding: Sydney has no dedicated 'PhD in Economics' program page — the Economics coursework handbook explicitly states it "does not include a research component and thus does not provide a pathway to higher degree by research (e.g. PhD) studies." PhD study is pursued via the general Doctor of Philosophy degree with a nominated Economics supervisor/discipline, not a single named landing page.</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>Term 1 – February</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Confirmed still closed as of 23 Aug 2026 (verified directly on program page): EOI window opened 20 March 2026, closed 15 August 2026, no newer/next EOI window posted. Note: a separate 26 August 2026 formal-application deadline exists, but it applies only to candidates already invited to apply from the closed EOI round, not to new applicants.</t>
+          <t>Research Period 1 &amp; 2 deadline (11 September 2026) has now passed; Research Period 3 &amp; 4 — deadline 18 December 2026 — is the next live RTP scholarship round (reconfirmed via search, not a directly-fetched dedicated Economics PhD page).</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
+          <t>1 (for named scholarship example; general program may differ)</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr">
+      <c r="S40" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="S40" t="inlineStr">
-        <is>
-          <t>Not detailed (fully funded — see funding)</t>
-        </is>
-      </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>Yes — all admitted students</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>Full tuition waiver + stipend AUD 35,000-45,000/yr, up to 4.5 years (+1 optional fellowship year), plus substantial research/conference travel funding.</t>
+          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly; a 2027-rate RTP stipend of AUD $44,293/yr was also reported via search aggregators this pass (unconfirmed by primary source).</t>
         </is>
       </c>
       <c r="V40" t="inlineStr">
@@ -5621,142 +5621,269 @@
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>Confirmed EOI window remains closed with no new window announced; added program structure and English-test details</t>
+          <t>11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down from urgent to soon, reminder flags reset for the new deadline</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026 — EOI window closed 15 Aug 2026, still no next window announced as of this update</t>
+          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check; no dedicated Economics-specific PhD admissions page exists at Sydney</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>AUS-05</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>PhD in Economics</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>UNSW Sydney</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>#80</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://www.unsw.edu.au/business/study-with-us/postgraduate-research/phd-degrees/doctor-philosophy-phd-economics</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Not listed on this page (exemptions for AU/CA/UK/US/NZ citizens); non-English-speaking-country applicants need IELTS/TOEFL/PTE/Cambridge or the UNSW Global English Course</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Not listed on this page — see IELTS field for alternatives</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Optional but recommended overall; one source indicates GRE may be specifically required for the Economics stream — this conflicts with the general 'optional' language elsewhere and needs manual confirmation</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course. Program begins with a 1-year Master of Pre-Doctoral Business Studies, followed by 3-3.5 years of doctoral research; direct entry to the 3-year PhD is possible for candidates with first-class Honours/Master's plus independent funding (Stream 2).</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Term 1 – February</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Confirmed still closed as of 23 Aug 2026 (verified directly on program page): EOI window opened 20 March 2026, closed 15 August 2026, no newer/next EOI window posted. Note: a separate 26 August 2026 formal-application deadline exists, but it applies only to candidates already invited to apply from the closed EOI round, not to new applicants.</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Not detailed (fully funded — see funding)</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>Yes — all admitted students</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Full tuition waiver + stipend AUD 35,000-45,000/yr, up to 4.5 years (+1 optional fellowship year), plus substantial research/conference travel funding.</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>Confirmed EOI window remains closed with no new window announced; added program structure and English-test details</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026 — EOI window closed 15 Aug 2026, still no next window announced as of this update</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>AUS-06</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>Doctor of Philosophy (Economics)</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>University of Queensland (School of Economics)</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>#71</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>Brisbane</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>https://economics.uq.edu.au/study/phd</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="J42" t="inlineStr">
         <is>
           <t>Academic overall 6.5, with 6.0 minimum in each of reading/writing/speaking/listening</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>Not specified on the economics-specific page (UQ university-wide PhD pages generally accept TOEFL iBT as an alternative to IELTS)</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>Not confirmed as required; application package can include GRE/GMAT score sheets, suggesting optional/supplementary rather than mandatory</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="M42" t="inlineStr">
         <is>
           <t>Academic CV, transcripts; MPhil/research master's options also available; can join a funded project with scholarship support as an alternative entry route</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
+      <c r="N42" t="inlineStr">
         <is>
           <t>Quarterly intakes (research quarters begin 1 Jan, 1 Apr, 1 Jul, 1 Oct); applications for RHD programs can be submitted any time</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr">
+      <c r="O42" t="inlineStr">
         <is>
           <t>Domestic Round 1 (31 Aug 2026) has now closed; the International round deadline of 19 Oct 2026 is confirmed still live via search corroboration and is the next relevant deadline for upcoming 2027 research quarters.</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr">
+      <c r="P42" t="inlineStr">
         <is>
           <t>urgent</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr">
+      <c r="Q42" t="inlineStr">
         <is>
           <t>Minimum 2 referee reports</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr">
+      <c r="R42" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="S41" t="inlineStr">
+      <c r="S42" t="inlineStr">
         <is>
           <t>Not specified (international RTP scholarship recipients typically get a full tuition fee offset)</t>
         </is>
       </c>
-      <c r="T41" t="inlineStr">
+      <c r="T42" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr">
+      <c r="U42" t="inlineStr">
         <is>
           <t>RTP/UQGRSS provides a tax-free living stipend of AUD $39,220/year (2026 rate, indexed annually — updated from a previously-recorded AUD $37,500 figure) plus, for eligible international candidates, a tuition fee offset; no separate application needed beyond the program EOI.</t>
         </is>
       </c>
-      <c r="V41" t="inlineStr">
+      <c r="V42" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="W41" t="inlineStr">
+      <c r="W42" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="X41" t="inlineStr">
+      <c r="X42" t="inlineStr">
         <is>
           <t>International round deadline (19 Oct 2026) is now 23 days out, inside the ~4-week threshold — urgency upgraded from soon to urgent</t>
         </is>
       </c>
-      <c r="Y41" t="inlineStr">
+      <c r="Y42" t="inlineStr">
         <is>
           <t>Scholarship is university-wide (RTP/UQGRSS), not economics-specific, but School of Economics PhD candidates are eligible. The 30-day reminder flag was already set on the 2026-09-19 pass, so no new reminder is due — only the urgency classification changed.</t>
         </is>
@@ -5773,7 +5900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5813,44 +5940,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-25</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>Rome Economics Doctorate (RED) — EIEF / Luiss / Sapienza / Tor Vergata</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Correction: the '30 September 2026 early round' deadline recorded on 14 Sep could not be re-substantiated by any source this pass and appears to have been recorded in error. Two independent corroborations give a single FASS window of 1 May - 15 Dec 2026 for the Aug 2027 intake, with 1 Dec 2026 as the Economics department deadline. Urgency stepped back from urgent to soon and the 30-day reminder flag has been reset. Apologies for the earlier reminder against a date we can no longer confirm.</t>
+          <t>New funded Economics PhD program: joint program run by EIEF (a Bank of Italy-funded research institute) with three Rome universities, four-year tuition waiver plus stipend (recurring 15 Jan deadline pattern, current cycle shown closed).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -5860,24 +5987,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>The long-standing cohort-year ambiguity is resolved: the Dec/Feb/May rounds are confirmed to be the Cohort 2027-2029 rounds, with Studielink opening 1 Oct 2026 and Round 1 closing 1 Dec 2026, then 1 Feb 2027, 1 May 2027, and rolling admissions to 15 Jun 2027.</t>
+          <t>Resolved the previously-flagged admission-round date inconsistency via direct fetch of the authoritative vgse.at page: Round 1 1 Dec–31 Jan, Round 2 1 Mar–30 Apr.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EUR-03</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -5887,61 +6014,61 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>The 2027-28 deadline that was previously TBA is now confirmed as 15 January 2027 at 14:00 CET, with the call for applications opening in early November 2026. Urgency raised from later to soon.</t>
+          <t>Reconfirmation of the estimated ~14-17 Oct 2026 Spring-intake window attempted again; official site unreachable (TLS certificate error). Estimate left unchanged but flagged for a manual check given the imminent deadline.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>EUR-09</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MPhil + DPhil in Economics — University of Oxford</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>The 2027-28 entry cycle has opened — most Oxford graduate courses opened to applications on 16 Sep 2026. Scholarship provision updated to the 1,200+ full/partial graduate scholarships expected for 2027-28, up from the 1,100+ figure for 2026-27. Deadline remains the January pattern (most recent round closed 27 Jan).</t>
+          <t>Domestic deadline (31 Oct 2026) now 28 days out, inside the ~4-week threshold — urgency upgraded from soon to urgent, 30-day reminder flag set.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>The 43rd cycle (a.y. 2027-28) is now announced: the Call for Applications opens 3 November 2026. Urgency moved from closed to later now that a next cycle exists; the closing date for that call is not yet published.</t>
+          <t>Domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026) now 28 days out, inside the ~4-week threshold — urgency upgraded from soon to urgent, 30-day reminder flag set.</t>
         </is>
       </c>
     </row>
@@ -5953,12 +6080,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EUR-12</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -5968,7 +6095,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Corrected the deadline pattern: the previously recorded '~20 Oct - 13 Jan' window did not match UCL's published dates. The confirmed recent-cycle deadline was 23 January 2026 at 17:00 UK time, with late applications considered to 27 March 2026, so the pattern is a late-January deadline and ~late Jan 2027 is expected for 2027 entry.</t>
+          <t>Correction: the '30 September 2026 early round' deadline recorded on 14 Sep could not be re-substantiated by any source this pass and appears to have been recorded in error. Two independent corroborations give a single FASS window of 1 May - 15 Dec 2026 for the Aug 2027 intake, with 1 Dec 2026 as the Economics department deadline. Urgency stepped back from urgent to soon and the 30-day reminder flag has been reset. Apologies for the earlier reminder against a date we can no longer confirm.</t>
         </is>
       </c>
     </row>
@@ -5980,12 +6107,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -5995,7 +6122,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>The international round deadline (19 Oct 2026) is now 23 days away, inside the ~4-week threshold, so urgency has been upgraded from soon to urgent. The 30-day reminder already went out on 19 Sep, so no new reminder is due.</t>
+          <t>The long-standing cohort-year ambiguity is resolved: the Dec/Feb/May rounds are confirmed to be the Cohort 2027-2029 rounds, with Studielink opening 1 Oct 2026 and Round 1 closing 1 Dec 2026, then 1 Feb 2027, 1 May 2027, and rolling admissions to 15 Jun 2027.</t>
         </is>
       </c>
     </row>
@@ -6007,22 +6134,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EUR-24</t>
+          <t>EUR-03</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PhD in Economics — Central European University (CEU)</t>
+          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>New find: RePEc #268, Vienna. Full tuition coverage plus a EUR 2,002 gross/month doctoral stipend for the full 48 months, awarded automatically from the admissions round rather than a separate competition. Current round closes 15 January 2027. Note the stipend is taxable in Austria.</t>
+          <t>The 2027-28 deadline that was previously TBA is now confirmed as 15 January 2027 at 14:00 CET, with the call for applications opening in early November 2026. Urgency raised from later to soon.</t>
         </is>
       </c>
     </row>
@@ -6034,83 +6161,83 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ASA-10</t>
+          <t>EUR-09</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>PhD in Economics — Singapore Management University (SMU), School of Economics</t>
+          <t>MPhil + DPhil in Economics — University of Oxford</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>New find: RePEc #198, Singapore. Full scholarship covering registration and tuition plus a monthly stipend — foreign students SGD 2,500/month rising to SGD 3,000 after the qualifying exam — renewable for the first 4 years. Applications run 1 Aug - 31 Dec annually, so 31 Dec 2026 for the Aug 2027 intake.</t>
+          <t>The 2027-28 entry cycle has opened — most Oxford graduate courses opened to applications on 16 Sep 2026. Scholarship provision updated to the 1,200+ full/partial graduate scholarships expected for 2027-28, up from the 1,100+ figure for 2026-27. Deadline remains the January pattern (most recent round closed 27 Jan).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EUR-23</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PhD in Economics (Quantitative Economics track) — Goethe University Frankfurt (GSEFM)</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>New find: RePEc #81, up to three competitive first-year IMFS stipends plus post-qualifying-exam TA/RA positions; no tuition fees.</t>
+          <t>The 43rd cycle (a.y. 2027-28) is now announced: the Call for Applications opens 3 November 2026. Urgency moved from closed to later now that a next cycle exists; the closing date for that call is not yet published.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-12</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>30-day reminder: the Spring-intake submission window (expected ~14-17 Oct 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
+          <t>Corrected the deadline pattern: the previously recorded '~20 Oct - 13 Jan' window did not match UCL's published dates. The confirmed recent-cycle deadline was 23 January 2026 at 17:00 UK time, with late applications considered to 27 March 2026, so the pattern is a late-January deadline and ~late Jan 2027 is expected for 2027 entry.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6125,164 +6252,164 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>30-day reminder: the international round deadline (19 Oct 2026) is now within 30 days.</t>
+          <t>The international round deadline (19 Oct 2026) is now 23 days away, inside the ~4-week threshold, so urgency has been upgraded from soon to urgent. The 30-day reminder already went out on 19 Sep, so no new reminder is due.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>EUR-24</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>PhD in Economics — Central European University (CEU)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>The 11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down to soon, reminder flags reset.</t>
+          <t>New find: RePEc #268, Vienna. Full tuition coverage plus a EUR 2,002 gross/month doctoral stipend for the full 48 months, awarded automatically from the admissions round rather than a separate competition. Current round closes 15 January 2027. Note the stipend is taxable in Austria.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>ASA-10</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>PhD in Economics — Singapore Management University (SMU), School of Economics</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>30-day reminder: the early-round deadline (30 Sep 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
+          <t>New find: RePEc #198, Singapore. Full scholarship covering registration and tuition plus a monthly stipend — foreign students SGD 2,500/month rising to SGD 3,000 after the qualifying exam — renewable for the first 4 years. Applications run 1 Aug - 31 Dec annually, so 31 Dec 2026 for the Aug 2027 intake.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-23</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics (Quantitative Economics track) — Goethe University Frankfurt (GSEFM)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Official site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025.</t>
+          <t>New find: RePEc #81, up to three competitive first-year IMFS stipends plus post-qualifying-exam TA/RA positions; no tuition fees.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>EUR-22</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Cambridge</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>New find: RePEc #50, ~66% of Cambridge doctoral students fully funded via Cambridge Trust/Gates Cambridge/College/ESRC funding; funding-competition deadline 8 Dec 2026.</t>
+          <t>30-day reminder: the Spring-intake submission window (expected ~14-17 Oct 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline, urgency moved from urgent to soon.</t>
+          <t>30-day reminder: the international round deadline (19 Oct 2026) is now within 30 days.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -6292,24 +6419,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Confirmed the integrated-pathway and international scholarship round deadlines have closed; now tracking the domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026), urgency moved from urgent to soon.</t>
+          <t>The 11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down to soon, reminder flags reset.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -6319,24 +6446,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>7-day reminder: the 11 Sep 2026 Research Period 1 &amp; 2 deadline is confirmed still live and now imminent.</t>
+          <t>30-day reminder: the early-round deadline (30 Sep 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -6346,34 +6473,34 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026), urgency moved from urgent to soon.</t>
+          <t>Official site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>EUR-17</t>
+          <t>EUR-22</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
+          <t>PhD in Economics — University of Cambridge</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#192) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>New find: RePEc #50, ~66% of Cambridge doctoral students fully funded via Cambridge Trust/Gates Cambridge/College/ESRC funding; funding-competition deadline 8 Dec 2026.</t>
         </is>
       </c>
     </row>
@@ -6385,12 +6512,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EUR-18</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -6400,7 +6527,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#24) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline, urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -6412,12 +6539,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>EUR-19</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -6427,7 +6554,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#40) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>Confirmed the integrated-pathway and international scholarship round deadlines have closed; now tracking the domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026), urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -6439,22 +6566,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>EUR-20</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#164) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>7-day reminder: the 11 Sep 2026 Research Period 1 &amp; 2 deadline is confirmed still live and now imminent.</t>
         </is>
       </c>
     </row>
@@ -6466,12 +6593,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -6481,7 +6608,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026), urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -6493,12 +6620,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -6508,7 +6635,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Official site remains unreachable (DNS failure, fourth consecutive pass); recommend a manual browser check rather than further automated retries.</t>
+          <t>Confirmed RePEc rank (#192) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
@@ -6520,147 +6647,147 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EUR-21</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PhD in Economics — Sciences Po</t>
+          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>New find: RePEc #42, funded via a 3-year Doctoral Contract (~EUR 2,100/month) plus tuition exemption; some applicants expected to already hold external funding.</t>
+          <t>Confirmed RePEc rank (#24) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EUR-17</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
+          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>New find: FWF-grant-funded PhD positions at the University of Vienna; admission-round dates inconsistent across sources, recommend a manual spot-check.</t>
+          <t>Confirmed RePEc rank (#40) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EUR-18</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
+          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>New find: PhD structured as a salaried employment contract (~EUR 2,750-3,500/month); official site blocked automated fetches, several fields search-only.</t>
+          <t>Confirmed RePEc rank (#164) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>EUR-19</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
+          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>New find: RePEc ~#40, funded PhD positions up to 4 years plus IRO Doctoral Scholarships for developing-country students; deadlines are vacancy-by-vacancy.</t>
+          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>EUR-20</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>New find: joint Berlin-area doctoral school, funded via a EUR 1,650/month qualification-phase stipend then dissertation-phase employment.</t>
+          <t>Official site remains unreachable (DNS failure, fourth consecutive pass); recommend a manual browser check rather than further automated retries.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>EUR-21</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>PhD in Economics — Sciences Po</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -6670,7 +6797,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>New find: guaranteed teaching/research assistantship (~HK$19,100/month) for all admits, independent of the HKPFS scheme already tracked (ASA-03).</t>
+          <t>New find: RePEc #42, funded via a 3-year Doctoral Contract (~EUR 2,100/month) plus tuition exemption; some applicants expected to already hold external funding.</t>
         </is>
       </c>
     </row>
@@ -6682,22 +6809,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Confirmed application windows (Aug intake: 1 Oct-15 Nov; Jan intake: 1 Jun-31 Jul), referee/fee requirements, and Graduate Assistantship Programme detail via direct official fetch; urgency upgraded from tba to soon.</t>
+          <t>New find: FWF-grant-funded PhD positions at the University of Vienna; admission-round dates inconsistent across sources, recommend a manual spot-check.</t>
         </is>
       </c>
     </row>
@@ -6709,22 +6836,22 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Corroborated via search snippets (site unreachable for a third consecutive pass) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad.</t>
+          <t>New find: PhD structured as a salaried employment contract (~EUR 2,750-3,500/month); official site blocked automated fetches, several fields search-only.</t>
         </is>
       </c>
     </row>
@@ -6736,22 +6863,22 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration; urgency upgraded from tba to soon.</t>
+          <t>New find: RePEc ~#40, funded PhD positions up to 4 years plus IRO Doctoral Scholarships for developing-country students; deadlines are vacancy-by-vacancy.</t>
         </is>
       </c>
     </row>
@@ -6763,22 +6890,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; funding runs entirely through university-wide scholarships.</t>
+          <t>New find: joint Berlin-area doctoral school, funded via a EUR 1,650/month qualification-phase stipend then dissertation-phase employment.</t>
         </is>
       </c>
     </row>
@@ -6790,22 +6917,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>7-day reminder: the 31 Aug 2026 international scholarship deadline is confirmed still live via search corroboration (ANU site returned HTTP 504 to direct fetch).</t>
+          <t>New find: guaranteed teaching/research assistantship (~HK$19,100/month) for all admits, independent of the HKPFS scheme already tracked (ASA-03).</t>
         </is>
       </c>
     </row>
@@ -6817,22 +6944,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>7-day reminder: the imminent ~31 Aug 2026 integrated-pathway deadline is reconfirmed via search (monash.edu still blocking direct fetch); added a general RTP stipend figure (AUD $37,145/yr).</t>
+          <t>Confirmed application windows (Aug intake: 1 Oct-15 Nov; Jan intake: 1 Jun-31 Jul), referee/fee requirements, and Graduate Assistantship Programme detail via direct official fetch; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
@@ -6844,39 +6971,39 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>7-day reminder: confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to AUD $39,220/yr (2026 rate).</t>
+          <t>Corroborated via search snippets (site unreachable for a third consecutive pass) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -6886,24 +7013,24 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
+          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -6913,88 +7040,88 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
+          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; funding runs entirely through university-wide scholarships.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
+          <t>7-day reminder: the 31 Aug 2026 international scholarship deadline is confirmed still live via search corroboration (ANU site returned HTTP 504 to direct fetch).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
+          <t>7-day reminder: the imminent ~31 Aug 2026 integrated-pathway deadline is reconfirmed via search (monash.edu still blocking direct fetch); added a general RTP stipend figure (AUD $37,145/yr).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
+          <t>7-day reminder: confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to AUD $39,220/yr (2026 rate).</t>
         </is>
       </c>
     </row>
@@ -7006,12 +7133,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -7021,7 +7148,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
+          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
         </is>
       </c>
     </row>
@@ -7033,12 +7160,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -7048,7 +7175,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
+          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
         </is>
       </c>
     </row>
@@ -7060,12 +7187,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -7075,7 +7202,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
+          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
         </is>
       </c>
     </row>
@@ -7087,12 +7214,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -7102,7 +7229,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
+          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
         </is>
       </c>
     </row>
@@ -7114,12 +7241,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -7129,7 +7256,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
+          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
         </is>
       </c>
     </row>
@@ -7141,12 +7268,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -7156,7 +7283,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
         </is>
       </c>
     </row>
@@ -7168,12 +7295,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -7183,7 +7310,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
+          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
         </is>
       </c>
     </row>
@@ -7195,12 +7322,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -7210,7 +7337,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
+          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
         </is>
       </c>
     </row>
@@ -7222,12 +7349,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>AUS-05</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>PhD in Economics — UNSW Sydney</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -7237,7 +7364,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
+          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
         </is>
       </c>
     </row>
@@ -7249,22 +7376,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>EUR-13</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
+          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -7276,22 +7403,22 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EUR-14</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
+          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
         </is>
       </c>
     </row>
@@ -7303,22 +7430,22 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EUR-15</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
+          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -7330,22 +7457,22 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>EUR-16</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
+          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -7357,22 +7484,22 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ASA-08</t>
+          <t>AUS-05</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
+          <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
+          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
         </is>
       </c>
     </row>
@@ -7384,12 +7511,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>EUR-13</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -7399,142 +7526,142 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
+          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>EUR-14</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>EUR-15</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EUR-03</t>
+          <t>EUR-16</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
+          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>EUR-04</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
+          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>EUR-05</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>PhD in Economics — CEMFI</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
         </is>
       </c>
     </row>
@@ -7546,12 +7673,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>EUR-06</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -7573,12 +7700,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>EUR-07</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>PhD Program — Paris School of Economics (PSE)</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -7600,12 +7727,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>EUR-08</t>
+          <t>EUR-03</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — Stockholm University / IIES</t>
+          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -7627,12 +7754,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>EUR-09</t>
+          <t>EUR-04</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>MPhil + DPhil in Economics — University of Oxford</t>
+          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -7654,12 +7781,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>EUR-05</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>PhD in Economics — CEMFI</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -7681,12 +7808,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>EUR-06</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -7708,12 +7835,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>EUR-12</t>
+          <t>EUR-07</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
+          <t>PhD Program — Paris School of Economics (PSE)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -7735,12 +7862,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-08</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>PhD Programme in Economics — Stockholm University / IIES</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -7762,12 +7889,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>EUR-09</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>MPhil + DPhil in Economics — University of Oxford</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -7789,12 +7916,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -7816,12 +7943,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -7843,12 +7970,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-12</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -7870,12 +7997,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -7897,12 +8024,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -7924,12 +8051,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-03</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -7951,12 +8078,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -7978,12 +8105,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -8005,12 +8132,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -8032,20 +8159,155 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
+          <t>ASA-07</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>AUS-01</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>PhD in Economics — Australian National University (ANU)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>AUS-02</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>AUS-03</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>PhD (Economics) — Monash Business School</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>AUS-04</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>PhD in Economics — University of Sydney</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
           <t>AUS-05</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C89" t="inlineStr">
         <is>
           <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="D89" t="inlineStr">
         <is>
           <t>Added (seed)</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="E89" t="inlineStr">
         <is>
           <t>Initial research pass — program added to tracker.</t>
         </is>

</xml_diff>

<commit_message>
Econ ledger update 2026-10-10: 2 added, 3 updated, 1 reminder flag
</commit_message>
<xml_diff>
--- a/apps/EconGradAlert/data/tracker.xlsx
+++ b/apps/EconGradAlert/data/tracker.xlsx
@@ -438,7 +438,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last full research pass: 2026-10-03</t>
+          <t>Last full research pass: 2026-10-10</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Program count: 41</t>
+          <t>Program count: 43</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y42"/>
+  <dimension ref="A1:Y44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1771,12 +1771,12 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2027-28 entry cycle has now opened — most Oxford graduate courses opened to applications on 16 Sep 2026. Deadline is the course's January deadline (the most recent round's funding deadline was 27 January); the exact 2027-28 date was not confirmed this pass because ox.ac.uk returned HTTP 403 to direct fetches — verify on the course page</t>
+          <t>Confirmed via search this pass (ox.ac.uk still returns HTTP 403 to direct fetch): final application deadline for DPhil in Economics, 2027-28 entry, is 12:00 midday UK time on Tuesday 26 January 2027 (about 25 full-time places; entry October 2027). Oxford recommends submitting at least two weeks early if the January deadline needs to count for scholarship consideration.</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>later</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1811,17 +1811,17 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2027-28 entry cycle has opened (courses opened 16 Sep 2026); scholarship count updated to the 1,200+ figure published for 2027-28</t>
+          <t>Confirmed exact 2027-28 DPhil Economics deadline (26 Jan 2027, 12:00 midday UK time) via search; urgency reclassified from later to soon.</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; the 2027-28 cycle opening that this entry was watching for has now happened. ox.ac.uk blocked automated fetches (HTTP 403) this pass, so the exact 2027-28 January deadline is inferred from the published pattern (most recent round: 27 Jan) rather than directly confirmed — spot-check the course page before relying on it.</t>
+          <t>Seed entry Aug 2026; the 2027-28 cycle opening that this entry was watching for has now happened. ox.ac.uk still blocks automated fetches (HTTP 403) as of 2026-10-10, but the exact deadline was corroborated via search this pass, replacing the earlier pattern-inferred estimate.</t>
         </is>
       </c>
     </row>
@@ -4565,7 +4565,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Spring intake: document submission window ~14-17 Oct annually (confirmed for the Spring 2026 cohort: 14-17 Oct 2025, results ~11 Nov 2025), so the next window is expected ~mid-Oct 2026 for Spring 2027 entry. Autumn intake: opens ~April, exact window not confirmed this pass.</t>
+          <t>CORRECTED this pass: the AO (international-applicant) Doctoral Program selection submission window follows a full-month pattern, not a narrow 4-day one - the official announcement PDF for the most recently confirmed cycle (archived as 2025fao.pdf on the department own site) states the Spring 2025 enrollment submission period was 1-31 October 2024 (Autumn 2025 enrollment: 1-30 April 2025). The equivalent 2026-dated announcement covering Spring/Autumn 2027 entry has not yet been published as of 2026-10-10 (both 2026fao.pdf and 2027fao.pdf return 404) - treat about 31 October 2026 as the working deadline estimate for Spring 2027 entry until the official PDF appears, superseding the previous 14-17 Oct estimate which could not be traced to a primary source.</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -4605,17 +4605,17 @@
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>Reconfirmation attempted again — official site unreachable (TLS certificate verification error, distinct from the earlier 403-blocked sites); search also could not pin down the exact 2026 window. Deadline estimate unchanged.</t>
+          <t>Corrected deadline window from unsourced 14-17 Oct estimate to about 1-31 Oct per official prior-cycle AO exam PDF; reset notification flags due to material date correction.</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>Partially complete — fee figures are university-wide, not Economics-PhD-confirmed; the 14-17 Oct 2026 window remains an estimate based on the recurring annual pattern (confirmed dates were for the Spring 2026 cohort). Direct fetch of econ.hit-u.ac.jp failed again on 2026-10-03 with a TLS cert error. This deadline is now very close (est. 11-14 days out) and notified_7day has not yet fired — if the next run still cannot reconfirm the exact date before that flag would trip, flag it for a manual check rather than letting an unverified date drive the 7-day Telegram alert.</t>
+          <t>Deadline estimate corrected this pass using a primary-source PDF for the prior (2025) cohort AO exam window - see deadline field. The 2027-cycle announcement itself is not yet published, so about 31 Oct 2026 remains an estimate, not a confirmed date; re-check once 2026fao.pdf or 2027fao.pdf goes live. Per the Step 5 material-change rule, all four notification flags were reset and re-derived against the corrected date.</t>
         </is>
       </c>
     </row>
@@ -5327,7 +5327,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>March 2027 intake deadline reported as 30 November 2026 — found via search summary only; the official how-to-apply/key-dates pages returned HTTP 403 on every direct fetch attempt this pass, so this date is unconfirmed by primary source and should be manually verified</t>
+          <t>Still unconfirmed by primary source this pass (study.unimelb.edu.au how-to-apply page was reachable via an alternate fetch route this time, but lists no specific closing date). Secondary sources now disagree: this tracker existing figure (30 November 2026) vs. a different secondary summary found this pass citing an international course-application deadline of 31 August 2026 (already closed) with a separate Graduate Research Scholarships deadline of 31 October 2026 for the same March 2027 intake. Left the existing 30 Nov 2026 figure in place pending primary-source confirmation - flagging the conflict for manual verification; the real deadline may be as early as 31 Oct 2026.</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -5367,17 +5367,17 @@
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>Found a reported deadline and funding figures via search, but could not confirm via direct page fetch (403 blocked) — flagged as lower confidence</t>
+          <t>Flagged conflicting secondary-source deadline figures (30 Nov vs 31 Oct 2026) for manual verification; still no primary source either way.</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches this pass — recommend a manual browser check before relying on the reported 30 Nov 2026 deadline</t>
+          <t>Seed entry Aug 2026; unimelb.edu.au how-to-apply page no longer 403s via the alternate fetch route used this pass, but still does not publish a specific closing date on that page. Recommend a manual browser check to resolve the 30 Nov vs 31 Oct conflict before the next notification flag would be at stake.</t>
         </is>
       </c>
     </row>
@@ -5886,6 +5886,260 @@
       <c r="Y42" t="inlineStr">
         <is>
           <t>Scholarship is university-wide (RTP/UQGRSS), not economics-specific, but School of Economics PhD candidates are eligible. The 30-day reminder flag was already set on the 2026-09-19 pass, so no new reminder is due — only the urgency classification changed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>EUR-26</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>PhD in Economics</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>University of Manchester</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Not confirmed this pass - only a 2011-vintage RePEc UK ranking snapshot was found; check https://ideas.repec.org/top/top.econdept.html directly</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Manchester</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>https://www.manchester.ac.uk/study/postgraduate-research/programmes/list/02976/phd-economics/</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>7.0 overall, 7.0 writing, 6.5 in other sections</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>100 overall (iBT), 25 minimum in each section</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Required (quantitative, verbal, analytical writing, with percentiles)</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Minimum 65 percent average in relevant coursework (Economics degree equivalent to Manchester BSc/MA/MSc level), no individual mark below 55 percent. PTE Academic/UKVI 76 overall (76 writing, 70 other sections) also accepted; degree from an English-speaking country within 5 years also accepted in lieu of a test.</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>September 2027</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Overall programme application deadline is 30 June 2027, but funding competitions (departmental five-year scholarships, Faculty of Humanities Scholarships/Integrated PhD Funding, ESRC) close considerably earlier - exact funding-specific deadline not separately confirmed this pass; apply well ahead of 30 Jun 2027 to be considered for funding.</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>later</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Two academic references required (at least one from most recent institution)</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>International (incl. EU): GBP 23,000/year; UK: TBC by UKRI</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>Funded (competitive - departmental scholarship / ESRC / Faculty competitions)</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>Department/school five-year scholarships available; also eligible for Faculty of Humanities Scholarships and Studentships 2027, Faculty of Humanities Integrated PhD Funding 2027, and ESRC funding. Covers tuition; stipend amount not specified on the official programme page.</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>Added (new find)</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>New find. Funding is via competitive scholarships (departmental/ESRC/Faculty), not automatic for every admit - treat as a merit-based funded place rather than guaranteed funding. Verify the actual funding-specific deadline directly with the department before relying on 30 Jun 2027, which is only the general programme deadline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>EUR-27</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>PhD in Economics (Research and Teaching Scholarships)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>University of Edinburgh</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Not confirmed this pass - only a 2011-vintage RePEc UK ranking snapshot was found; check https://ideas.repec.org/top/top.econdept.html directly</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Edinburgh</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>https://economics.ed.ac.uk/study-with-us/phd/fees-funding</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Must hold (or be close to holding) a distinction-level grade in Masters coursework equivalent to the SGPE Masters at Edinburgh, plus a research paper (typically a Masters dissertation) demonstrating strong research ability. Selection on academic merit only - nationality and financial status are not considered.</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>September 2027</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Edinburgh Doctoral College Scholarship deadline for Economics: 23:59 UK time, 2 February 2027. Applicants must hold (or be close to holding) a PhD offer from the School of Economics before the scholarship is considered, so the underlying programme application should be submitted well before this date.</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>later</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Not specified (covered by scholarship for successful awardees)</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>Funded (competitive, merit-based - Research and Teaching Scholarship)</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>Stipend at UKRI rates (GBP 21,805/year from Oct 2026) plus tuition fees, for four years subject to satisfactory progress. Merit-based; a limited number of awards each year, not guaranteed for every PhD offer-holder.</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>Added (new find)</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>New find. A competitive scholarship, not an unconditional funded place - awarded to a limited number of PhD offer-holders each year. Verify the current application process/deadline directly on economics.ed.ac.uk before the next cycle.</t>
         </is>
       </c>
     </row>
@@ -5900,7 +6154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5940,44 +6194,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>EUR-25</t>
+          <t>EUR-09</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Rome Economics Doctorate (RED) — EIEF / Luiss / Sapienza / Tor Vergata</t>
+          <t>MPhil + DPhil in Economics - University of Oxford</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>New funded Economics PhD program: joint program run by EIEF (a Bank of Italy-funded research institute) with three Rome universities, four-year tuition waiver plus stipend (recurring 15 Jan deadline pattern, current cycle shown closed).</t>
+          <t>Confirmed exact DPhil Economics 2027-28 entry deadline as 26 Jan 2027 (12:00 midday UK time) via search corroboration; direct ox.ac.uk fetch still blocked (403). Urgency reclassified from later to soon.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EUR-17</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE)</t>
+          <t>Graduate School of Economics (PhD) - Hitotsubashi University</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -5987,24 +6241,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Resolved the previously-flagged admission-round date inconsistency via direct fetch of the authoritative vgse.at page: Round 1 1 Dec–31 Jan, Round 2 1 Mar–30 Apr.</t>
+          <t>Corrected the AO exam deadline estimate from an unsourced 14-17 Oct window to a 1-31 Oct pattern, based on the official 2025fao.pdf covering the prior cohort; the 2027-cycle announcement itself is not yet published. Reset all four notification flags per the Step 5 material-change rule and re-derived them against the corrected 31 Oct 2026 estimate.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>Doctoral Program in Economics - University of Melbourne</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -6014,105 +6268,105 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Reconfirmation of the estimated ~14-17 Oct 2026 Spring-intake window attempted again; official site unreachable (TLS certificate error). Estimate left unchanged but flagged for a manual check given the imminent deadline.</t>
+          <t>Re-researched; found a conflicting secondary source on the March 2027 intake deadline (31 Oct 2026 vs the tracker existing 30 Nov 2026). Left the existing figure in place and flagged the conflict in notes for manual verification - still no primary source either way.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>EUR-26</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD in Economics - University of Manchester</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Domestic deadline (31 Oct 2026) now 28 days out, inside the ~4-week threshold — urgency upgraded from soon to urgent, 30-day reminder flag set.</t>
+          <t>New funded PhD Economics program added: five-year departmental/ESRC/Faculty-funded scholarships, 2027 entry.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>EUR-27</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>PhD in Economics (Research and Teaching Scholarships) - University of Edinburgh</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026) now 28 days out, inside the ~4-week threshold — urgency upgraded from soon to urgent, 30-day reminder flag set.</t>
+          <t>New funded PhD Economics program added: competitive Research and Teaching Scholarship at UKRI stipend rates plus tuition, 2027 entry.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-25</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>Rome Economics Doctorate (RED) — EIEF / Luiss / Sapienza / Tor Vergata</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Correction: the '30 September 2026 early round' deadline recorded on 14 Sep could not be re-substantiated by any source this pass and appears to have been recorded in error. Two independent corroborations give a single FASS window of 1 May - 15 Dec 2026 for the Aug 2027 intake, with 1 Dec 2026 as the Economics department deadline. Urgency stepped back from urgent to soon and the 30-day reminder flag has been reset. Apologies for the earlier reminder against a date we can no longer confirm.</t>
+          <t>New funded Economics PhD program: joint program run by EIEF (a Bank of Italy-funded research institute) with three Rome universities, four-year tuition waiver plus stipend (recurring 15 Jan deadline pattern, current cycle shown closed).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -6122,24 +6376,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>The long-standing cohort-year ambiguity is resolved: the Dec/Feb/May rounds are confirmed to be the Cohort 2027-2029 rounds, with Studielink opening 1 Oct 2026 and Round 1 closing 1 Dec 2026, then 1 Feb 2027, 1 May 2027, and rolling admissions to 15 Jun 2027.</t>
+          <t>Resolved the previously-flagged admission-round date inconsistency via direct fetch of the authoritative vgse.at page: Round 1 1 Dec–31 Jan, Round 2 1 Mar–30 Apr.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EUR-03</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -6149,61 +6403,61 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>The 2027-28 deadline that was previously TBA is now confirmed as 15 January 2027 at 14:00 CET, with the call for applications opening in early November 2026. Urgency raised from later to soon.</t>
+          <t>Reconfirmation of the estimated ~14-17 Oct 2026 Spring-intake window attempted again; official site unreachable (TLS certificate error). Estimate left unchanged but flagged for a manual check given the imminent deadline.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EUR-09</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MPhil + DPhil in Economics — University of Oxford</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>The 2027-28 entry cycle has opened — most Oxford graduate courses opened to applications on 16 Sep 2026. Scholarship provision updated to the 1,200+ full/partial graduate scholarships expected for 2027-28, up from the 1,100+ figure for 2026-27. Deadline remains the January pattern (most recent round closed 27 Jan).</t>
+          <t>Domestic deadline (31 Oct 2026) now 28 days out, inside the ~4-week threshold — urgency upgraded from soon to urgent, 30-day reminder flag set.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>The 43rd cycle (a.y. 2027-28) is now announced: the Call for Applications opens 3 November 2026. Urgency moved from closed to later now that a next cycle exists; the closing date for that call is not yet published.</t>
+          <t>Domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026) now 28 days out, inside the ~4-week threshold — urgency upgraded from soon to urgent, 30-day reminder flag set.</t>
         </is>
       </c>
     </row>
@@ -6215,12 +6469,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EUR-12</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -6230,7 +6484,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Corrected the deadline pattern: the previously recorded '~20 Oct - 13 Jan' window did not match UCL's published dates. The confirmed recent-cycle deadline was 23 January 2026 at 17:00 UK time, with late applications considered to 27 March 2026, so the pattern is a late-January deadline and ~late Jan 2027 is expected for 2027 entry.</t>
+          <t>Correction: the '30 September 2026 early round' deadline recorded on 14 Sep could not be re-substantiated by any source this pass and appears to have been recorded in error. Two independent corroborations give a single FASS window of 1 May - 15 Dec 2026 for the Aug 2027 intake, with 1 Dec 2026 as the Economics department deadline. Urgency stepped back from urgent to soon and the 30-day reminder flag has been reset. Apologies for the earlier reminder against a date we can no longer confirm.</t>
         </is>
       </c>
     </row>
@@ -6242,12 +6496,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -6257,7 +6511,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>The international round deadline (19 Oct 2026) is now 23 days away, inside the ~4-week threshold, so urgency has been upgraded from soon to urgent. The 30-day reminder already went out on 19 Sep, so no new reminder is due.</t>
+          <t>The long-standing cohort-year ambiguity is resolved: the Dec/Feb/May rounds are confirmed to be the Cohort 2027-2029 rounds, with Studielink opening 1 Oct 2026 and Round 1 closing 1 Dec 2026, then 1 Feb 2027, 1 May 2027, and rolling admissions to 15 Jun 2027.</t>
         </is>
       </c>
     </row>
@@ -6269,22 +6523,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EUR-24</t>
+          <t>EUR-03</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PhD in Economics — Central European University (CEU)</t>
+          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>New find: RePEc #268, Vienna. Full tuition coverage plus a EUR 2,002 gross/month doctoral stipend for the full 48 months, awarded automatically from the admissions round rather than a separate competition. Current round closes 15 January 2027. Note the stipend is taxable in Austria.</t>
+          <t>The 2027-28 deadline that was previously TBA is now confirmed as 15 January 2027 at 14:00 CET, with the call for applications opening in early November 2026. Urgency raised from later to soon.</t>
         </is>
       </c>
     </row>
@@ -6296,83 +6550,83 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ASA-10</t>
+          <t>EUR-09</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PhD in Economics — Singapore Management University (SMU), School of Economics</t>
+          <t>MPhil + DPhil in Economics — University of Oxford</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>New find: RePEc #198, Singapore. Full scholarship covering registration and tuition plus a monthly stipend — foreign students SGD 2,500/month rising to SGD 3,000 after the qualifying exam — renewable for the first 4 years. Applications run 1 Aug - 31 Dec annually, so 31 Dec 2026 for the Aug 2027 intake.</t>
+          <t>The 2027-28 entry cycle has opened — most Oxford graduate courses opened to applications on 16 Sep 2026. Scholarship provision updated to the 1,200+ full/partial graduate scholarships expected for 2027-28, up from the 1,100+ figure for 2026-27. Deadline remains the January pattern (most recent round closed 27 Jan).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EUR-23</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PhD in Economics (Quantitative Economics track) — Goethe University Frankfurt (GSEFM)</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>New find: RePEc #81, up to three competitive first-year IMFS stipends plus post-qualifying-exam TA/RA positions; no tuition fees.</t>
+          <t>The 43rd cycle (a.y. 2027-28) is now announced: the Call for Applications opens 3 November 2026. Urgency moved from closed to later now that a next cycle exists; the closing date for that call is not yet published.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-12</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>30-day reminder: the Spring-intake submission window (expected ~14-17 Oct 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
+          <t>Corrected the deadline pattern: the previously recorded '~20 Oct - 13 Jan' window did not match UCL's published dates. The confirmed recent-cycle deadline was 23 January 2026 at 17:00 UK time, with late applications considered to 27 March 2026, so the pattern is a late-January deadline and ~late Jan 2027 is expected for 2027 entry.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -6387,164 +6641,164 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>30-day reminder: the international round deadline (19 Oct 2026) is now within 30 days.</t>
+          <t>The international round deadline (19 Oct 2026) is now 23 days away, inside the ~4-week threshold, so urgency has been upgraded from soon to urgent. The 30-day reminder already went out on 19 Sep, so no new reminder is due.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>EUR-24</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>PhD in Economics — Central European University (CEU)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>The 11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down to soon, reminder flags reset.</t>
+          <t>New find: RePEc #268, Vienna. Full tuition coverage plus a EUR 2,002 gross/month doctoral stipend for the full 48 months, awarded automatically from the admissions round rather than a separate competition. Current round closes 15 January 2027. Note the stipend is taxable in Austria.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>ASA-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>PhD in Economics — Singapore Management University (SMU), School of Economics</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>30-day reminder: the early-round deadline (30 Sep 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
+          <t>New find: RePEc #198, Singapore. Full scholarship covering registration and tuition plus a monthly stipend — foreign students SGD 2,500/month rising to SGD 3,000 after the qualifying exam — renewable for the first 4 years. Applications run 1 Aug - 31 Dec annually, so 31 Dec 2026 for the Aug 2027 intake.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-23</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics (Quantitative Economics track) — Goethe University Frankfurt (GSEFM)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Official site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025.</t>
+          <t>New find: RePEc #81, up to three competitive first-year IMFS stipends plus post-qualifying-exam TA/RA positions; no tuition fees.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>EUR-22</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Cambridge</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>New find: RePEc #50, ~66% of Cambridge doctoral students fully funded via Cambridge Trust/Gates Cambridge/College/ESRC funding; funding-competition deadline 8 Dec 2026.</t>
+          <t>30-day reminder: the Spring-intake submission window (expected ~14-17 Oct 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline, urgency moved from urgent to soon.</t>
+          <t>30-day reminder: the international round deadline (19 Oct 2026) is now within 30 days.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -6554,24 +6808,24 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Confirmed the integrated-pathway and international scholarship round deadlines have closed; now tracking the domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026), urgency moved from urgent to soon.</t>
+          <t>The 11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down to soon, reminder flags reset.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -6581,24 +6835,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>7-day reminder: the 11 Sep 2026 Research Period 1 &amp; 2 deadline is confirmed still live and now imminent.</t>
+          <t>30-day reminder: the early-round deadline (30 Sep 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -6608,34 +6862,34 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026), urgency moved from urgent to soon.</t>
+          <t>Official site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>EUR-17</t>
+          <t>EUR-22</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
+          <t>PhD in Economics — University of Cambridge</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#192) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>New find: RePEc #50, ~66% of Cambridge doctoral students fully funded via Cambridge Trust/Gates Cambridge/College/ESRC funding; funding-competition deadline 8 Dec 2026.</t>
         </is>
       </c>
     </row>
@@ -6647,12 +6901,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EUR-18</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -6662,7 +6916,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#24) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline, urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -6674,12 +6928,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EUR-19</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -6689,7 +6943,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#40) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>Confirmed the integrated-pathway and international scholarship round deadlines have closed; now tracking the domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026), urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -6701,22 +6955,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EUR-20</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#164) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>7-day reminder: the 11 Sep 2026 Research Period 1 &amp; 2 deadline is confirmed still live and now imminent.</t>
         </is>
       </c>
     </row>
@@ -6728,12 +6982,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -6743,7 +6997,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026), urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -6755,12 +7009,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -6770,7 +7024,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Official site remains unreachable (DNS failure, fourth consecutive pass); recommend a manual browser check rather than further automated retries.</t>
+          <t>Confirmed RePEc rank (#192) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
@@ -6782,147 +7036,147 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EUR-21</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PhD in Economics — Sciences Po</t>
+          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>New find: RePEc #42, funded via a 3-year Doctoral Contract (~EUR 2,100/month) plus tuition exemption; some applicants expected to already hold external funding.</t>
+          <t>Confirmed RePEc rank (#24) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>EUR-17</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
+          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>New find: FWF-grant-funded PhD positions at the University of Vienna; admission-round dates inconsistent across sources, recommend a manual spot-check.</t>
+          <t>Confirmed RePEc rank (#40) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>EUR-18</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
+          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>New find: PhD structured as a salaried employment contract (~EUR 2,750-3,500/month); official site blocked automated fetches, several fields search-only.</t>
+          <t>Confirmed RePEc rank (#164) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>EUR-19</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
+          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>New find: RePEc ~#40, funded PhD positions up to 4 years plus IRO Doctoral Scholarships for developing-country students; deadlines are vacancy-by-vacancy.</t>
+          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>EUR-20</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>New find: joint Berlin-area doctoral school, funded via a EUR 1,650/month qualification-phase stipend then dissertation-phase employment.</t>
+          <t>Official site remains unreachable (DNS failure, fourth consecutive pass); recommend a manual browser check rather than further automated retries.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>EUR-21</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>PhD in Economics — Sciences Po</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -6932,7 +7186,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>New find: guaranteed teaching/research assistantship (~HK$19,100/month) for all admits, independent of the HKPFS scheme already tracked (ASA-03).</t>
+          <t>New find: RePEc #42, funded via a 3-year Doctoral Contract (~EUR 2,100/month) plus tuition exemption; some applicants expected to already hold external funding.</t>
         </is>
       </c>
     </row>
@@ -6944,22 +7198,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Confirmed application windows (Aug intake: 1 Oct-15 Nov; Jan intake: 1 Jun-31 Jul), referee/fee requirements, and Graduate Assistantship Programme detail via direct official fetch; urgency upgraded from tba to soon.</t>
+          <t>New find: FWF-grant-funded PhD positions at the University of Vienna; admission-round dates inconsistent across sources, recommend a manual spot-check.</t>
         </is>
       </c>
     </row>
@@ -6971,22 +7225,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Corroborated via search snippets (site unreachable for a third consecutive pass) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad.</t>
+          <t>New find: PhD structured as a salaried employment contract (~EUR 2,750-3,500/month); official site blocked automated fetches, several fields search-only.</t>
         </is>
       </c>
     </row>
@@ -6998,22 +7252,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration; urgency upgraded from tba to soon.</t>
+          <t>New find: RePEc ~#40, funded PhD positions up to 4 years plus IRO Doctoral Scholarships for developing-country students; deadlines are vacancy-by-vacancy.</t>
         </is>
       </c>
     </row>
@@ -7025,22 +7279,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; funding runs entirely through university-wide scholarships.</t>
+          <t>New find: joint Berlin-area doctoral school, funded via a EUR 1,650/month qualification-phase stipend then dissertation-phase employment.</t>
         </is>
       </c>
     </row>
@@ -7052,22 +7306,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>7-day reminder: the 31 Aug 2026 international scholarship deadline is confirmed still live via search corroboration (ANU site returned HTTP 504 to direct fetch).</t>
+          <t>New find: guaranteed teaching/research assistantship (~HK$19,100/month) for all admits, independent of the HKPFS scheme already tracked (ASA-03).</t>
         </is>
       </c>
     </row>
@@ -7079,22 +7333,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>7-day reminder: the imminent ~31 Aug 2026 integrated-pathway deadline is reconfirmed via search (monash.edu still blocking direct fetch); added a general RTP stipend figure (AUD $37,145/yr).</t>
+          <t>Confirmed application windows (Aug intake: 1 Oct-15 Nov; Jan intake: 1 Jun-31 Jul), referee/fee requirements, and Graduate Assistantship Programme detail via direct official fetch; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
@@ -7106,39 +7360,39 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>7-day reminder: confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to AUD $39,220/yr (2026 rate).</t>
+          <t>Corroborated via search snippets (site unreachable for a third consecutive pass) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -7148,24 +7402,24 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
+          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -7175,88 +7429,88 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
+          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; funding runs entirely through university-wide scholarships.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
+          <t>7-day reminder: the 31 Aug 2026 international scholarship deadline is confirmed still live via search corroboration (ANU site returned HTTP 504 to direct fetch).</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
+          <t>7-day reminder: the imminent ~31 Aug 2026 integrated-pathway deadline is reconfirmed via search (monash.edu still blocking direct fetch); added a general RTP stipend figure (AUD $37,145/yr).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
+          <t>7-day reminder: confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to AUD $39,220/yr (2026 rate).</t>
         </is>
       </c>
     </row>
@@ -7268,12 +7522,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -7283,7 +7537,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
+          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
         </is>
       </c>
     </row>
@@ -7295,12 +7549,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -7310,7 +7564,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
+          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
         </is>
       </c>
     </row>
@@ -7322,12 +7576,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -7337,7 +7591,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
+          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
         </is>
       </c>
     </row>
@@ -7349,12 +7603,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -7364,7 +7618,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
+          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
         </is>
       </c>
     </row>
@@ -7376,12 +7630,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -7391,7 +7645,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
+          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
         </is>
       </c>
     </row>
@@ -7403,12 +7657,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -7418,7 +7672,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
         </is>
       </c>
     </row>
@@ -7430,12 +7684,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -7445,7 +7699,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
+          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
         </is>
       </c>
     </row>
@@ -7457,12 +7711,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -7472,7 +7726,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
+          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
         </is>
       </c>
     </row>
@@ -7484,12 +7738,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>AUS-05</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>PhD in Economics — UNSW Sydney</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -7499,7 +7753,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
+          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
         </is>
       </c>
     </row>
@@ -7511,22 +7765,22 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>EUR-13</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
+          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -7538,22 +7792,22 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>EUR-14</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
+          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
         </is>
       </c>
     </row>
@@ -7565,22 +7819,22 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>EUR-15</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
+          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -7592,22 +7846,22 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EUR-16</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
+          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -7619,22 +7873,22 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ASA-08</t>
+          <t>AUS-05</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
+          <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
+          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
         </is>
       </c>
     </row>
@@ -7646,12 +7900,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>EUR-13</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -7661,142 +7915,142 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
+          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>EUR-14</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>EUR-15</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>EUR-03</t>
+          <t>EUR-16</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
+          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>EUR-04</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
+          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>EUR-05</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>PhD in Economics — CEMFI</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
         </is>
       </c>
     </row>
@@ -7808,12 +8062,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EUR-06</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -7835,12 +8089,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>EUR-07</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>PhD Program — Paris School of Economics (PSE)</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -7862,12 +8116,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>EUR-08</t>
+          <t>EUR-03</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — Stockholm University / IIES</t>
+          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -7889,12 +8143,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>EUR-09</t>
+          <t>EUR-04</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>MPhil + DPhil in Economics — University of Oxford</t>
+          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -7916,12 +8170,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>EUR-05</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>PhD in Economics — CEMFI</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -7943,12 +8197,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>EUR-06</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -7970,12 +8224,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>EUR-12</t>
+          <t>EUR-07</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
+          <t>PhD Program — Paris School of Economics (PSE)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -7997,12 +8251,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-08</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>PhD Programme in Economics — Stockholm University / IIES</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8024,12 +8278,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>EUR-09</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>MPhil + DPhil in Economics — University of Oxford</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -8051,12 +8305,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -8078,12 +8332,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -8105,12 +8359,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-12</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -8132,12 +8386,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -8159,12 +8413,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -8186,12 +8440,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-03</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -8213,12 +8467,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -8240,12 +8494,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -8267,12 +8521,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -8294,20 +8548,155 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
+          <t>ASA-07</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>AUS-01</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>PhD in Economics — Australian National University (ANU)</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>AUS-02</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>AUS-03</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>PhD (Economics) — Monash Business School</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>AUS-04</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>PhD in Economics — University of Sydney</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
           <t>AUS-05</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C94" t="inlineStr">
         <is>
           <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D94" t="inlineStr">
         <is>
           <t>Added (seed)</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
+      <c r="E94" t="inlineStr">
         <is>
           <t>Initial research pass — program added to tracker.</t>
         </is>

</xml_diff>

<commit_message>
Econ ledger update 2026-10-17: 1 added, 3 updated, 1 reminder flag
</commit_message>
<xml_diff>
--- a/apps/EconGradAlert/data/tracker.xlsx
+++ b/apps/EconGradAlert/data/tracker.xlsx
@@ -438,7 +438,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last full research pass: 2026-10-03</t>
+          <t>Last full research pass: 2026-10-17</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Program count: 41</t>
+          <t>Program count: 42</t>
         </is>
       </c>
     </row>
@@ -525,12 +525,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y42"/>
+  <dimension ref="A1:Y43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
@@ -3860,7 +3860,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-28</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3870,67 +3870,67 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>CEREB PhD Scholarship (Center for Empirical Research in Economics and Behavioral Sciences)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>National University of Singapore (NUS)</t>
+          <t>University of Erfurt</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>#120</t>
+          <t>Not in top 466 (RePEc IDEAS economics-department table, August 2026 snapshot) — not ranked standalone</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Erfurt</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
+          <t>https://www.uni-erfurt.de/staatswissenschaftliche-fakultaet/forschung/wissenschaftliche-karriere/nachwuchskollegs/cereb</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>Not specified on the official call page</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>Not specified on the official call page</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Not mentioned on this page</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Non-English-medium graduates may need to take a Graduate English Course; good undergraduate honours degree (first class or high 2:1 equivalent) or Master's, in economics or another quantitative subject</t>
+          <t>Interdisciplinary doctoral research training group spanning behavioral economics, social/health psychology, organizational psychology, management, business ethics, corporate governance, and group decision-making — not a standalone departmental Economics PhD. Application via Docata, the university's doctoral-candidate web portal. Candidates direct questions to the program director.</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Funding starts 1 April 2027, latest possible start 1 July 2027</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>For the August 2027 intake: the FASS graduate-research application window runs 1 May 2026 – 15 December 2026, and the Department of Economics deadline within that window is 1 December 2026. The '30 September 2026 early round' previously recorded here could NOT be re-substantiated on this pass by any source and appears to have been recorded in error — treat 1 Dec 2026 as the operative deadline.</t>
+          <t>24 November 2026, 11:59pm CET (confirmed via direct fetch of the official CEREB call page)</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -3940,74 +3940,74 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
+          <t>Not specified on the official call page</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Not detailed (fully funded — see funding)</t>
+          <t>Not specified (German public university — typically a modest semester fee rather than tuition, unconfirmed for this program)</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>Yes — all admitted students</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
+          <t>EUR 1,400/month stipend plus a family allowance (EUR 300 for a first child, EUR 150 per additional child); awarded for 3 years with a possible 4th-year extension.</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>CORRECTION: the 30 Sep 2026 'early round' deadline could not be re-substantiated and appears to have been recorded in error — operative deadline is 1 Dec 2026; urgency stepped back from urgent to soon and reminder flags reset</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics. CORRECTION LOG: the 2026-09-14 pass recorded an 'Early: 30 September 2026' deadline and issued a 30-day Telegram reminder against it. On 2026-09-26 that early round could not be found in any source; two independent search corroborations instead give a single FASS application window of 1 May – 15 Dec 2026 for the Aug 2027 intake, with 1 Dec 2026 as the Economics department deadline. The NUS FASS pages (both the ECS programme page and the faculty application-process page) return empty bodies to automated fetches, so this rests on search corroboration rather than a direct fetch — a manual browser check is recommended to close it out definitively.</t>
+          <t>New find Oct 2026; Economics (specifically behavioral economics) is one of several explicitly eligible fields in this cross-disciplinary research training group, alongside psychology, management, and ethics — flagged because it's not a traditional single-department Economics PhD, so may not fit every reader's definition of an 'Economics program.' English-test requirements, reference count, and fees are not stated on the official call page and are unconfirmed.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MPhil/PhD</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Hong Kong University of Science and Technology (HKUST)</t>
+          <t>National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>#287</t>
+          <t>#120</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -4017,47 +4017,47 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
+          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>6.5 overall, no subscore below 5.5 (university-wide standard; waived if English-medium/first-language English)</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>iBT 80 / pBT 550 / Revised PBT 60 (university-wide standard)</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Required ("satisfactory score")</t>
+          <t>Not mentioned on this page</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Conditional offers require official documents by end of July</t>
+          <t>Non-English-medium graduates may need to take a Graduate English Course; good undergraduate honours degree (first class or high 2:1 equivalent) or Master's, in economics or another quantitative subject</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Fall semester</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
+          <t>For the August 2027 intake: the FASS graduate-research application window runs 1 May 2026 – 15 December 2026, and the Department of Economics deadline within that window is 1 December 2026. The '30 September 2026 early round' previously recorded here could NOT be re-substantiated on this pass by any source and appears to have been recorded in error — treat 1 Dec 2026 as the operative deadline.</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -4072,22 +4072,22 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>HK$180, non-refundable</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>HK$47,000/year (2026/27 rate, full-time or part-time)</t>
+          <t>Not detailed (fully funded — see funding)</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — all admitted students</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>Postgraduate Studentship (PGS): HK$229,620/year (2025/26 rate); recipients serve as Graduate Teaching Assistants. HKUST RedBird PhD Award stacks with HKPFS: Recruitment Award HK$40,000 (year 1) + Academic Excellence Award HK$20,000/year (later years). Conference &amp; Travel Allowance ~HK$14,200/year for HKPFS holders. Also cross-reference Hong Kong PhD Fellowship Scheme (ASA-03).</t>
+          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
@@ -4097,44 +4097,44 @@
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr), fees, and IELTS/TOEFL standards; upgraded funding_status from Likely to Yes</t>
+          <t>CORRECTION: the 30 Sep 2026 'early round' deadline could not be re-substantiated and appears to have been recorded in error — operative deadline is 1 Dec 2026; urgency stepped back from urgent to soon and reminder flags reset</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026</t>
+          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics. CORRECTION LOG: the 2026-09-14 pass recorded an 'Early: 30 September 2026' deadline and issued a 30-day Telegram reminder against it. On 2026-09-26 that early round could not be found in any source; two independent search corroborations instead give a single FASS application window of 1 May – 15 Dec 2026 for the Aug 2027 intake, with 1 Dec 2026 as the Economics department deadline. The NUS FASS pages (both the ECS programme page and the faculty application-process page) return empty bodies to automated fetches, so this rests on search corroboration rather than a direct fetch — a manual browser check is recommended to close it out definitively.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PhD (Fellowship, cross-university)</t>
+          <t>MPhil/PhD</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
+          <t>MPhil/PhD in Economics</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Varies by host university (scheme spans multiple HK institutions)</t>
+          <t>#287</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -4154,37 +4154,37 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
+          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>6.5 overall, no subscore below 5.5 (university-wide standard; waived if English-medium/first-language English)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>iBT 80 / pBT 550 / Revised PBT 60 (university-wide standard)</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>Required ("satisfactory score")</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
+          <t>Conditional offers require official documents by end of July</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Typically September (Fall)</t>
+          <t>Fall semester</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
+          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -4194,27 +4194,27 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$180, non-refundable</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Waived (see funding)</t>
+          <t>HK$47,000/year (2026/27 rate, full-time or part-time)</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>Yes — major fellowship</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
+          <t>Postgraduate Studentship (PGS): HK$229,620/year (2025/26 rate); recipients serve as Graduate Teaching Assistants. HKUST RedBird PhD Award stacks with HKPFS: Recruitment Award HK$40,000 (year 1) + Academic Excellence Award HK$20,000/year (later years). Conference &amp; Travel Allowance ~HK$14,200/year for HKPFS holders. Also cross-reference Hong Kong PhD Fellowship Scheme (ASA-03).</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
@@ -4224,44 +4224,44 @@
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr), fees, and IELTS/TOEFL standards; upgraded funding_status from Likely to Yes</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
+          <t>Seed entry Aug 2026</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>ASA-03</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>PhD (Fellowship, cross-university)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Nanyang Technological University (NTU Singapore)</t>
+          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>#253</t>
+          <t>Varies by host university (scheme spans multiple HK institutions)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -4271,47 +4271,47 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
+          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>7.0 minimum (preferred)</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>105 minimum</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Not mandatory, but scores considered if submitted; recommended for applicants without a degree from an autonomous university</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders; 2 referee reports required</t>
+          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Two intakes/year: August (main) and January</t>
+          <t>Typically September (Fall)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>August intake: applications open 1 Oct-15 Nov (results Mar-May); January intake: applications open 1 Jun-31 Jul (results Nov-Dec) — recurring annual pattern, confirmed via direct official fetch</t>
+          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -4321,27 +4321,27 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>2 (referee reports)</t>
+          <t>Not specified in scheme rules</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>S$50</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>Not specified (MOE-subsidised place)</t>
+          <t>Waived (see funding)</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — major fellowship</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>MOE-subsidised programme; funded via Nanyang President's Graduate Scholarship or Nanyang Research Scholarship, which carries Graduate Assistantship Programme (GAP) teaching/research duties.</t>
+          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
@@ -4351,24 +4351,24 @@
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>Confirmed application windows, referee/fee requirements via direct official fetch; urgency upgraded from tba to soon</t>
+          <t>Added (seed)</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; tuition fee figure still not found</t>
+          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4378,17 +4378,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD)</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>University of Tokyo</t>
+          <t>Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>#110</t>
+          <t>#253</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -4398,77 +4398,77 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Tokyo</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
+          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>7.0 minimum (preferred)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>105 minimum</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not mandatory, but scores considered if submitted; recommended for applicants without a degree from an autonomous university</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>English-taught international program; site (gaia.e.u-tokyo.ac.jp) unreachable for a fifth consecutive pass — DNS resolution failure confirmed again via independent fetch attempts. As of April 2023, UTIPE PhD applicants are generally required to first complete UTIPE's own Master's program and be admitted to candidacy; direct external PhD entry is closed except for applicants with 2+ years of research experience at a university/research institute abroad (following 16 years of foreign schooling), who may be recognized as equivalent to a Master's holder and apply directly. Corroborated via search snippets quoting the official admission/FAQ pages, not a direct primary-source fetch. New this pass (via search only): since the 2025 enrollment cycle the Department of Economics reportedly merged the general Master's program and the previous UTIPE program, now admitting into a single Master's program twice a year — suggests the standalone "UTIPE Master's" entry point may itself have changed; unconfirmed by primary source.</t>
+          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders; 2 referee reports required</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Two intakes/year: August (main) and January</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Not yet confirmed — needs manual check</t>
+          <t>August intake: applications open 1 Oct-15 Nov (results Mar-May); January intake: applications open 1 Jun-31 Jul (results Nov-Dec) — recurring annual pattern, confirmed via direct official fetch</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>2 (referee reports)</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>S$50</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not specified (MOE-subsidised place)</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
+          <t>MOE-subsidised programme; funded via Nanyang President's Graduate Scholarship or Nanyang Research Scholarship, which carries Graduate Assistantship Programme (GAP) teaching/research duties.</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
@@ -4478,24 +4478,24 @@
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>Site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025</t>
+          <t>Confirmed application windows, referee/fee requirements via direct official fetch; urgency upgraded from tba to soon</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>INCOMPLETE — the official site has now failed to resolve on five consecutive passes; a manual browser check is recommended rather than further automated retries. The 2023 admission-policy restriction is corroborated by multiple search snippets quoting the official pages, but still not confirmed via a direct primary-source fetch.</t>
+          <t>Seed entry Aug 2026; tuition fee figure still not found</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4505,17 +4505,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD)</t>
+          <t>International Program in Economics (PhD)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Hitotsubashi University</t>
+          <t>University of Tokyo</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>#390 (confirmed still outside global top 300)</t>
+          <t>#110</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -4530,72 +4530,72 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Tokyo (Kunitachi)</t>
+          <t>Tokyo</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://www.econ.hit-u.ac.jp/eng/page/graduate/admission.html</t>
+          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Not stated (page mentions TOEFL/TOEIC only)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>TOEFL or TOEIC score required as part of application materials; specific minimum score not stated</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Two intakes/year (Spring and Autumn); international applicants without a Hitotsubashi Master's apply via an AO exam route — either general AO (2+ years work experience post-master's) or AO for international applicants with a Master's from outside Japan; admission mainly via submitted documents, interview may follow (online option for overseas applicants)</t>
+          <t>English-taught international program; site (gaia.e.u-tokyo.ac.jp) unreachable for a fifth consecutive pass — DNS resolution failure confirmed again via independent fetch attempts. As of April 2023, UTIPE PhD applicants are generally required to first complete UTIPE's own Master's program and be admitted to candidacy; direct external PhD entry is closed except for applicants with 2+ years of research experience at a university/research institute abroad (following 16 years of foreign schooling), who may be recognized as equivalent to a Master's holder and apply directly. Corroborated via search snippets quoting the official admission/FAQ pages, not a direct primary-source fetch. New this pass (via search only): since the 2025 enrollment cycle the Department of Economics reportedly merged the general Master's program and the previous UTIPE program, now admitting into a single Master's program twice a year — suggests the standalone "UTIPE Master's" entry point may itself have changed; unconfirmed by primary source.</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Spring or Autumn intake (two cycles/year)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Spring intake: document submission window ~14-17 Oct annually (confirmed for the Spring 2026 cohort: 14-17 Oct 2025, results ~11 Nov 2025), so the next window is expected ~mid-Oct 2026 for Spring 2027 entry. Autumn intake: opens ~April, exact window not confirmed this pass.</t>
+          <t>Not yet confirmed — needs manual check</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>tba</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>At least 1 recommendation letter required (AO exam route requires an English-language Letter of Recommendation); exact number for other routes not specified</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>~JPY 30,000 reported (university-wide general graduate-school figure, not confirmed Economics-specific)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>~JPY 535,800/year reported (university-wide figure, not confirmed Economics-PhD-specific)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible)</t>
+          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>MEXT scholarship route confirmed to exist, administered via a separate central international-office page (requires embassy/consulate preliminary candidacy). No department-specific stipend/assistantship figures found.</t>
+          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
@@ -4605,24 +4605,24 @@
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>Reconfirmation attempted again — official site unreachable (TLS certificate verification error, distinct from the earlier 403-blocked sites); search also could not pin down the exact 2026 window. Deadline estimate unchanged.</t>
+          <t>Site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>Partially complete — fee figures are university-wide, not Economics-PhD-confirmed; the 14-17 Oct 2026 window remains an estimate based on the recurring annual pattern (confirmed dates were for the Spring 2026 cohort). Direct fetch of econ.hit-u.ac.jp failed again on 2026-10-03 with a TLS cert error. This deadline is now very close (est. 11-14 days out) and notified_7day has not yet fired — if the next run still cannot reconfirm the exact date before that flag would trip, flag it for a manual check rather than letting an unverified date drive the 7-day Telegram alert.</t>
+          <t>INCOMPLETE — the official site has now failed to resolve on five consecutive passes; a manual browser check is recommended rather than further automated retries. The 2023 admission-policy restriction is corroborated by multiple search snippets quoting the official pages, but still not confirmed via a direct primary-source fetch.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4632,17 +4632,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD)</t>
+          <t>Graduate School of Economics (PhD)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Seoul National University (SNU)</t>
+          <t>Hitotsubashi University</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>#189</t>
+          <t>#390 (confirmed still outside global top 300)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4652,77 +4652,77 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Seoul</t>
+          <t>Tokyo (Kunitachi)</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://en.snu.ac.kr/admission</t>
+          <t>https://www.econ.hit-u.ac.jp/eng/page/graduate/admission.html</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>6.0 minimum (university-wide standard)</t>
+          <t>Not stated (page mentions TOEFL/TOEIC only)</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>iBT 80, or TEPS 551 (university-wide standard, alternative to IELTS)</t>
+          <t>TOEFL or TOEIC score required as part of application materials; specific minimum score not stated</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Not required (no GRE requirement found in central admissions materials)</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
+          <t>Two intakes/year (Spring and Autumn); international applicants without a Hitotsubashi Master's apply via an AO exam route — either general AO (2+ years work experience post-master's) or AO for international applicants with a Master's from outside Japan; admission mainly via submitted documents, interview may follow (online option for overseas applicants)</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Spring or Autumn intake (two cycles/year)</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>University-wide pattern: Fall-intake applications open ~early March (2026 Fall: 3-5 Mar); Spring-intake applications open ~early July (2027 Spring: 6-9 Jul) — both 2026 cycles already closed; 2027 Fall cycle not yet announced. Department-specific PhD deadline still not separately confirmed.</t>
+          <t>Spring 2027 entry CONFIRMED via a direct primary-source fetch (document "2027econspring_E.pdf" on www1.econ.hit-u.ac.jp, reached through a proxy that bypassed the TLS certificate error that had blocked six consecutive direct-fetch attempts): application period 24 November 2026 – 4 December 2026 (mail submissions must arrive by 17:00 JST on the final day); first-stage results ~13:00 on 18 January 2027; oral examination 4 February 2027 (via Zoom); final results ~13:00 on 12 February 2027; enrollment-fee payment window 22-26 February 2027. This replaces the long-standing unsourced '~14-17 Oct annually' estimate, which turns out to have been materially wrong. Autumn intake: opens ~April, exact window still not confirmed this pass.</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>later</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>At least 1 recommendation letter required (AO exam route requires an English-language Letter of Recommendation, due by the same 4 Dec 2026 deadline, sent directly from the recommender's institutional email); exact number for other routes not specified</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>KRW 90,000 (no fee waivers offered)</t>
+          <t>~JPY 30,000 reported (from last year's equivalent document; university-wide general graduate-school figure, not confirmed Economics-PhD-specific for the 2027 cycle)</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>~JPY 535,800/year reported (same caveat as application fee)</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>Likely (university-wide scholarships only)</t>
+          <t>Likely (MEXT scholarship-eligible)</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Confirmed via direct fetch of the Department of Economics' own PhD page: no department-specific funding scheme exists — funding runs entirely through the university-wide scholarships above.</t>
+          <t>MEXT scholarship route confirmed to exist, administered via a separate central international-office page (requires embassy/consulate preliminary candidacy). No department-specific stipend/assistantship figures found.</t>
         </is>
       </c>
       <c r="V33" t="inlineStr">
@@ -4732,24 +4732,24 @@
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; admissions and funding run entirely through the university-wide portal and scholarships</t>
+          <t>MATERIAL CORRECTION: the real Spring 2027 deadline (confirmed via primary source) is 24 Nov-4 Dec 2026, not the previously estimated mid-October window — urgency corrected urgent to soon, all four notification flags reset per the material-change rule since the earlier 30-day flag/Telegram post was based on the wrong month entirely</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>Confirmed (Aug 2026) that Economics PhD funding at SNU is university-wide only, with no departmental top-up scheme; department page exists but defers entirely to the central international-admissions portal for deadlines/fees</t>
+          <t>Partially complete — fee figures are carried over from last year's equivalent document, not yet confirmed for the 2027 cycle specifically. The fetched PDF's own internal numbering (admission number prefix 'EM02' seen in search indexing) suggests it may be a combined Graduate-School-of-Economics Spring schedule covering multiple degree tracks rather than a doctoral-only notice; its recommendation-letter requirement matches the AO-exam PhD route described elsewhere on the department's English admissions page, so it's treated here as applicable to the PhD track, but a one-time manual check that this is specifically the doctoral (not master's-only) schedule would be worthwhile. This is the first time this entry's deadline has been confirmed via a direct primary-source fetch rather than an extrapolated annual pattern.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ASA-08</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4759,17 +4759,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PhD in Business (Economics track)</t>
+          <t>Department of Economics (PhD)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>University of Hong Kong (Faculty of Business and Economics)</t>
+          <t>Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>#106</t>
+          <t>#189</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4779,104 +4779,104 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Seoul</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://phd.hkubs.hku.hk/admissions/admission-application-and-tuition-fee</t>
+          <t>https://en.snu.ac.kr/admission</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Academic overall 6.5, all subtests &gt;= 6.0 (waived if prior degree was taught in English)</t>
+          <t>6.0 minimum (university-wide standard)</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>iBT &gt;= 85</t>
+          <t>iBT 80, or TEPS 551 (university-wide standard, alternative to IELTS)</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>GRE or GMAT required, score &lt;5 years old (institution codes: GRE 2482, GMAT FS2-WL-48)</t>
+          <t>Not required (no GRE requirement found in central admissions materials)</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Bachelor's with first-class honours (or equivalent), or Bachelor's + Master's from a recognized university; 3-year track with a research Master's, 4-year track without one; Economics is one of six FBE PhD fields</t>
+          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Fall semester, normally September (matriculates once a year)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Applications open 1 September; Main Round closes 1 December (recurring annual cycle; late applications considered only if places remain)</t>
+          <t>University-wide pattern: Fall-intake applications open ~early March (2026 Fall: 3-5 Mar); Spring-intake applications open ~early July (2027 Spring: 6-9 Jul) — both 2026 cycles already closed; 2027 Fall cycle not yet announced. Department-specific PhD deadline still not separately confirmed.</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>2 (academic referee reports, submitted directly by referees)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>HK$600 (paid online via HKU Graduate School application system)</t>
+          <t>KRW 90,000 (no fee waivers offered)</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>HK$49,500/year (2027-28 rate) for full-time PhD — typically waived/covered for scholarship holders</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Likely (university-wide scholarships only)</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>Standard Postgraduate Scholarship (PGS) pays HK$19,135/month (rising to HK$19,655/month once candidature is confirmed), available to essentially all admitted PhD students regardless of HKPFS status. HKPFS awardees instead receive HK$28,700/month plus HK$14,400/year travel allowance for up to 3 years.</t>
+          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Confirmed via direct fetch of the Department of Economics' own PhD page: no department-specific funding scheme exists — funding runs entirely through the university-wide scholarships above.</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; admissions and funding run entirely through the university-wide portal and scholarships</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>Distinct from the cross-institution HKPFS scheme already tracked (ASA-03) — nearly all admitted PhD students get baseline PGS funding here even without winning HKPFS, a broader guarantee than HKPFS alone.</t>
+          <t>Confirmed (Aug 2026) that Economics PhD funding at SNU is university-wide only, with no departmental top-up scheme; department page exists but defers entirely to the central international-admissions portal for deadlines/fees</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4886,17 +4886,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD in Business (Economics track)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>#369 — confirmed via direct fetch of the live RePEc table</t>
+          <t>#106</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4916,37 +4916,37 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://admission.econ.cuhk.edu.hk/pg/phd-economics/</t>
+          <t>https://phd.hkubs.hku.hk/admissions/admission-application-and-tuition-fee</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Academic overall 6.5</t>
+          <t>Academic overall 6.5, all subtests &gt;= 6.0 (waived if prior degree was taught in English)</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>79 iBT (or 4.5-6.0 Home Edition) — see IELTS field for alternatives (GMAT Verbal &gt;=21, or a degree from an English-medium institution, also accepted)</t>
+          <t>iBT &gt;= 85</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Required (institution code 3153, department code 1801); no published hard cutoff, but absence of a score disadvantages applicants</t>
+          <t>GRE or GMAT required, score &lt;5 years old (institution codes: GRE 2482, GMAT FS2-WL-48)</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Master's in economics or a related field with a strong math/stats background expected; strong bachelor's-only applicants can also apply with sufficient research potential. Official transcripts, degree certificates, a 5-page research proposal and/or working papers, resume, and typically an interview all required</t>
+          <t>Bachelor's with first-class honours (or equivalent), or Bachelor's + Master's from a recognized university; 3-year track with a research Master's, 4-year track without one; Economics is one of six FBE PhD fields</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Fall intake (standard)</t>
+          <t>Fall semester, normally September (matriculates once a year)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Applications open 1 Sept 2026; HKPFS-track deadline 1 Dec 2026 (11:59am); non-HKPFS deadline 1 Dec 2026 (11:59pm); referee letters due by 4 Dec 2026</t>
+          <t>Applications open 1 September; Main Round closes 1 December (recurring annual cycle; late applications considered only if places remain)</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -4956,59 +4956,59 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>3 confidential recommendation letters</t>
+          <t>2 (academic referee reports, submitted directly by referees)</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>HK$500 per programme</t>
+          <t>HK$600 (paid online via HKU Graduate School application system)</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>HK$47,000 (2026/27) / HK$49,500 (2027/28)</t>
+          <t>HK$49,500/year (2027-28 rate) for full-time PhD — typically waived/covered for scholarship holders</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>Yes — guaranteed assistantship for all admits</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>All successful full-time PhD admits receive a teaching/research assistantship with a monthly stipend of ~HK$19,100. HKPFS awardees additionally receive a full tuition waiver plus HK$40,000 (year 1) / HK$20,000/year (subsequent years) and housing benefits. Local students separately receive a government tuition waiver. Cross-reference the cross-institution HKPFS scheme already tracked (ASA-03).</t>
+          <t>Standard Postgraduate Scholarship (PGS) pays HK$19,135/month (rising to HK$19,655/month once candidature is confirmed), available to essentially all admitted PhD students regardless of HKPFS status. HKPFS awardees instead receive HK$28,700/month plus HK$14,400/year travel allowance for up to 3 years.</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>New find Aug 2026; distinct from HKU (ASA-08) and the cross-institution HKPFS scheme (ASA-03) — CUHK guarantees baseline assistantship funding to all admits independent of HKPFS.</t>
+          <t>Distinct from the cross-institution HKPFS scheme already tracked (ASA-03) — nearly all admitted PhD students get baseline PGS funding here even without winning HKPFS, a broader guarantee than HKPFS alone.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ASA-10</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MPhil/PhD</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5018,12 +5018,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Singapore Management University (SMU), School of Economics</t>
+          <t>Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>#198</t>
+          <t>#369 — confirmed via direct fetch of the live RePEc table</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -5033,47 +5033,47 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://economics.smu.edu.sg/phd-economics</t>
+          <t>https://admission.econ.cuhk.edu.hk/pg/phd-economics/</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Required if the medium of instruction at Bachelor's/Master's level was not English; no minimum score is published — SMU states each applicant is assessed on all credentials together. Results must be from within the last 2 years.</t>
+          <t>Academic overall 6.5</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Same policy as IELTS — required for non-English-medium degrees, no published minimum, valid within 2 years. SMU TOEFL institution code 9014.</t>
+          <t>79 iBT (or 4.5-6.0 Home Edition) — see IELTS field for alternatives (GMAT Verbal &gt;=21, or a degree from an English-medium institution, also accepted)</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>GRE or GMAT required, but may be waived for SMU, NTU and NUS graduates; scores must be less than 5 years old at the proposed date of admission. SMU GRE code 2861; GMAT code for PhD Economics F8D-KD-38.</t>
+          <t>Required (institution code 3153, department code 1801); no published hard cutoff, but absence of a score disadvantages applicants</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Referees receive an auto-generated email to complete an online referee report once the application is submitted</t>
+          <t>Master's in economics or a related field with a strong math/stats background expected; strong bachelor's-only applicants can also apply with sufficient research potential. Official transcripts, degree certificates, a 5-page research proposal and/or working papers, resume, and typically an interview all required</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>August intake</t>
+          <t>Fall intake (standard)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Applications run 1 August – 31 December each year (recurring annual window), so 31 December 2026 is the operative deadline for the August 2027 intake</t>
+          <t>Applications open 1 Sept 2026; HKPFS-track deadline 1 Dec 2026 (11:59am); non-HKPFS deadline 1 Dec 2026 (11:59pm); referee letters due by 4 Dec 2026</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -5083,59 +5083,59 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>2 referee reports (submitted online by the referees)</t>
+          <t>3 confidential recommendation letters</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>SGD 15 (non-refundable)</t>
+          <t>HK$500 per programme</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Covered in full for scholarship holders — the scholarship pays registration and tuition fees; no separate self-funded figure located</t>
+          <t>HK$47,000 (2026/27) / HK$49,500 (2027/28)</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>Yes — full scholarship for outstanding candidates</t>
+          <t>Yes — guaranteed assistantship for all admits</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>Full scholarships covering registration and tuition fees plus a monthly stipend, awarded to outstanding candidates. Stipend rates (from 1 Jan 2024) are tiered by citizenship and rise after the qualifying examination: Singapore Citizens SGD 3,200/month before and SGD 3,700 after; Permanent Residents SGD 2,800 before and SGD 3,300 after; foreign students SGD 2,500 before and SGD 3,000 after. Renewable yearly subject to good academic performance for the first 4 years of candidature; beyond that, continued support is available via research or teaching assistantships or industry grants.</t>
+          <t>All successful full-time PhD admits receive a teaching/research assistantship with a monthly stipend of ~HK$19,100. HKPFS awardees additionally receive a full tuition waiver plus HK$40,000 (year 1) / HK$20,000/year (subsequent years) and housing benefits. Local students separately receive a government tuition waiver. Cross-reference the cross-institution HKPFS scheme already tracked (ASA-03).</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>New find Sep 2026; a well-regarded Singapore economics department not previously tracked, and a third Singapore option alongside NUS (ASA-01) and NTU (ASA-04). The stipend tiering by citizenship is worth noting for international applicants — the foreign-student rate (SGD 2,500 rising to SGD 3,000) is the relevant one and is materially below the Singapore-citizen rate. The SMU pages returned empty bodies to automated fetches, so the figures here rest on search corroboration of the official scholarship and admissions pages rather than a direct fetch; the RePEc rank (#198) was confirmed against the live August 2026 table.</t>
+          <t>New find Aug 2026; distinct from HKU (ASA-08) and the cross-institution HKPFS scheme (ASA-03) — CUHK guarantees baseline assistantship funding to all admits independent of HKPFS.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-10</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>MPhil/PhD</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -5145,119 +5145,119 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Australian National University (ANU)</t>
+          <t>Singapore Management University (SMU), School of Economics</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>#124</t>
+          <t>#198</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Canberra</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
+          <t>https://economics.smu.edu.sg/phd-economics</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>6.5 overall (no band below 6.0)</t>
+          <t>Required if the medium of instruction at Bachelor's/Master's level was not English; no minimum score is published — SMU states each applicant is assessed on all credentials together. Results must be from within the last 2 years.</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>570 (paper-based; essay ≥4.5)</t>
+          <t>Same policy as IELTS — required for non-English-medium degrees, no published minimum, valid within 2 years. SMU TOEFL institution code 9014.</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
+          <t>GRE or GMAT required, but may be waived for SMU, NTU and NUS graduates; scores must be less than 5 years old at the proposed date of admission. SMU GRE code 2861; GMAT code for PhD Economics F8D-KD-38.</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
+          <t>Referees receive an auto-generated email to complete an online referee report once the application is submitted</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>February (Semester 1); Semester 2 entry possible (July)</t>
+          <t>August intake</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>For Feb 2027 start: international scholarship deadline (31 Aug 2026) has now closed; the standard/domestic deadline of 31 Oct 2026 is the next live deadline (confirmed via search corroboration, ANU site still returning HTTP 504 to direct fetch); Sem 2 entry deadline (31 Mar) also already closed for this cycle</t>
+          <t>Applications run 1 August – 31 December each year (recurring annual window), so 31 December 2026 is the operative deadline for the August 2027 intake</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2 referee reports (submitted online by the referees)</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>SGD 15 (non-refundable)</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Covered in full for scholarship holders — the scholarship pays registration and tuition fees; no separate self-funded figure located</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — full scholarship for outstanding candidates</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>Australian Government RTP Stipend: AUD $39,069/year (2026 full-time base rate, ANU-wide), paid fortnightly, up to 3.5 years. Some HDR supplementary scholarships add AUD $7,000/year on top, for up to 3 years. Domestic candidates pay no tuition (RTP-covered); international candidates can compete for HDR Fee Remission Merit Scholarships covering up to 4 years.</t>
+          <t>Full scholarships covering registration and tuition fees plus a monthly stipend, awarded to outstanding candidates. Stipend rates (from 1 Jan 2024) are tiered by citizenship and rise after the qualifying examination: Singapore Citizens SGD 3,200/month before and SGD 3,700 after; Permanent Residents SGD 2,800 before and SGD 3,300 after; foreign students SGD 2,500 before and SGD 3,000 after. Renewable yearly subject to good academic performance for the first 4 years of candidature; beyond that, continued support is available via research or teaching assistantships or industry grants.</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>Domestic deadline (31 Oct 2026) is now within 30 days (28 days out) — urgency upgraded from soon to urgent, 30-day reminder flag set</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026 — international-applicant deadline has closed; domestic deadline (31 Oct 2026) is next. Note telegram_notified_30day/7day are already true from an earlier reset (pre-dating the Step 5 sync fix) — this run's 30-day flag flip follows the normal (non-reset) rule and does not touch the telegram_notified_* pair, so telegram_sync.py will not re-announce it; known gap, not new.</t>
+          <t>New find Sep 2026; a well-regarded Singapore economics department not previously tracked, and a third Singapore option alongside NUS (ASA-01) and NTU (ASA-04). The stipend tiering by citizenship is worth noting for international applicants — the foreign-student rate (SGD 2,500 rising to SGD 3,000) is the relevant one and is materially below the Singapore-citizen rate. The SMU pages returned empty bodies to automated fetches, so the figures here rest on search corroboration of the official scholarship and admissions pages rather than a direct fetch; the RePEc rank (#198) was confirmed against the live August 2026 table.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -5267,17 +5267,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>University of Melbourne</t>
+          <t>Australian National University (ANU)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>#151</t>
+          <t>#124</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -5292,62 +5292,62 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Melbourne</t>
+          <t>Canberra</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
+          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
+          <t>6.5 overall (no band below 6.0)</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>94 iBT (W27/S18/R13/L13)</t>
+          <t>570 (paper-based; essay ≥4.5)</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Not mentioned in entry requirements</t>
+          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
+          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>March intake</t>
+          <t>February (Semester 1); Semester 2 entry possible (July)</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>March 2027 intake deadline reported as 30 November 2026 — found via search summary only; the official how-to-apply/key-dates pages returned HTTP 403 on every direct fetch attempt this pass, so this date is unconfirmed by primary source and should be manually verified</t>
+          <t>For Feb 2027 start: international scholarship deadline (31 Aug 2026) has now closed; the standard/domestic deadline of 31 Oct 2026 is the next live deadline (confirmed via search corroboration, ANU site still returning HTTP 504 to direct fetch); Sem 2 entry deadline (31 Mar) also already closed for this cycle</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>urgent</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>Not detailed — full tuition fee waiver reported (see funding)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
@@ -5357,7 +5357,7 @@
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>Australian Government Research Training Program (RTP) funded places available: RTP stipend reported at AUD $39,500/year (2026 rate) plus full tuition fee waiver and AUD $15,000 research/conference travel funding for confirmed PhD candidates (unconfirmed by primary source — see deadline note). Program structure: 2-year Master of Commerce coursework + 3-year PhD.</t>
+          <t>Australian Government RTP Stipend: AUD $39,069/year (2026 full-time base rate, ANU-wide), paid fortnightly, up to 3.5 years. Some HDR supplementary scholarships add AUD $7,000/year on top, for up to 3 years. Domestic candidates pay no tuition (RTP-covered); international candidates can compete for HDR Fee Remission Merit Scholarships covering up to 4 years.</t>
         </is>
       </c>
       <c r="V38" t="inlineStr">
@@ -5367,24 +5367,24 @@
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>Found a reported deadline and funding figures via search, but could not confirm via direct page fetch (403 blocked) — flagged as lower confidence</t>
+          <t>Domestic deadline (31 Oct 2026) is now within 30 days (28 days out) — urgency upgraded from soon to urgent, 30-day reminder flag set</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches this pass — recommend a manual browser check before relying on the reported 30 Nov 2026 deadline</t>
+          <t>Seed entry Aug 2026 — international-applicant deadline has closed; domestic deadline (31 Oct 2026) is next. Note telegram_notified_30day/7day are already true from an earlier reset (pre-dating the Step 5 sync fix) — this run's 30-day flag flip follows the normal (non-reset) rule and does not touch the telegram_notified_* pair, so telegram_sync.py will not re-announce it; known gap, not new.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -5394,17 +5394,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PhD (Economics)</t>
+          <t>Doctoral Program in Economics</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Monash Business School</t>
+          <t>University of Melbourne</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>#46</t>
+          <t>#151</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -5419,47 +5419,47 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Melbourne (Clayton)</t>
+          <t>Melbourne</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
+          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>7.0 minimum reported (third-party source, not confirmed on official Monash page — page returned HTTP 403 to direct fetch)</t>
+          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>94 minimum reported (same caveat as IELTS — unconfirmed by primary source)</t>
+          <t>94 iBT (W27/S18/R13/L13)</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Not mentioned in entry requirements</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
+          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>March intake</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Integrated-pathway Feb/Semester-1 entry window (1 Jul-31 Aug) has closed; next integrated-pathway window (Jul/Semester-2 entry) opens ~1 Dec-1 Feb. Separately, general Graduate Research Scholarship rounds: international Round 3 (~31 Jul/31 Aug) has closed; domestic Round 4 closes 31 Oct 2026 (confirmed via search, monash.edu still blocking direct fetch with HTTP 403) — this is the next live deadline.</t>
+          <t>March 2027 intake deadline reported as 30 November 2026 via one search summary; a second independent search this pass instead reported 31 August 2026 for the same intake (which, if accurate, would already be closed) — the official how-to-apply/key-dates pages continue to return HTTP 403 on every direct fetch attempt (including via a proxy), so neither date is confirmed by primary source. One plausible reading is that 31 Aug is an earlier scholarship-priority round and 30 Nov a later general-application round (a split seen at other Australian universities in this tracker), but that's a guess, not a finding — still needs a manual browser check.</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -5469,12 +5469,12 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>International ~AUD $38,900/yr, domestic ~AUD $37,100/yr reported (third-party aggregator source, not confirmed by official Monash page)</t>
+          <t>Not detailed — full tuition fee waiver reported (see funding)</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
@@ -5484,7 +5484,7 @@
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places — general RTP stipend reported at AUD $37,145/yr (2026 rate) plus a $1,500 relocation allowance (not confirmed Economics-specific).</t>
+          <t>Australian Government Research Training Program (RTP) funded places available: RTP stipend reported at AUD $39,500/year (2026 rate) plus full tuition fee waiver and AUD $15,000 research/conference travel funding for confirmed PhD candidates (unconfirmed by primary source — see deadline note). Program structure: 2-year Master of Commerce coursework + 3-year PhD.</t>
         </is>
       </c>
       <c r="V39" t="inlineStr">
@@ -5494,24 +5494,24 @@
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>Domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026) is now within 30 days (28 days out) — urgency upgraded from soon to urgent, 30-day reminder flag set</t>
+          <t>Re-attempted reconfirmation (including via a proxy) — official page still blocked; found a second, conflicting search-reported deadline (31 Aug 2026) alongside the existing 30 Nov 2026 figure. Noted the conflict; deadline/urgency left unchanged pending manual verification.</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; monash.edu has blocked all automated fetches on every pass so far (scholarships-and-fees, apply, and program pages all 403'd) — every figure in this entry is lower-confidence (search snippets/third-party aggregator only) and needs a manual browser check. Note telegram_notified_30day/7day are already true from an earlier reset (pre-dating the Step 5 sync fix) — this run's 30-day flag flip follows the normal (non-reset) rule and does not touch the telegram_notified_* pair; known gap, not new.</t>
+          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches on every pass so far, including through a proxy this time — recommend a manual browser check before relying on either the 30 Nov 2026 or 31 Aug 2026 deadline figures now in circulation</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -5521,17 +5521,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD (Economics)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>University of Sydney</t>
+          <t>Monash Business School</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>#87</t>
+          <t>#46</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -5546,32 +5546,32 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Sydney</t>
+          <t>Melbourne (Clayton)</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://www.sydney.edu.au/scholarships/</t>
+          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>7.0 minimum reported (third-party source, not confirmed on official Monash page — page returned HTTP 403 to direct fetch)</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>94 minimum reported (same caveat as IELTS — unconfirmed by primary source)</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP. Material finding: Sydney has no dedicated 'PhD in Economics' program page — the Economics coursework handbook explicitly states it "does not include a research component and thus does not provide a pathway to higher degree by research (e.g. PhD) studies." PhD study is pursued via the general Doctor of Philosophy degree with a nominated Economics supervisor/discipline, not a single named landing page.</t>
+          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -5581,17 +5581,17 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Research Period 1 &amp; 2 deadline (11 September 2026) has now passed; Research Period 3 &amp; 4 — deadline 18 December 2026 — is the next live RTP scholarship round (reconfirmed via search, not a directly-fetched dedicated Economics PhD page).</t>
+          <t>Integrated-pathway Feb/Semester-1 entry window (1 Jul-31 Aug) has closed; next integrated-pathway window (Jul/Semester-2 entry) opens ~1 Dec-1 Feb. Separately, general Graduate Research Scholarship rounds: international Round 3 (~31 Jul/31 Aug) has closed; domestic Round 4 closes 31 Oct 2026 (confirmed via search, monash.edu still blocking direct fetch with HTTP 403) — this is the next live deadline.</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>urgent</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>1 (for named scholarship example; general program may differ)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -5601,7 +5601,7 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>International ~AUD $38,900/yr, domestic ~AUD $37,100/yr reported (third-party aggregator source, not confirmed by official Monash page)</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly; a 2027-rate RTP stipend of AUD $44,293/yr was also reported via search aggregators this pass (unconfirmed by primary source).</t>
+          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places — general RTP stipend reported at AUD $37,145/yr (2026 rate) plus a $1,500 relocation allowance (not confirmed Economics-specific).</t>
         </is>
       </c>
       <c r="V40" t="inlineStr">
@@ -5621,24 +5621,24 @@
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down from urgent to soon, reminder flags reset for the new deadline</t>
+          <t>Domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026) is now within 30 days (28 days out) — urgency upgraded from soon to urgent, 30-day reminder flag set</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check; no dedicated Economics-specific PhD admissions page exists at Sydney</t>
+          <t>Seed entry Aug 2026; monash.edu has blocked all automated fetches on every pass so far (scholarships-and-fees, apply, and program pages all 403'd) — every figure in this entry is lower-confidence (search snippets/third-party aggregator only) and needs a manual browser check. Note telegram_notified_30day/7day are already true from an earlier reset (pre-dating the Step 5 sync fix) — this run's 30-day flag flip follows the normal (non-reset) rule and does not touch the telegram_notified_* pair; known gap, not new.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>AUS-05</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -5653,12 +5653,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>UNSW Sydney</t>
+          <t>University of Sydney</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>#80</t>
+          <t>#87</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -5678,67 +5678,67 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>https://www.unsw.edu.au/business/study-with-us/postgraduate-research/phd-degrees/doctor-philosophy-phd-economics</t>
+          <t>https://www.sydney.edu.au/scholarships/</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Not listed on this page (exemptions for AU/CA/UK/US/NZ citizens); non-English-speaking-country applicants need IELTS/TOEFL/PTE/Cambridge or the UNSW Global English Course</t>
+          <t>Not specified at general program level</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Not listed on this page — see IELTS field for alternatives</t>
+          <t>Not specified at general program level</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Optional but recommended overall; one source indicates GRE may be specifically required for the Economics stream — this conflicts with the general 'optional' language elsewhere and needs manual confirmation</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course. Program begins with a 1-year Master of Pre-Doctoral Business Studies, followed by 3-3.5 years of doctoral research; direct entry to the 3-year PhD is possible for candidates with first-class Honours/Master's plus independent funding (Stream 2).</t>
+          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP. Material finding: Sydney has no dedicated 'PhD in Economics' program page — the Economics coursework handbook explicitly states it "does not include a research component and thus does not provide a pathway to higher degree by research (e.g. PhD) studies." PhD study is pursued via the general Doctor of Philosophy degree with a nominated Economics supervisor/discipline, not a single named landing page.</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Term 1 – February</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Confirmed still closed as of 23 Aug 2026 (verified directly on program page): EOI window opened 20 March 2026, closed 15 August 2026, no newer/next EOI window posted. Note: a separate 26 August 2026 formal-application deadline exists, but it applies only to candidates already invited to apply from the closed EOI round, not to new applicants.</t>
+          <t>Research Period 1 &amp; 2 deadline (11 September 2026) has now passed; Research Period 3 &amp; 4 — deadline 18 December 2026 — is the next live RTP scholarship round (reconfirmed via search, not a directly-fetched dedicated Economics PhD page).</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
+          <t>1 (for named scholarship example; general program may differ)</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr">
+      <c r="S41" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="S41" t="inlineStr">
-        <is>
-          <t>Not detailed (fully funded — see funding)</t>
-        </is>
-      </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>Yes — all admitted students</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>Full tuition waiver + stipend AUD 35,000-45,000/yr, up to 4.5 years (+1 optional fellowship year), plus substantial research/conference travel funding.</t>
+          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly; a 2027-rate RTP stipend of AUD $44,293/yr was also reported via search aggregators this pass (unconfirmed by primary source).</t>
         </is>
       </c>
       <c r="V41" t="inlineStr">
@@ -5748,144 +5748,271 @@
       </c>
       <c r="W41" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>Confirmed EOI window remains closed with no new window announced; added program structure and English-test details</t>
+          <t>11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down from urgent to soon, reminder flags reset for the new deadline</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026 — EOI window closed 15 Aug 2026, still no next window announced as of this update</t>
+          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check; no dedicated Economics-specific PhD admissions page exists at Sydney</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>AUS-05</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>PhD in Economics</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>UNSW Sydney</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>#80</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://www.unsw.edu.au/business/study-with-us/postgraduate-research/phd-degrees/doctor-philosophy-phd-economics</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Not listed on this page (exemptions for AU/CA/UK/US/NZ citizens); non-English-speaking-country applicants need IELTS/TOEFL/PTE/Cambridge or the UNSW Global English Course</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Not listed on this page — see IELTS field for alternatives</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Optional but recommended overall; one source indicates GRE may be specifically required for the Economics stream — this conflicts with the general 'optional' language elsewhere and needs manual confirmation</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course. Program begins with a 1-year Master of Pre-Doctoral Business Studies, followed by 3-3.5 years of doctoral research; direct entry to the 3-year PhD is possible for candidates with first-class Honours/Master's plus independent funding (Stream 2).</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Term 1 – February</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Confirmed still closed as of 23 Aug 2026 (verified directly on program page): EOI window opened 20 March 2026, closed 15 August 2026, no newer/next EOI window posted. Note: a separate 26 August 2026 formal-application deadline exists, but it applies only to candidates already invited to apply from the closed EOI round, not to new applicants.</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Not detailed (fully funded — see funding)</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>Yes — all admitted students</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>Full tuition waiver + stipend AUD 35,000-45,000/yr, up to 4.5 years (+1 optional fellowship year), plus substantial research/conference travel funding.</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>Confirmed EOI window remains closed with no new window announced; added program structure and English-test details</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026 — EOI window closed 15 Aug 2026, still no next window announced as of this update</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>AUS-06</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>Doctor of Philosophy (Economics)</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>University of Queensland (School of Economics)</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>#71</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>Brisbane</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>https://economics.uq.edu.au/study/phd</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>Academic overall 6.5, with 6.0 minimum in each of reading/writing/speaking/listening</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>Not specified on the economics-specific page (UQ university-wide PhD pages generally accept TOEFL iBT as an alternative to IELTS)</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>Not confirmed as required; application package can include GRE/GMAT score sheets, suggesting optional/supplementary rather than mandatory</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="M43" t="inlineStr">
         <is>
           <t>Academic CV, transcripts; MPhil/research master's options also available; can join a funded project with scholarship support as an alternative entry route</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
+      <c r="N43" t="inlineStr">
         <is>
           <t>Quarterly intakes (research quarters begin 1 Jan, 1 Apr, 1 Jul, 1 Oct); applications for RHD programs can be submitted any time</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr">
+      <c r="O43" t="inlineStr">
         <is>
           <t>Domestic Round 1 (31 Aug 2026) has now closed; the International round deadline of 19 Oct 2026 is confirmed still live via search corroboration and is the next relevant deadline for upcoming 2027 research quarters.</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr">
+      <c r="P43" t="inlineStr">
         <is>
           <t>urgent</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr">
+      <c r="Q43" t="inlineStr">
         <is>
           <t>Minimum 2 referee reports</t>
         </is>
       </c>
-      <c r="R42" t="inlineStr">
+      <c r="R43" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="S42" t="inlineStr">
+      <c r="S43" t="inlineStr">
         <is>
           <t>Not specified (international RTP scholarship recipients typically get a full tuition fee offset)</t>
         </is>
       </c>
-      <c r="T42" t="inlineStr">
+      <c r="T43" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="U43" t="inlineStr">
         <is>
           <t>RTP/UQGRSS provides a tax-free living stipend of AUD $39,220/year (2026 rate, indexed annually — updated from a previously-recorded AUD $37,500 figure) plus, for eligible international candidates, a tuition fee offset; no separate application needed beyond the program EOI.</t>
         </is>
       </c>
-      <c r="V42" t="inlineStr">
+      <c r="V43" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="W42" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="X42" t="inlineStr">
-        <is>
-          <t>International round deadline (19 Oct 2026) is now 23 days out, inside the ~4-week threshold — urgency upgraded from soon to urgent</t>
-        </is>
-      </c>
-      <c r="Y42" t="inlineStr">
-        <is>
-          <t>Scholarship is university-wide (RTP/UQGRSS), not economics-specific, but School of Economics PhD candidates are eligible. The 30-day reminder flag was already set on the 2026-09-19 pass, so no new reminder is due — only the urgency classification changed.</t>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>International round deadline (19 Oct 2026) reconfirmed via two independent sources — now only 2 days out, inside the 7-day threshold; 7-day reminder flag tripped</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>Scholarship is university-wide (RTP/UQGRSS), not economics-specific, but School of Economics PhD candidates are eligible. The 30-day reminder flag was already set on the 2026-09-19 pass; this pass trips the 7-day flag as the deadline closes in.</t>
         </is>
       </c>
     </row>
@@ -5900,7 +6027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5940,17 +6067,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>EUR-25</t>
+          <t>EUR-28</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Rome Economics Doctorate (RED) — EIEF / Luiss / Sapienza / Tor Vergata</t>
+          <t>CEREB PhD Scholarship — University of Erfurt</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -5960,24 +6087,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>New funded Economics PhD program: joint program run by EIEF (a Bank of Italy-funded research institute) with three Rome universities, four-year tuition waiver plus stipend (recurring 15 Jan deadline pattern, current cycle shown closed).</t>
+          <t>New find — interdisciplinary doctoral scholarship (behavioral economics among its covered fields), EUR 1,400/month for 3-4 years, deadline 24 Nov 2026.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EUR-17</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE)</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -5987,61 +6114,61 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Resolved the previously-flagged admission-round date inconsistency via direct fetch of the authoritative vgse.at page: Round 1 1 Dec–31 Jan, Round 2 1 Mar–30 Apr.</t>
+          <t>MATERIAL CORRECTION: confirmed via primary-source PDF (reached through a proxy after six passes blocked by a TLS error) that the Spring 2027 deadline is 24 Nov-4 Dec 2026, not the previously estimated mid-October window — urgency stepped back from urgent to soon, all four notification flags reset.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Reconfirmation of the estimated ~14-17 Oct 2026 Spring-intake window attempted again; official site unreachable (TLS certificate error). Estimate left unchanged but flagged for a manual check given the imminent deadline.</t>
+          <t>International round deadline (19 Oct 2026) reconfirmed via two independent sources, now 2 days out — 7-day reminder flag tripped.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Domestic deadline (31 Oct 2026) now 28 days out, inside the ~4-week threshold — urgency upgraded from soon to urgent, 30-day reminder flag set.</t>
+          <t>Official page remains blocked to automated fetches (403, including via a proxy); found a second search-reported deadline (31 Aug 2026) that conflicts with the previously recorded 30 Nov 2026 figure — flagged for manual verification rather than guessed at.</t>
         </is>
       </c>
     </row>
@@ -6053,39 +6180,39 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>EUR-25</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>Rome Economics Doctorate (RED) — EIEF / Luiss / Sapienza / Tor Vergata</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026) now 28 days out, inside the ~4-week threshold — urgency upgraded from soon to urgent, 30-day reminder flag set.</t>
+          <t>New funded Economics PhD program: joint program run by EIEF (a Bank of Italy-funded research institute) with three Rome universities, four-year tuition waiver plus stipend (recurring 15 Jan deadline pattern, current cycle shown closed).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -6095,24 +6222,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Correction: the '30 September 2026 early round' deadline recorded on 14 Sep could not be re-substantiated by any source this pass and appears to have been recorded in error. Two independent corroborations give a single FASS window of 1 May - 15 Dec 2026 for the Aug 2027 intake, with 1 Dec 2026 as the Economics department deadline. Urgency stepped back from urgent to soon and the 30-day reminder flag has been reset. Apologies for the earlier reminder against a date we can no longer confirm.</t>
+          <t>Resolved the previously-flagged admission-round date inconsistency via direct fetch of the authoritative vgse.at page: Round 1 1 Dec–31 Jan, Round 2 1 Mar–30 Apr.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -6122,61 +6249,61 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>The long-standing cohort-year ambiguity is resolved: the Dec/Feb/May rounds are confirmed to be the Cohort 2027-2029 rounds, with Studielink opening 1 Oct 2026 and Round 1 closing 1 Dec 2026, then 1 Feb 2027, 1 May 2027, and rolling admissions to 15 Jun 2027.</t>
+          <t>Reconfirmation of the estimated ~14-17 Oct 2026 Spring-intake window attempted again; official site unreachable (TLS certificate error). Estimate left unchanged but flagged for a manual check given the imminent deadline.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EUR-03</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>The 2027-28 deadline that was previously TBA is now confirmed as 15 January 2027 at 14:00 CET, with the call for applications opening in early November 2026. Urgency raised from later to soon.</t>
+          <t>Domestic deadline (31 Oct 2026) now 28 days out, inside the ~4-week threshold — urgency upgraded from soon to urgent, 30-day reminder flag set.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EUR-09</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MPhil + DPhil in Economics — University of Oxford</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>The 2027-28 entry cycle has opened — most Oxford graduate courses opened to applications on 16 Sep 2026. Scholarship provision updated to the 1,200+ full/partial graduate scholarships expected for 2027-28, up from the 1,100+ figure for 2026-27. Deadline remains the January pattern (most recent round closed 27 Jan).</t>
+          <t>Domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026) now 28 days out, inside the ~4-week threshold — urgency upgraded from soon to urgent, 30-day reminder flag set.</t>
         </is>
       </c>
     </row>
@@ -6188,12 +6315,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -6203,7 +6330,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>The 43rd cycle (a.y. 2027-28) is now announced: the Call for Applications opens 3 November 2026. Urgency moved from closed to later now that a next cycle exists; the closing date for that call is not yet published.</t>
+          <t>Correction: the '30 September 2026 early round' deadline recorded on 14 Sep could not be re-substantiated by any source this pass and appears to have been recorded in error. Two independent corroborations give a single FASS window of 1 May - 15 Dec 2026 for the Aug 2027 intake, with 1 Dec 2026 as the Economics department deadline. Urgency stepped back from urgent to soon and the 30-day reminder flag has been reset. Apologies for the earlier reminder against a date we can no longer confirm.</t>
         </is>
       </c>
     </row>
@@ -6215,12 +6342,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EUR-12</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -6230,7 +6357,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Corrected the deadline pattern: the previously recorded '~20 Oct - 13 Jan' window did not match UCL's published dates. The confirmed recent-cycle deadline was 23 January 2026 at 17:00 UK time, with late applications considered to 27 March 2026, so the pattern is a late-January deadline and ~late Jan 2027 is expected for 2027 entry.</t>
+          <t>The long-standing cohort-year ambiguity is resolved: the Dec/Feb/May rounds are confirmed to be the Cohort 2027-2029 rounds, with Studielink opening 1 Oct 2026 and Round 1 closing 1 Dec 2026, then 1 Feb 2027, 1 May 2027, and rolling admissions to 15 Jun 2027.</t>
         </is>
       </c>
     </row>
@@ -6242,12 +6369,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>EUR-03</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -6257,7 +6384,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>The international round deadline (19 Oct 2026) is now 23 days away, inside the ~4-week threshold, so urgency has been upgraded from soon to urgent. The 30-day reminder already went out on 19 Sep, so no new reminder is due.</t>
+          <t>The 2027-28 deadline that was previously TBA is now confirmed as 15 January 2027 at 14:00 CET, with the call for applications opening in early November 2026. Urgency raised from later to soon.</t>
         </is>
       </c>
     </row>
@@ -6269,22 +6396,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EUR-24</t>
+          <t>EUR-09</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PhD in Economics — Central European University (CEU)</t>
+          <t>MPhil + DPhil in Economics — University of Oxford</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>New find: RePEc #268, Vienna. Full tuition coverage plus a EUR 2,002 gross/month doctoral stipend for the full 48 months, awarded automatically from the admissions round rather than a separate competition. Current round closes 15 January 2027. Note the stipend is taxable in Austria.</t>
+          <t>The 2027-28 entry cycle has opened — most Oxford graduate courses opened to applications on 16 Sep 2026. Scholarship provision updated to the 1,200+ full/partial graduate scholarships expected for 2027-28, up from the 1,100+ figure for 2026-27. Deadline remains the January pattern (most recent round closed 27 Jan).</t>
         </is>
       </c>
     </row>
@@ -6296,228 +6423,228 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ASA-10</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PhD in Economics — Singapore Management University (SMU), School of Economics</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>New find: RePEc #198, Singapore. Full scholarship covering registration and tuition plus a monthly stipend — foreign students SGD 2,500/month rising to SGD 3,000 after the qualifying exam — renewable for the first 4 years. Applications run 1 Aug - 31 Dec annually, so 31 Dec 2026 for the Aug 2027 intake.</t>
+          <t>The 43rd cycle (a.y. 2027-28) is now announced: the Call for Applications opens 3 November 2026. Urgency moved from closed to later now that a next cycle exists; the closing date for that call is not yet published.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EUR-23</t>
+          <t>EUR-12</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PhD in Economics (Quantitative Economics track) — Goethe University Frankfurt (GSEFM)</t>
+          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>New find: RePEc #81, up to three competitive first-year IMFS stipends plus post-qualifying-exam TA/RA positions; no tuition fees.</t>
+          <t>Corrected the deadline pattern: the previously recorded '~20 Oct - 13 Jan' window did not match UCL's published dates. The confirmed recent-cycle deadline was 23 January 2026 at 17:00 UK time, with late applications considered to 27 March 2026, so the pattern is a late-January deadline and ~late Jan 2027 is expected for 2027 entry.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>30-day reminder: the Spring-intake submission window (expected ~14-17 Oct 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
+          <t>The international round deadline (19 Oct 2026) is now 23 days away, inside the ~4-week threshold, so urgency has been upgraded from soon to urgent. The 30-day reminder already went out on 19 Sep, so no new reminder is due.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>EUR-24</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>PhD in Economics — Central European University (CEU)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>30-day reminder: the international round deadline (19 Oct 2026) is now within 30 days.</t>
+          <t>New find: RePEc #268, Vienna. Full tuition coverage plus a EUR 2,002 gross/month doctoral stipend for the full 48 months, awarded automatically from the admissions round rather than a separate competition. Current round closes 15 January 2027. Note the stipend is taxable in Austria.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-10</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>PhD in Economics — Singapore Management University (SMU), School of Economics</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>The 11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down to soon, reminder flags reset.</t>
+          <t>New find: RePEc #198, Singapore. Full scholarship covering registration and tuition plus a monthly stipend — foreign students SGD 2,500/month rising to SGD 3,000 after the qualifying exam — renewable for the first 4 years. Applications run 1 Aug - 31 Dec annually, so 31 Dec 2026 for the Aug 2027 intake.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-23</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>PhD in Economics (Quantitative Economics track) — Goethe University Frankfurt (GSEFM)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>30-day reminder: the early-round deadline (30 Sep 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
+          <t>New find: RePEc #81, up to three competitive first-year IMFS stipends plus post-qualifying-exam TA/RA positions; no tuition fees.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Official site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025.</t>
+          <t>30-day reminder: the Spring-intake submission window (expected ~14-17 Oct 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>EUR-22</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Cambridge</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>New find: RePEc #50, ~66% of Cambridge doctoral students fully funded via Cambridge Trust/Gates Cambridge/College/ESRC funding; funding-competition deadline 8 Dec 2026.</t>
+          <t>30-day reminder: the international round deadline (19 Oct 2026) is now within 30 days.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -6527,88 +6654,88 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline, urgency moved from urgent to soon.</t>
+          <t>The 11 Sep 2026 Research Period 1 &amp; 2 deadline has passed; now tracking Research Period 3 &amp; 4 (18 Dec 2026) — urgency stepped back down to soon, reminder flags reset.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Confirmed the integrated-pathway and international scholarship round deadlines have closed; now tracking the domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026), urgency moved from urgent to soon.</t>
+          <t>30-day reminder: the early-round deadline (30 Sep 2026) is now within 30 days — urgency upgraded from soon to urgent.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>7-day reminder: the 11 Sep 2026 Research Period 1 &amp; 2 deadline is confirmed still live and now imminent.</t>
+          <t>Official site remains unreachable (DNS failure, fifth consecutive pass); found an unconfirmed search-only lead that the Master's-level entry point may have changed since 2025.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>EUR-22</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>PhD in Economics — University of Cambridge</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026), urgency moved from urgent to soon.</t>
+          <t>New find: RePEc #50, ~66% of Cambridge doctoral students fully funded via Cambridge Trust/Gates Cambridge/College/ESRC funding; funding-competition deadline 8 Dec 2026.</t>
         </is>
       </c>
     </row>
@@ -6620,12 +6747,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>EUR-17</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -6635,7 +6762,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#192) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>International scholarship deadline (31 Aug 2026) has closed; now tracking the domestic 31 Oct 2026 deadline, urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -6647,12 +6774,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EUR-18</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -6662,7 +6789,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#24) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>Confirmed the integrated-pathway and international scholarship round deadlines have closed; now tracking the domestic Graduate Research Scholarship Round 4 deadline (31 Oct 2026), urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -6674,22 +6801,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EUR-19</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#40) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>7-day reminder: the 11 Sep 2026 Research Period 1 &amp; 2 deadline is confirmed still live and now imminent.</t>
         </is>
       </c>
     </row>
@@ -6701,12 +6828,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EUR-20</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -6716,7 +6843,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#164) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>Confirmed the domestic round (31 Aug 2026) has closed; now tracking the international round deadline (19 Oct 2026), urgency moved from urgent to soon.</t>
         </is>
       </c>
     </row>
@@ -6728,12 +6855,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -6743,7 +6870,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat.</t>
+          <t>Confirmed RePEc rank (#192) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
@@ -6755,12 +6882,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -6770,7 +6897,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Official site remains unreachable (DNS failure, fourth consecutive pass); recommend a manual browser check rather than further automated retries.</t>
+          <t>Confirmed RePEc rank (#24) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
@@ -6782,120 +6909,120 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EUR-21</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PhD in Economics — Sciences Po</t>
+          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>New find: RePEc #42, funded via a 3-year Doctoral Contract (~EUR 2,100/month) plus tuition exemption; some applicants expected to already hold external funding.</t>
+          <t>Confirmed RePEc rank (#40) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>EUR-17</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
+          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>New find: FWF-grant-funded PhD positions at the University of Vienna; admission-round dates inconsistent across sources, recommend a manual spot-check.</t>
+          <t>Confirmed RePEc rank (#164) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>EUR-18</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
+          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>New find: PhD structured as a salaried employment contract (~EUR 2,750-3,500/month); official site blocked automated fetches, several fields search-only.</t>
+          <t>Confirmed RePEc rank (#369) via direct fetch of the live table, removing the prior unverified caveat.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>EUR-19</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>New find: RePEc ~#40, funded PhD positions up to 4 years plus IRO Doctoral Scholarships for developing-country students; deadlines are vacancy-by-vacancy.</t>
+          <t>Official site remains unreachable (DNS failure, fourth consecutive pass); recommend a manual browser check rather than further automated retries.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>EUR-20</t>
+          <t>EUR-21</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
+          <t>PhD in Economics — Sciences Po</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -6905,7 +7032,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>New find: joint Berlin-area doctoral school, funded via a EUR 1,650/month qualification-phase stipend then dissertation-phase employment.</t>
+          <t>New find: RePEc #42, funded via a 3-year Doctoral Contract (~EUR 2,100/month) plus tuition exemption; some applicants expected to already hold external funding.</t>
         </is>
       </c>
     </row>
@@ -6917,12 +7044,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ASA-09</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -6932,7 +7059,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>New find: guaranteed teaching/research assistantship (~HK$19,100/month) for all admits, independent of the HKPFS scheme already tracked (ASA-03).</t>
+          <t>New find: FWF-grant-funded PhD positions at the University of Vienna; admission-round dates inconsistent across sources, recommend a manual spot-check.</t>
         </is>
       </c>
     </row>
@@ -6944,22 +7071,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Confirmed application windows (Aug intake: 1 Oct-15 Nov; Jan intake: 1 Jun-31 Jul), referee/fee requirements, and Graduate Assistantship Programme detail via direct official fetch; urgency upgraded from tba to soon.</t>
+          <t>New find: PhD structured as a salaried employment contract (~EUR 2,750-3,500/month); official site blocked automated fetches, several fields search-only.</t>
         </is>
       </c>
     </row>
@@ -6971,22 +7098,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Corroborated via search snippets (site unreachable for a third consecutive pass) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad.</t>
+          <t>New find: RePEc ~#40, funded PhD positions up to 4 years plus IRO Doctoral Scholarships for developing-country students; deadlines are vacancy-by-vacancy.</t>
         </is>
       </c>
     </row>
@@ -6998,22 +7125,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration; urgency upgraded from tba to soon.</t>
+          <t>New find: joint Berlin-area doctoral school, funded via a EUR 1,650/month qualification-phase stipend then dissertation-phase employment.</t>
         </is>
       </c>
     </row>
@@ -7025,22 +7152,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; funding runs entirely through university-wide scholarships.</t>
+          <t>New find: guaranteed teaching/research assistantship (~HK$19,100/month) for all admits, independent of the HKPFS scheme already tracked (ASA-03).</t>
         </is>
       </c>
     </row>
@@ -7052,22 +7179,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>7-day reminder: the 31 Aug 2026 international scholarship deadline is confirmed still live via search corroboration (ANU site returned HTTP 504 to direct fetch).</t>
+          <t>Confirmed application windows (Aug intake: 1 Oct-15 Nov; Jan intake: 1 Jun-31 Jul), referee/fee requirements, and Graduate Assistantship Programme detail via direct official fetch; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
@@ -7079,22 +7206,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>7-day reminder: the imminent ~31 Aug 2026 integrated-pathway deadline is reconfirmed via search (monash.edu still blocking direct fetch); added a general RTP stipend figure (AUD $37,145/yr).</t>
+          <t>Corroborated via search snippets (site unreachable for a third consecutive pass) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad.</t>
         </is>
       </c>
     </row>
@@ -7106,39 +7233,39 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Deadline reminder</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>7-day reminder: confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to AUD $39,220/yr (2026 rate).</t>
+          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -7148,88 +7275,88 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
+          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; funding runs entirely through university-wide scholarships.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
+          <t>7-day reminder: the 31 Aug 2026 international scholarship deadline is confirmed still live via search corroboration (ANU site returned HTTP 504 to direct fetch).</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
+          <t>7-day reminder: the imminent ~31 Aug 2026 integrated-pathway deadline is reconfirmed via search (monash.edu still blocking direct fetch); added a general RTP stipend figure (AUD $37,145/yr).</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
+          <t>7-day reminder: confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to AUD $39,220/yr (2026 rate).</t>
         </is>
       </c>
     </row>
@@ -7241,12 +7368,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -7256,7 +7383,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
+          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
         </is>
       </c>
     </row>
@@ -7268,12 +7395,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -7283,7 +7410,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
+          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
         </is>
       </c>
     </row>
@@ -7295,12 +7422,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -7310,7 +7437,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
+          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
         </is>
       </c>
     </row>
@@ -7322,12 +7449,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -7337,7 +7464,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
+          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
         </is>
       </c>
     </row>
@@ -7349,12 +7476,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -7364,7 +7491,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
+          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
         </is>
       </c>
     </row>
@@ -7376,12 +7503,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -7391,7 +7518,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
         </is>
       </c>
     </row>
@@ -7403,12 +7530,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -7418,7 +7545,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
+          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
         </is>
       </c>
     </row>
@@ -7430,12 +7557,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -7445,7 +7572,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
+          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
         </is>
       </c>
     </row>
@@ -7457,12 +7584,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -7472,7 +7599,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
+          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
         </is>
       </c>
     </row>
@@ -7484,12 +7611,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>AUS-05</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>PhD in Economics — UNSW Sydney</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -7499,7 +7626,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
+          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -7511,22 +7638,22 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>EUR-13</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
+          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
         </is>
       </c>
     </row>
@@ -7538,22 +7665,22 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>EUR-14</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
+          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -7565,22 +7692,22 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>EUR-15</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
+          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
@@ -7592,22 +7719,22 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EUR-16</t>
+          <t>AUS-05</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
+          <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
+          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
         </is>
       </c>
     </row>
@@ -7619,12 +7746,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ASA-08</t>
+          <t>EUR-13</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
+          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -7634,7 +7761,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
+          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
         </is>
       </c>
     </row>
@@ -7646,12 +7773,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>EUR-14</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -7661,115 +7788,115 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
+          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>EUR-15</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>EUR-16</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>EUR-03</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
+          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>EUR-04</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
         </is>
       </c>
     </row>
@@ -7781,12 +7908,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>EUR-05</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>PhD in Economics — CEMFI</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -7808,12 +7935,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EUR-06</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -7835,12 +7962,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>EUR-07</t>
+          <t>EUR-03</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>PhD Program — Paris School of Economics (PSE)</t>
+          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -7862,12 +7989,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>EUR-08</t>
+          <t>EUR-04</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — Stockholm University / IIES</t>
+          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -7889,12 +8016,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>EUR-09</t>
+          <t>EUR-05</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>MPhil + DPhil in Economics — University of Oxford</t>
+          <t>PhD in Economics — CEMFI</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -7916,12 +8043,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>EUR-06</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -7943,12 +8070,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>EUR-07</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>PhD Program — Paris School of Economics (PSE)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -7970,12 +8097,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>EUR-12</t>
+          <t>EUR-08</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
+          <t>PhD Programme in Economics — Stockholm University / IIES</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -7997,12 +8124,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-09</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>MPhil + DPhil in Economics — University of Oxford</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8024,12 +8151,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -8051,12 +8178,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -8078,12 +8205,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-12</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -8105,12 +8232,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -8132,12 +8259,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -8159,12 +8286,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-03</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -8186,12 +8313,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -8213,12 +8340,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -8240,12 +8367,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -8267,12 +8394,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -8294,20 +8421,128 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
+          <t>AUS-01</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>PhD in Economics — Australian National University (ANU)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>AUS-02</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>AUS-03</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>PhD (Economics) — Monash Business School</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>AUS-04</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>PhD in Economics — University of Sydney</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
           <t>AUS-05</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D93" t="inlineStr">
         <is>
           <t>Added (seed)</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
+      <c r="E93" t="inlineStr">
         <is>
           <t>Initial research pass — program added to tracker.</t>
         </is>

</xml_diff>